<commit_message>
Restructure Method section, fill repair K-sweep results, add eval and training artifacts
Paper: auction moved to standalone Preliminary section before Method
(assignment problem first, exact tractability condition: nonlinearity,
not many-to-one, breaks optimality); terminology unified to many-to-one
auction; repair K-sweep table (12/12 configs, mean 0.1528 -> 0.1323)
filled into sec:repair-results.

Code: eval_repair_paper_table.py, joint mfloop training artifacts
(best audited mean 0.1325 at step 60), figure generator, and session
evaluation scripts/results.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/code_DWTA/TEST_INSTANCE/10M_15N_5T.xlsx
+++ b/code_DWTA/TEST_INSTANCE/10M_15N_5T.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,33 +413,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>TW</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>AMM</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>PREP</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>COST</t>
         </is>
       </c>
     </row>
@@ -462,19 +470,37 @@
       <c r="B2" t="n">
         <v>15</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>[9, 2, 3, 5, 6, 9, 9, 7, 9, 8, 5, 7, 9, 1, 7]</t>
-        </is>
+      <c r="C2" t="n">
+        <v>5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[[0.2424, 0.1731, 0.3241, 0.3545, 0.4303, 0.3524, 0.4089, 0.3075, 0.2013, 0.3091, 0.1522, 0.4466, 0.4272, 0.4475, 0.1191], [0.2555, 0.2954, 0.2976, 0.1939, 0.4713, 0.1069, 0.2768, 0.3387, 0.4879, 0.3459, 0.1628, 0.1537, 0.3368, 0.3992, 0.1357], [0.483, 0.2804, 0.4454, 0.3337, 0.2602, 0.1341, 0.487, 0.1498, 0.3139, 0.3423, 0.3725, 0.421, 0.1901, 0.173, 0.2998], [0.1247, 0.2332, 0.3693, 0.1248, 0.3174, 0.1865, 0.3654, 0.1327, 0.1045, 0.2624, 0.4232, 0.2009, 0.4656, 0.4117, 0.3815], [0.4164, 0.292, 0.4044, 0.4318, 0.3256, 0.1689, 0.2143, 0.1066, 0.2303, 0.1335, 0.1072, 0.2206, 0.4268, 0.2076, 0.1909], [0.2894, 0.426, 0.3643, 0.2107, 0.2161, 0.2106, 0.3082, 0.3426, 0.3999, 0.1267, 0.1805, 0.2914, 0.4217, 0.3507, 0.4365], [0.2243, 0.4815, 0.4806, 0.1701, 0.2296, 0.3995, 0.4506, 0.4111, 0.2922, 0.3786, 0.1974, 0.1785, 0.1009, 0.162, 0.1996], [0.2293, 0.2337, 0.3201, 0.4303, 0.441, 0.1833, 0.3448, 0.1196, 0.3324, 0.3611, 0.4606, 0.1312, 0.3628, 0.2595, 0.4058], [0.2813, 0.432, 0.3521, 0.1902, 0.1517, 0.2247, 0.1661, 0.1729, 0.4436, 0.3374, 0.234, 0.3157, 0.3937, 0.4704, 0.4094], [0.1362, 0.4294, 0.4501, 0.2702, 0.2682, 0.1916, 0.3741, 0.3845, 0.2125, 0.1675, 0.3813, 0.2605, 0.1731, 0.4818, 0.1252]]</t>
+          <t>[2,1,5,4,4,3,2,9,2,10,7,1,1,2,4]</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>[[3, 5], [0, 5], [3, 5], [1, 5], [2, 5], [2, 5], [2, 5], [2, 5], [2, 5], [1, 5], [3, 5], [0, 5], [2, 5], [3, 5], [0, 5]]</t>
+          <t>[[0.46,0.87,0.71,0.62,0.31,0.31,0.24,0.81,0.62,0.7,0.21,0.88,0.78,0.35,0.33],[0.33,0.41,0.57,0.5,0.4,0.63,0.3,0.4,0.46,0.52,0.75,0.34,0.56,0.61,0.23],[0.63,0.32,0.25,0.86,0.88,0.77,0.41,0.27,0.68,0.51,0.29,0.55,0.22,0.84,0.38],[0.66,0.42,0.56,0.58,0.33,0.88,0.74,0.86,0.83,0.62,0.85,0.26,0.34,0.23,0.43],[0.47,0.39,0.78,0.45,0.4,0.58,0.3,0.76,0.25,0.89,0.74,0.34,0.2,0.77,0.69],[0.71,0.74,0.25,0.45,0.28,0.8,0.64,0.43,0.24,0.42,0.43,0.71,0.65,0.82,0.53],[0.28,0.7,0.73,0.59,0.74,0.55,0.57,0.5,0.22,0.28,0.22,0.65,0.42,0.56,0.84],[0.37,0.49,0.73,0.36,0.25,0.4,0.31,0.85,0.77,0.64,0.81,0.76,0.33,0.82,0.58],[0.77,0.83,0.42,0.28,0.36,0.5,0.77,0.8,0.2,0.56,0.49,0.36,0.28,0.44,0.86],[0.43,0.56,0.69,0.45,0.88,0.87,0.38,0.55,0.41,0.4,0.23,0.63,0.55,0.24,0.4]]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[2,5],[0,5],[2,5],[0,5],[2,5],[2,5],[2,5],[2,5],[1,5],[0,5],[1,5],[2,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,2,1,1,2,1,1]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>[2,1,2,2,2,1,2,1,2,1]</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>[100,60,70,50,30,20,50,60,30,50]</t>
         </is>
       </c>
     </row>
@@ -485,19 +511,37 @@
       <c r="B3" t="n">
         <v>15</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>[9, 5, 7, 9, 1, 8, 6, 2, 10, 9, 1, 8, 2, 9, 2]</t>
-        </is>
+      <c r="C3" t="n">
+        <v>5</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>[[0.4923, 0.4661, 0.3131, 0.1394, 0.2816, 0.3762, 0.3167, 0.2804, 0.1463, 0.1013, 0.3375, 0.2224, 0.4875, 0.3178, 0.2485], [0.3182, 0.3161, 0.1437, 0.4518, 0.4496, 0.3655, 0.1608, 0.3639, 0.271, 0.1871, 0.2812, 0.1936, 0.2569, 0.294, 0.3184], [0.1196, 0.4954, 0.345, 0.405, 0.4217, 0.2005, 0.1995, 0.3797, 0.3317, 0.4785, 0.256, 0.4206, 0.3676, 0.239, 0.2047], [0.1135, 0.4288, 0.3108, 0.4149, 0.196, 0.469, 0.1628, 0.4232, 0.1187, 0.4317, 0.4056, 0.4598, 0.1744, 0.3313, 0.1903], [0.1761, 0.3819, 0.4698, 0.101, 0.1203, 0.3653, 0.1902, 0.4183, 0.3065, 0.4883, 0.3473, 0.1404, 0.2996, 0.3753, 0.4396], [0.1371, 0.2822, 0.3254, 0.4083, 0.291, 0.4287, 0.3091, 0.1339, 0.4549, 0.4633, 0.143, 0.2166, 0.2372, 0.1935, 0.395], [0.1252, 0.3372, 0.214, 0.1474, 0.3306, 0.2316, 0.2543, 0.3817, 0.1894, 0.2787, 0.4296, 0.3262, 0.4894, 0.1595, 0.1239], [0.4805, 0.3519, 0.4812, 0.1649, 0.4476, 0.2819, 0.4359, 0.3313, 0.3349, 0.3366, 0.4002, 0.2027, 0.2554, 0.4365, 0.2666], [0.2765, 0.1546, 0.2609, 0.2393, 0.2093, 0.1873, 0.4138, 0.2307, 0.4459, 0.1719, 0.385, 0.4679, 0.3487, 0.4523, 0.1292], [0.4462, 0.2691, 0.2335, 0.4207, 0.3407, 0.1466, 0.229, 0.4708, 0.1105, 0.2543, 0.3367, 0.3111, 0.2137, 0.4169, 0.4217]]</t>
+          <t>[2,7,5,8,6,3,6,6,4,5,2,10,3,9,4]</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[[2, 5], [0, 5], [2, 5], [3, 5], [0, 5], [0, 5], [1, 5], [3, 5], [2, 5], [2, 5], [1, 5], [2, 5], [2, 5], [3, 5], [2, 5]]</t>
+          <t>[[0.84,0.37,0.3,0.54,0.89,0.37,0.67,0.73,0.37,0.71,0.46,0.64,0.64,0.58,0.26],[0.78,0.42,0.33,0.23,0.61,0.67,0.21,0.56,0.36,0.65,0.32,0.68,0.47,0.86,0.3],[0.44,0.28,0.85,0.81,0.38,0.66,0.77,0.59,0.57,0.37,0.27,0.83,0.83,0.64,0.44],[0.44,0.71,0.83,0.82,0.75,0.65,0.26,0.31,0.83,0.62,0.21,0.27,0.66,0.2,0.31],[0.58,0.68,0.66,0.36,0.7,0.37,0.43,0.72,0.65,0.79,0.66,0.6,0.27,0.46,0.39],[0.37,0.88,0.48,0.82,0.64,0.76,0.55,0.6,0.54,0.34,0.71,0.4,0.22,0.65,0.32],[0.86,0.87,0.84,0.46,0.21,0.85,0.5,0.88,0.87,0.8,0.41,0.47,0.8,0.42,0.32],[0.59,0.86,0.69,0.6,0.27,0.63,0.89,0.3,0.56,0.81,0.72,0.69,0.69,0.45,0.41],[0.77,0.77,0.81,0.84,0.56,0.55,0.76,0.65,0.69,0.76,0.82,0.44,0.46,0.27,0.6],[0.23,0.53,0.58,0.4,0.61,0.22,0.23,0.78,0.45,0.29,0.57,0.74,0.35,0.64,0.26]]</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>[[0,5],[1,5],[1,5],[1,5],[2,5],[2,5],[2,5],[0,5],[2,5],[1,5],[0,5],[0,5],[0,5],[1,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,1,2,2,2,1,2]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,2,2,1,1,2,1]</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>[20,30,40,40,80,30,80,80,90,100]</t>
         </is>
       </c>
     </row>
@@ -508,19 +552,37 @@
       <c r="B4" t="n">
         <v>15</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>[2, 9, 10, 10, 4, 8, 5, 6, 4, 9, 6, 9, 4, 2, 2]</t>
-        </is>
+      <c r="C4" t="n">
+        <v>5</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>[[0.4348, 0.359, 0.4218, 0.4322, 0.4829, 0.237, 0.4049, 0.4309, 0.1511, 0.4901, 0.3257, 0.3177, 0.2959, 0.438, 0.4829], [0.2999, 0.14, 0.4361, 0.2277, 0.2918, 0.2797, 0.4888, 0.1605, 0.2634, 0.1919, 0.1017, 0.2711, 0.3931, 0.1821, 0.3657], [0.3921, 0.3671, 0.1414, 0.117, 0.4224, 0.3612, 0.2117, 0.3771, 0.1393, 0.3151, 0.1348, 0.2025, 0.2906, 0.3965, 0.2061], [0.2741, 0.1611, 0.2725, 0.5, 0.2826, 0.3789, 0.1776, 0.3828, 0.1318, 0.4243, 0.497, 0.2622, 0.421, 0.2377, 0.3299], [0.3769, 0.3447, 0.3363, 0.2607, 0.1334, 0.1592, 0.1847, 0.4827, 0.184, 0.2967, 0.2666, 0.3692, 0.4255, 0.155, 0.3217], [0.4372, 0.4943, 0.4246, 0.3058, 0.4117, 0.4118, 0.1871, 0.2512, 0.3868, 0.3, 0.3202, 0.4804, 0.1184, 0.1588, 0.3892], [0.2987, 0.1916, 0.3463, 0.2119, 0.4945, 0.189, 0.1085, 0.2413, 0.298, 0.1862, 0.1472, 0.1025, 0.1164, 0.1302, 0.3791], [0.4696, 0.267, 0.4468, 0.3129, 0.1311, 0.164, 0.3598, 0.4943, 0.2681, 0.3374, 0.3226, 0.3659, 0.1532, 0.1247, 0.3473], [0.2133, 0.1947, 0.3309, 0.2186, 0.1214, 0.1641, 0.4381, 0.4553, 0.4813, 0.1708, 0.2961, 0.4768, 0.1546, 0.1416, 0.2609], [0.1369, 0.1554, 0.4265, 0.4286, 0.4969, 0.3574, 0.19, 0.2404, 0.1755, 0.3997, 0.4621, 0.2152, 0.2798, 0.3338, 0.1641]]</t>
+          <t>[5,9,1,2,9,5,6,2,5,7,3,8,1,5,9]</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>[[1, 5], [3, 5], [1, 5], [1, 5], [3, 5], [2, 5], [2, 5], [2, 5], [0, 5], [3, 5], [3, 5], [1, 5], [1, 5], [2, 5], [3, 5]]</t>
+          <t>[[0.24,0.57,0.58,0.65,0.71,0.88,0.56,0.43,0.76,0.39,0.51,0.25,0.22,0.87,0.79],[0.69,0.49,0.32,0.31,0.38,0.58,0.7,0.66,0.4,0.87,0.72,0.59,0.63,0.49,0.37],[0.45,0.73,0.21,0.28,0.23,0.23,0.8,0.69,0.53,0.27,0.54,0.53,0.32,0.5,0.48],[0.63,0.64,0.23,0.46,0.64,0.55,0.8,0.66,0.31,0.25,0.65,0.22,0.61,0.86,0.6],[0.47,0.65,0.52,0.58,0.86,0.47,0.87,0.83,0.34,0.25,0.27,0.21,0.27,0.68,0.25],[0.42,0.79,0.22,0.77,0.4,0.28,0.69,0.64,0.81,0.71,0.76,0.4,0.32,0.73,0.76],[0.89,0.49,0.46,0.74,0.44,0.85,0.8,0.5,0.73,0.73,0.27,0.83,0.55,0.78,0.42],[0.83,0.47,0.21,0.83,0.26,0.42,0.87,0.87,0.6,0.64,0.51,0.41,0.43,0.67,0.73],[0.75,0.75,0.26,0.55,0.24,0.58,0.51,0.82,0.45,0.28,0.3,0.73,0.63,0.27,0.26],[0.69,0.25,0.78,0.69,0.26,0.26,0.89,0.46,0.46,0.77,0.86,0.89,0.73,0.46,0.26]]</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[0,5],[2,5],[1,5],[2,5],[2,5],[2,5],[0,5],[0,5],[1,5],[0,5],[2,5],[2,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>[2,2,1,1,2,2,1,1,1,1]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[1,2,1,1,1,2,1,2,2,1]</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>[100,50,60,80,70,90,100,90,30,50]</t>
         </is>
       </c>
     </row>
@@ -531,19 +593,37 @@
       <c r="B5" t="n">
         <v>15</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>[5, 4, 9, 4, 1, 10, 3, 2, 1, 1, 3, 10, 4, 9, 6]</t>
-        </is>
+      <c r="C5" t="n">
+        <v>5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>[[0.3036, 0.296, 0.1871, 0.3294, 0.2406, 0.3265, 0.1453, 0.4768, 0.2082, 0.3594, 0.144, 0.1939, 0.149, 0.3092, 0.2917], [0.4784, 0.3656, 0.34, 0.1012, 0.2483, 0.3948, 0.1487, 0.3314, 0.4291, 0.3346, 0.1396, 0.4443, 0.3853, 0.1334, 0.469], [0.3077, 0.3633, 0.1213, 0.3511, 0.3767, 0.3646, 0.2924, 0.1401, 0.229, 0.401, 0.223, 0.279, 0.2846, 0.2501, 0.3238], [0.1367, 0.1658, 0.2373, 0.4557, 0.3109, 0.2911, 0.3091, 0.2421, 0.1921, 0.2053, 0.476, 0.4643, 0.4465, 0.2317, 0.1907], [0.2844, 0.3462, 0.1781, 0.3914, 0.4465, 0.23, 0.2699, 0.4966, 0.161, 0.4929, 0.1901, 0.2356, 0.3689, 0.3832, 0.3062], [0.388, 0.494, 0.4067, 0.1865, 0.2131, 0.2979, 0.1982, 0.4072, 0.3615, 0.4298, 0.3886, 0.2597, 0.1119, 0.2149, 0.4164], [0.1396, 0.4498, 0.2663, 0.1535, 0.2782, 0.3226, 0.3407, 0.4801, 0.2585, 0.3764, 0.4929, 0.1421, 0.2802, 0.1736, 0.1464], [0.3396, 0.4847, 0.2319, 0.1074, 0.3888, 0.3615, 0.1209, 0.2462, 0.208, 0.4374, 0.1401, 0.2538, 0.3157, 0.183, 0.259], [0.4156, 0.1469, 0.2368, 0.1825, 0.382, 0.4927, 0.4226, 0.3715, 0.2802, 0.4116, 0.1705, 0.1161, 0.1652, 0.1412, 0.1454], [0.4925, 0.3335, 0.4737, 0.2738, 0.4981, 0.1422, 0.3981, 0.4065, 0.2761, 0.2923, 0.3835, 0.31, 0.1983, 0.1256, 0.3175]]</t>
+          <t>[4,2,6,1,10,9,4,10,4,1,2,1,4,2,1]</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[[3, 5], [3, 5], [3, 5], [0, 5], [0, 5], [3, 5], [1, 5], [2, 5], [2, 5], [3, 5], [0, 5], [3, 5], [1, 5], [2, 5], [2, 5]]</t>
+          <t>[[0.74,0.59,0.5,0.83,0.28,0.54,0.21,0.53,0.24,0.28,0.28,0.65,0.72,0.61,0.87],[0.46,0.4,0.81,0.36,0.87,0.21,0.88,0.23,0.82,0.57,0.9,0.25,0.59,0.88,0.57],[0.64,0.69,0.52,0.64,0.61,0.83,0.23,0.4,0.87,0.82,0.52,0.63,0.39,0.33,0.52],[0.45,0.61,0.25,0.88,0.89,0.69,0.58,0.42,0.77,0.68,0.31,0.84,0.78,0.86,0.71],[0.63,0.49,0.85,0.81,0.23,0.22,0.46,0.77,0.89,0.31,0.62,0.47,0.88,0.79,0.79],[0.53,0.49,0.39,0.24,0.81,0.77,0.9,0.9,0.59,0.74,0.86,0.79,0.37,0.52,0.29],[0.87,0.62,0.36,0.67,0.63,0.45,0.28,0.67,0.56,0.74,0.56,0.8,0.59,0.59,0.81],[0.48,0.29,0.22,0.73,0.63,0.69,0.35,0.3,0.21,0.45,0.61,0.47,0.51,0.83,0.44],[0.56,0.75,0.48,0.64,0.8,0.86,0.3,0.85,0.54,0.38,0.52,0.89,0.54,0.43,0.64],[0.37,0.25,0.29,0.29,0.31,0.3,0.65,0.33,0.44,0.83,0.53,0.67,0.32,0.33,0.23]]</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>[[1,5],[0,5],[2,5],[0,5],[1,5],[2,5],[1,5],[0,5],[2,5],[0,5],[2,5],[2,5],[2,5],[1,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[2,2,1,1,1,2,2,2,2,2]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>[1,1,1,2,2,1,1,1,1,2]</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>[40,80,40,60,90,50,30,90,100,30]</t>
         </is>
       </c>
     </row>
@@ -554,19 +634,37 @@
       <c r="B6" t="n">
         <v>15</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>[6, 7, 5, 1, 4, 2, 1, 10, 1, 3, 9, 4, 10, 6, 5]</t>
-        </is>
+      <c r="C6" t="n">
+        <v>5</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[[0.2087, 0.4865, 0.4678, 0.1853, 0.1172, 0.2215, 0.4447, 0.3114, 0.1195, 0.2121, 0.1781, 0.3781, 0.2685, 0.2201, 0.163], [0.2161, 0.1581, 0.3492, 0.2126, 0.4937, 0.3785, 0.4477, 0.2576, 0.4152, 0.4782, 0.4931, 0.1275, 0.1176, 0.1807, 0.3034], [0.4167, 0.4016, 0.2002, 0.1066, 0.3428, 0.4615, 0.2675, 0.4831, 0.3726, 0.2089, 0.2674, 0.2775, 0.1551, 0.3149, 0.2301], [0.4476, 0.3917, 0.4038, 0.3999, 0.4409, 0.4865, 0.3065, 0.2743, 0.2903, 0.2921, 0.1041, 0.242, 0.2978, 0.1836, 0.3671], [0.1467, 0.2227, 0.4379, 0.339, 0.331, 0.1633, 0.2896, 0.3333, 0.2002, 0.3569, 0.4589, 0.1432, 0.2686, 0.1964, 0.3239], [0.3402, 0.4849, 0.1867, 0.2305, 0.2673, 0.2175, 0.2902, 0.4572, 0.1442, 0.2048, 0.4154, 0.409, 0.1068, 0.1345, 0.2325], [0.3977, 0.3288, 0.3771, 0.2183, 0.39, 0.1272, 0.4961, 0.3127, 0.2892, 0.3824, 0.3383, 0.1434, 0.3193, 0.1937, 0.1209], [0.3716, 0.2833, 0.4586, 0.2496, 0.3718, 0.3948, 0.209, 0.2794, 0.3189, 0.4423, 0.2049, 0.4168, 0.34, 0.162, 0.3509], [0.2804, 0.375, 0.4086, 0.2814, 0.2874, 0.4008, 0.4241, 0.1395, 0.1565, 0.427, 0.4339, 0.335, 0.1621, 0.4896, 0.4899], [0.4469, 0.3271, 0.4351, 0.2798, 0.4839, 0.2998, 0.3805, 0.2046, 0.1336, 0.3308, 0.4115, 0.2185, 0.1549, 0.2622, 0.2184]]</t>
+          <t>[1,9,1,2,4,3,7,8,8,4,7,1,3,7,1]</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>[[0, 5], [0, 5], [0, 5], [1, 5], [1, 5], [3, 5], [3, 5], [0, 5], [3, 5], [3, 5], [1, 5], [0, 5], [0, 5], [2, 5], [2, 5]]</t>
+          <t>[[0.32,0.4,0.32,0.26,0.28,0.52,0.34,0.45,0.55,0.68,0.23,0.76,0.64,0.26,0.81],[0.84,0.24,0.39,0.76,0.72,0.33,0.35,0.46,0.54,0.63,0.46,0.52,0.72,0.23,0.38],[0.7,0.83,0.56,0.57,0.28,0.51,0.57,0.37,0.39,0.46,0.21,0.43,0.35,0.43,0.28],[0.82,0.62,0.68,0.75,0.55,0.26,0.58,0.61,0.72,0.5,0.29,0.4,0.45,0.65,0.6],[0.45,0.89,0.62,0.37,0.27,0.31,0.37,0.31,0.33,0.4,0.32,0.83,0.26,0.57,0.49],[0.89,0.28,0.48,0.88,0.81,0.77,0.38,0.32,0.67,0.85,0.59,0.6,0.4,0.74,0.33],[0.43,0.5,0.56,0.37,0.28,0.63,0.4,0.61,0.31,0.54,0.57,0.24,0.44,0.29,0.24],[0.89,0.43,0.77,0.38,0.68,0.73,0.62,0.53,0.49,0.44,0.85,0.78,0.88,0.29,0.71],[0.86,0.33,0.25,0.72,0.6,0.79,0.3,0.76,0.34,0.31,0.31,0.77,0.67,0.57,0.45],[0.81,0.47,0.77,0.51,0.46,0.52,0.41,0.72,0.55,0.36,0.83,0.47,0.58,0.83,0.64]]</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>[[1,5],[1,5],[1,5],[1,5],[1,5],[2,5],[2,5],[2,5],[2,5],[2,5],[1,5],[0,5],[0,5],[1,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>[1,1,2,1,1,2,1,1,1,1]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[1,1,1,2,1,1,1,1,2,2]</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>[60,50,70,50,60,80,40,60,90,70]</t>
         </is>
       </c>
     </row>
@@ -577,19 +675,37 @@
       <c r="B7" t="n">
         <v>15</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>[2, 1, 9, 6, 9, 9, 5, 6, 5, 8, 10, 6, 6, 8, 8]</t>
-        </is>
+      <c r="C7" t="n">
+        <v>5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>[[0.3748, 0.1177, 0.4246, 0.2176, 0.1431, 0.4064, 0.1161, 0.1182, 0.2894, 0.2221, 0.1116, 0.206, 0.2501, 0.322, 0.295], [0.3004, 0.4275, 0.2165, 0.106, 0.374, 0.4504, 0.1437, 0.2995, 0.1738, 0.1943, 0.4965, 0.2462, 0.4351, 0.3306, 0.1055], [0.312, 0.3194, 0.4734, 0.4845, 0.1205, 0.1526, 0.3166, 0.3843, 0.1253, 0.4224, 0.2643, 0.1364, 0.2611, 0.3531, 0.3668], [0.4411, 0.1231, 0.1965, 0.1272, 0.3817, 0.3637, 0.4016, 0.2325, 0.1397, 0.238, 0.1973, 0.1247, 0.3736, 0.1006, 0.3792], [0.3447, 0.1629, 0.3674, 0.2322, 0.3407, 0.371, 0.4107, 0.1544, 0.1413, 0.4761, 0.3027, 0.3905, 0.4448, 0.2737, 0.4233], [0.3892, 0.2363, 0.1861, 0.2393, 0.1745, 0.3986, 0.1984, 0.2583, 0.4958, 0.3818, 0.4368, 0.1231, 0.1237, 0.4691, 0.4283], [0.2774, 0.1738, 0.414, 0.1286, 0.3111, 0.4926, 0.2271, 0.4651, 0.4043, 0.1205, 0.3352, 0.1614, 0.2823, 0.243, 0.3078], [0.3289, 0.3379, 0.4054, 0.4958, 0.1029, 0.2353, 0.1966, 0.1441, 0.1313, 0.3862, 0.1487, 0.3056, 0.3273, 0.2084, 0.1035], [0.2594, 0.3636, 0.1975, 0.2156, 0.2415, 0.1551, 0.2181, 0.1603, 0.1481, 0.2825, 0.1275, 0.2863, 0.4805, 0.3839, 0.129], [0.3437, 0.3624, 0.1279, 0.2487, 0.4634, 0.488, 0.1743, 0.2682, 0.2374, 0.3357, 0.2994, 0.4781, 0.3286, 0.3123, 0.3882]]</t>
+          <t>[2,1,8,10,10,2,2,9,4,9,5,3,6,2,4]</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[[3, 5], [2, 5], [3, 5], [2, 5], [1, 5], [1, 5], [1, 5], [1, 5], [1, 5], [2, 5], [0, 5], [3, 5], [1, 5], [1, 5], [2, 5]]</t>
+          <t>[[0.28,0.86,0.64,0.43,0.3,0.76,0.63,0.57,0.83,0.75,0.31,0.42,0.37,0.72,0.22],[0.6,0.73,0.81,0.44,0.77,0.28,0.79,0.29,0.48,0.76,0.3,0.36,0.71,0.7,0.65],[0.69,0.58,0.38,0.44,0.33,0.84,0.61,0.48,0.52,0.86,0.31,0.61,0.55,0.63,0.21],[0.81,0.85,0.6,0.69,0.85,0.7,0.31,0.6,0.62,0.5,0.72,0.85,0.85,0.52,0.28],[0.89,0.79,0.29,0.84,0.81,0.56,0.61,0.48,0.24,0.43,0.76,0.2,0.43,0.48,0.58],[0.84,0.44,0.44,0.72,0.52,0.36,0.52,0.3,0.32,0.55,0.49,0.84,0.45,0.61,0.64],[0.21,0.66,0.32,0.87,0.3,0.49,0.26,0.9,0.55,0.62,0.25,0.72,0.35,0.83,0.34],[0.33,0.23,0.53,0.6,0.25,0.74,0.52,0.57,0.51,0.48,0.59,0.31,0.33,0.8,0.86],[0.46,0.39,0.65,0.49,0.22,0.31,0.7,0.66,0.22,0.36,0.36,0.67,0.21,0.27,0.76],[0.32,0.66,0.37,0.27,0.37,0.71,0.8,0.78,0.48,0.67,0.34,0.41,0.83,0.21,0.26]]</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>[[1,5],[1,5],[0,5],[1,5],[2,5],[2,5],[1,5],[2,5],[2,5],[2,5],[0,5],[2,5],[2,5],[1,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>[1,1,2,1,1,1,2,2,1,2]</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[1,2,2,2,1,1,2,2,1,1]</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>[70,40,60,40,90,100,80,100,20,30]</t>
         </is>
       </c>
     </row>
@@ -600,19 +716,37 @@
       <c r="B8" t="n">
         <v>15</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>[10, 4, 1, 3, 5, 3, 6, 6, 6, 5, 9, 10, 9, 1, 1]</t>
-        </is>
+      <c r="C8" t="n">
+        <v>5</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>[[0.2271, 0.4932, 0.1325, 0.4993, 0.4217, 0.2644, 0.1886, 0.4673, 0.3539, 0.3736, 0.3948, 0.486, 0.3332, 0.2509, 0.1689], [0.3048, 0.3439, 0.1072, 0.4222, 0.3681, 0.297, 0.2294, 0.3199, 0.4614, 0.3595, 0.2691, 0.4036, 0.143, 0.3318, 0.1208], [0.1969, 0.3803, 0.1998, 0.2444, 0.1847, 0.324, 0.4392, 0.4748, 0.3231, 0.2002, 0.4216, 0.1604, 0.493, 0.3418, 0.497], [0.1705, 0.4398, 0.3382, 0.1319, 0.2143, 0.3254, 0.489, 0.1836, 0.1885, 0.3973, 0.2238, 0.2581, 0.1349, 0.4523, 0.1183], [0.4839, 0.1735, 0.4514, 0.4355, 0.4297, 0.2551, 0.3236, 0.3074, 0.3023, 0.1602, 0.3371, 0.3923, 0.1506, 0.2253, 0.1147], [0.2155, 0.3793, 0.2286, 0.1342, 0.2002, 0.2223, 0.2874, 0.3184, 0.2854, 0.295, 0.3629, 0.4024, 0.2757, 0.3484, 0.4376], [0.1025, 0.4494, 0.3533, 0.4488, 0.2636, 0.3928, 0.4593, 0.4341, 0.1939, 0.1488, 0.1811, 0.3326, 0.4934, 0.3689, 0.4776], [0.3045, 0.367, 0.1592, 0.418, 0.408, 0.2171, 0.4683, 0.4438, 0.4884, 0.3877, 0.162, 0.1613, 0.2426, 0.3794, 0.1928], [0.1037, 0.1262, 0.4105, 0.4477, 0.4407, 0.2919, 0.4127, 0.392, 0.2655, 0.4049, 0.49, 0.1678, 0.4042, 0.1994, 0.4206], [0.385, 0.2683, 0.3708, 0.2789, 0.3059, 0.4137, 0.2113, 0.2788, 0.1149, 0.1811, 0.1166, 0.3511, 0.4097, 0.1727, 0.3983]]</t>
+          <t>[2,3,9,1,6,10,9,3,7,3,1,5,6,1,6]</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>[[1, 5], [3, 5], [1, 5], [3, 5], [1, 5], [1, 5], [2, 5], [3, 5], [2, 5], [2, 5], [0, 5], [1, 5], [0, 5], [1, 5], [2, 5]]</t>
+          <t>[[0.35,0.22,0.33,0.61,0.49,0.82,0.77,0.44,0.38,0.47,0.61,0.39,0.64,0.49,0.59],[0.51,0.41,0.86,0.73,0.3,0.81,0.54,0.83,0.76,0.5,0.22,0.39,0.58,0.64,0.38],[0.3,0.78,0.89,0.57,0.32,0.39,0.21,0.84,0.28,0.6,0.39,0.59,0.66,0.78,0.34],[0.21,0.3,0.83,0.81,0.62,0.62,0.67,0.32,0.84,0.49,0.47,0.56,0.23,0.32,0.72],[0.26,0.62,0.37,0.47,0.4,0.45,0.7,0.41,0.6,0.53,0.66,0.86,0.71,0.35,0.22],[0.38,0.62,0.24,0.55,0.62,0.43,0.74,0.27,0.25,0.71,0.55,0.68,0.5,0.37,0.77],[0.76,0.69,0.39,0.61,0.45,0.26,0.84,0.3,0.87,0.51,0.33,0.58,0.81,0.71,0.76],[0.66,0.68,0.79,0.37,0.54,0.35,0.89,0.86,0.23,0.69,0.85,0.33,0.6,0.84,0.22],[0.69,0.41,0.85,0.88,0.86,0.53,0.8,0.79,0.42,0.78,0.23,0.62,0.36,0.28,0.25],[0.69,0.44,0.71,0.25,0.42,0.58,0.75,0.42,0.64,0.82,0.63,0.36,0.22,0.81,0.21]]</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[0,5],[2,5],[0,5],[1,5],[2,5],[1,5],[2,5],[2,5],[0,5],[0,5],[0,5],[0,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,1,2,1,1,2,1]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,2,2,1,1,1,1]</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>[80,70,60,30,60,70,100,80,100,70]</t>
         </is>
       </c>
     </row>
@@ -623,19 +757,37 @@
       <c r="B9" t="n">
         <v>15</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>[9, 3, 6, 5, 9, 3, 1, 8, 7, 10, 1, 2, 7, 3, 3]</t>
-        </is>
+      <c r="C9" t="n">
+        <v>5</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>[[0.2026, 0.1344, 0.4369, 0.3075, 0.4358, 0.4844, 0.3317, 0.3506, 0.2916, 0.2354, 0.3577, 0.1115, 0.3177, 0.4553, 0.3637], [0.3687, 0.4374, 0.1234, 0.2347, 0.4556, 0.1259, 0.3869, 0.4809, 0.2037, 0.4036, 0.1411, 0.3551, 0.286, 0.3026, 0.1125], [0.4092, 0.2363, 0.3005, 0.4708, 0.4602, 0.4255, 0.1023, 0.4538, 0.1293, 0.443, 0.4905, 0.464, 0.3383, 0.3943, 0.4635], [0.182, 0.3783, 0.3697, 0.2107, 0.3746, 0.3246, 0.1712, 0.2698, 0.3723, 0.1498, 0.4509, 0.4935, 0.4333, 0.4012, 0.1403], [0.4855, 0.2681, 0.2488, 0.1749, 0.4842, 0.3598, 0.2956, 0.4867, 0.1058, 0.3825, 0.1552, 0.1247, 0.3751, 0.4597, 0.1628], [0.43, 0.3504, 0.3822, 0.1034, 0.1613, 0.1266, 0.4282, 0.3907, 0.4944, 0.3162, 0.3072, 0.4572, 0.1194, 0.2389, 0.1782], [0.2475, 0.1467, 0.3564, 0.43, 0.4503, 0.2113, 0.4924, 0.4001, 0.444, 0.4634, 0.4802, 0.1266, 0.4954, 0.3442, 0.4999], [0.255, 0.4965, 0.2358, 0.3219, 0.1259, 0.2544, 0.1239, 0.1615, 0.172, 0.4953, 0.3096, 0.3981, 0.4238, 0.3319, 0.281], [0.494, 0.1058, 0.2527, 0.1902, 0.4057, 0.407, 0.365, 0.4191, 0.4053, 0.4702, 0.4663, 0.1234, 0.1583, 0.1336, 0.1747], [0.2694, 0.1012, 0.2099, 0.2281, 0.3832, 0.3289, 0.4195, 0.2326, 0.4792, 0.1667, 0.2304, 0.3115, 0.3446, 0.3916, 0.3394]]</t>
+          <t>[1,2,5,3,10,5,1,2,10,7,6,6,7,10,9]</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>[[2, 5], [3, 5], [1, 5], [1, 5], [1, 5], [2, 5], [1, 5], [0, 5], [0, 5], [1, 5], [2, 5], [2, 5], [1, 5], [1, 5], [0, 5]]</t>
+          <t>[[0.81,0.57,0.86,0.76,0.9,0.45,0.74,0.48,0.54,0.64,0.81,0.89,0.74,0.49,0.49],[0.72,0.37,0.28,0.45,0.4,0.41,0.36,0.23,0.21,0.89,0.5,0.47,0.68,0.35,0.86],[0.75,0.26,0.49,0.82,0.86,0.53,0.63,0.32,0.89,0.36,0.86,0.65,0.63,0.56,0.36],[0.32,0.35,0.33,0.75,0.45,0.24,0.88,0.82,0.85,0.9,0.32,0.48,0.73,0.69,0.31],[0.77,0.36,0.36,0.58,0.62,0.61,0.26,0.81,0.39,0.29,0.82,0.87,0.8,0.77,0.66],[0.59,0.26,0.49,0.46,0.38,0.71,0.55,0.26,0.35,0.68,0.25,0.8,0.55,0.54,0.61],[0.78,0.44,0.67,0.6,0.39,0.82,0.76,0.66,0.8,0.81,0.7,0.79,0.69,0.68,0.63],[0.73,0.31,0.82,0.81,0.22,0.78,0.29,0.43,0.72,0.31,0.77,0.78,0.56,0.2,0.4],[0.63,0.89,0.64,0.38,0.64,0.58,0.75,0.27,0.73,0.58,0.87,0.44,0.64,0.85,0.27],[0.86,0.68,0.25,0.41,0.7,0.25,0.61,0.44,0.63,0.23,0.81,0.88,0.88,0.72,0.29]]</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>[[0,5],[1,5],[2,5],[0,5],[1,5],[0,5],[2,5],[1,5],[0,5],[2,5],[2,5],[2,5],[2,5],[2,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>[1,2,2,1,2,2,1,2,2,2]</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>[2,2,2,1,1,2,2,1,2,2]</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>[100,20,60,60,50,80,70,90,90,90]</t>
         </is>
       </c>
     </row>
@@ -646,19 +798,37 @@
       <c r="B10" t="n">
         <v>15</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>[5, 10, 3, 3, 9, 4, 10, 7, 2, 5, 5, 1, 1, 2, 7]</t>
-        </is>
+      <c r="C10" t="n">
+        <v>5</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>[[0.2055, 0.4433, 0.188, 0.4766, 0.2059, 0.2847, 0.2115, 0.1237, 0.4617, 0.4471, 0.241, 0.3377, 0.331, 0.1086, 0.1057], [0.1671, 0.492, 0.1238, 0.4506, 0.4879, 0.4721, 0.1829, 0.4948, 0.2568, 0.2863, 0.27, 0.4112, 0.2022, 0.2169, 0.4139], [0.311, 0.125, 0.1636, 0.1498, 0.4692, 0.3413, 0.4194, 0.2358, 0.3484, 0.2631, 0.3925, 0.2203, 0.279, 0.3934, 0.3244], [0.2375, 0.4513, 0.3538, 0.3275, 0.119, 0.4865, 0.2392, 0.2997, 0.3361, 0.4544, 0.1627, 0.178, 0.4101, 0.1258, 0.2691], [0.4429, 0.413, 0.1153, 0.3499, 0.4261, 0.1965, 0.4268, 0.4961, 0.1966, 0.2874, 0.2651, 0.1515, 0.3386, 0.3234, 0.2641], [0.492, 0.3398, 0.207, 0.3043, 0.4281, 0.1143, 0.3983, 0.1587, 0.4596, 0.4027, 0.246, 0.2266, 0.3136, 0.234, 0.1487], [0.2747, 0.2813, 0.4814, 0.2763, 0.1932, 0.29, 0.3938, 0.2995, 0.321, 0.3049, 0.4396, 0.3957, 0.2279, 0.1972, 0.2231], [0.3171, 0.4927, 0.1714, 0.2755, 0.1863, 0.1907, 0.3896, 0.399, 0.3301, 0.2602, 0.4806, 0.4609, 0.1749, 0.2989, 0.4569], [0.2771, 0.2958, 0.3698, 0.2727, 0.465, 0.2361, 0.1644, 0.2609, 0.4537, 0.1313, 0.3497, 0.4338, 0.2628, 0.4309, 0.1007], [0.3519, 0.3376, 0.1261, 0.1443, 0.2762, 0.403, 0.1507, 0.2001, 0.4639, 0.4924, 0.1887, 0.2389, 0.2137, 0.362, 0.1023]]</t>
+          <t>[4,9,8,3,2,5,9,10,6,2,4,5,4,4,3]</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>[[0, 5], [3, 5], [1, 5], [2, 5], [2, 5], [1, 5], [0, 5], [1, 5], [3, 5], [3, 5], [0, 5], [1, 5], [0, 5], [2, 5], [2, 5]]</t>
+          <t>[[0.73,0.22,0.22,0.43,0.54,0.74,0.68,0.51,0.39,0.9,0.5,0.52,0.31,0.76,0.69],[0.35,0.26,0.68,0.66,0.39,0.87,0.31,0.5,0.86,0.49,0.65,0.48,0.39,0.89,0.49],[0.83,0.36,0.35,0.22,0.66,0.46,0.81,0.53,0.88,0.33,0.81,0.74,0.74,0.79,0.73],[0.64,0.29,0.22,0.84,0.63,0.76,0.54,0.28,0.29,0.68,0.5,0.34,0.54,0.24,0.61],[0.39,0.76,0.42,0.52,0.21,0.25,0.47,0.54,0.62,0.4,0.69,0.8,0.75,0.23,0.54],[0.27,0.37,0.89,0.3,0.55,0.63,0.69,0.59,0.21,0.43,0.56,0.26,0.45,0.22,0.26],[0.48,0.29,0.6,0.68,0.76,0.34,0.32,0.27,0.65,0.69,0.22,0.86,0.24,0.58,0.7],[0.81,0.7,0.76,0.44,0.77,0.26,0.83,0.58,0.77,0.52,0.65,0.57,0.71,0.26,0.24],[0.37,0.31,0.81,0.35,0.88,0.44,0.33,0.75,0.66,0.55,0.59,0.7,0.36,0.9,0.88],[0.66,0.34,0.68,0.25,0.22,0.38,0.52,0.81,0.71,0.72,0.5,0.44,0.46,0.89,0.23]]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>[[0,5],[0,5],[0,5],[1,5],[2,5],[0,5],[1,5],[1,5],[2,5],[2,5],[0,5],[2,5],[2,5],[1,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>[2,1,1,1,1,2,1,1,2,1]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>[1,1,2,1,2,2,2,2,2,1]</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>[90,90,60,50,60,100,90,50,60,90]</t>
         </is>
       </c>
     </row>
@@ -669,19 +839,37 @@
       <c r="B11" t="n">
         <v>15</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>[3, 8, 6, 1, 6, 8, 10, 7, 6, 6, 3, 6, 3, 1, 6]</t>
-        </is>
+      <c r="C11" t="n">
+        <v>5</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>[[0.2878, 0.3724, 0.3398, 0.4376, 0.1442, 0.4895, 0.1045, 0.2503, 0.397, 0.2474, 0.2042, 0.1884, 0.3051, 0.4065, 0.3511], [0.2828, 0.121, 0.3812, 0.1225, 0.371, 0.137, 0.4155, 0.2219, 0.4411, 0.4253, 0.3387, 0.4652, 0.3471, 0.4717, 0.4917], [0.4938, 0.369, 0.2434, 0.1079, 0.2142, 0.2968, 0.319, 0.1204, 0.3382, 0.4155, 0.3476, 0.1915, 0.3737, 0.4852, 0.2746], [0.166, 0.3604, 0.282, 0.4308, 0.2273, 0.1015, 0.2616, 0.4954, 0.4255, 0.4679, 0.4302, 0.2732, 0.2052, 0.1058, 0.1775], [0.4431, 0.1095, 0.1881, 0.1446, 0.3389, 0.1249, 0.1398, 0.1762, 0.4208, 0.3549, 0.2073, 0.2475, 0.1131, 0.4716, 0.4205], [0.1923, 0.1776, 0.2931, 0.4253, 0.4349, 0.1662, 0.4106, 0.4644, 0.3673, 0.411, 0.2718, 0.244, 0.1205, 0.1747, 0.362], [0.2624, 0.3902, 0.4286, 0.367, 0.1979, 0.1411, 0.3309, 0.3425, 0.42, 0.2245, 0.3014, 0.4757, 0.2791, 0.3739, 0.2425], [0.4036, 0.1608, 0.2319, 0.1157, 0.4014, 0.2751, 0.1976, 0.4254, 0.2, 0.2603, 0.2569, 0.2695, 0.4239, 0.4936, 0.4209], [0.253, 0.4888, 0.3249, 0.1495, 0.268, 0.3757, 0.1603, 0.1027, 0.4598, 0.1689, 0.2307, 0.1891, 0.2804, 0.1705, 0.4716], [0.4652, 0.3994, 0.3448, 0.4269, 0.2649, 0.3473, 0.4613, 0.3821, 0.3857, 0.3189, 0.4457, 0.2936, 0.394, 0.1343, 0.1869]]</t>
+          <t>[2,5,4,5,6,6,9,2,3,3,4,7,3,4,2]</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[[1, 5], [3, 5], [1, 5], [1, 5], [1, 5], [3, 5], [3, 5], [3, 5], [1, 5], [3, 5], [2, 5], [1, 5], [1, 5], [0, 5], [0, 5]]</t>
+          <t>[[0.81,0.61,0.51,0.71,0.54,0.81,0.83,0.5,0.39,0.61,0.84,0.35,0.64,0.64,0.71],[0.29,0.7,0.84,0.33,0.37,0.88,0.33,0.8,0.54,0.37,0.81,0.51,0.56,0.45,0.62],[0.31,0.47,0.88,0.38,0.66,0.43,0.74,0.29,0.88,0.52,0.37,0.25,0.32,0.56,0.44],[0.78,0.5,0.37,0.63,0.69,0.32,0.32,0.23,0.72,0.66,0.53,0.79,0.76,0.61,0.81],[0.34,0.28,0.39,0.24,0.57,0.86,0.23,0.29,0.52,0.85,0.42,0.56,0.23,0.3,0.89],[0.88,0.2,0.87,0.65,0.81,0.52,0.56,0.54,0.67,0.3,0.22,0.42,0.69,0.34,0.67],[0.88,0.27,0.67,0.51,0.81,0.32,0.68,0.79,0.86,0.68,0.55,0.63,0.81,0.6,0.22],[0.85,0.68,0.67,0.35,0.66,0.48,0.66,0.27,0.66,0.9,0.23,0.88,0.48,0.81,0.75],[0.6,0.72,0.81,0.48,0.43,0.67,0.77,0.73,0.76,0.5,0.77,0.28,0.58,0.2,0.43],[0.46,0.48,0.69,0.47,0.51,0.37,0.46,0.36,0.25,0.62,0.67,0.63,0.52,0.47,0.8]]</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>[[1,5],[1,5],[1,5],[2,5],[1,5],[1,5],[0,5],[0,5],[1,5],[1,5],[2,5],[2,5],[0,5],[2,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>[2,1,2,2,2,2,1,2,1,2]</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>[2,2,1,2,2,2,1,2,1,1]</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>[80,20,30,80,40,90,40,20,60,80]</t>
         </is>
       </c>
     </row>
@@ -692,19 +880,37 @@
       <c r="B12" t="n">
         <v>15</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>[4, 5, 2, 8, 7, 4, 4, 5, 3, 4, 4, 10, 9, 4, 5]</t>
-        </is>
+      <c r="C12" t="n">
+        <v>5</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>[[0.4187, 0.4163, 0.4797, 0.3443, 0.3687, 0.2455, 0.1831, 0.1883, 0.2529, 0.2672, 0.1924, 0.1141, 0.4983, 0.441, 0.4206], [0.2918, 0.4316, 0.4055, 0.442, 0.3622, 0.1735, 0.3121, 0.4145, 0.2922, 0.1817, 0.4409, 0.2986, 0.4608, 0.4107, 0.2982], [0.2603, 0.476, 0.4689, 0.1976, 0.4039, 0.1916, 0.1097, 0.1969, 0.1508, 0.2709, 0.3864, 0.136, 0.2278, 0.1449, 0.2818], [0.4136, 0.4489, 0.4291, 0.1345, 0.2323, 0.2962, 0.2036, 0.4729, 0.1697, 0.282, 0.3332, 0.3879, 0.2828, 0.1919, 0.4635], [0.119, 0.1121, 0.1345, 0.3418, 0.3016, 0.4535, 0.2878, 0.3928, 0.2148, 0.1151, 0.3024, 0.3577, 0.3407, 0.1424, 0.4511], [0.1868, 0.2689, 0.1232, 0.1237, 0.3391, 0.2802, 0.4268, 0.2637, 0.3427, 0.1636, 0.2295, 0.3651, 0.4473, 0.2337, 0.2057], [0.495, 0.1402, 0.1361, 0.4705, 0.3414, 0.4596, 0.4012, 0.4072, 0.1863, 0.1573, 0.2951, 0.2776, 0.1589, 0.4314, 0.2754], [0.2482, 0.4655, 0.2531, 0.4425, 0.2178, 0.3462, 0.1545, 0.3166, 0.4727, 0.2459, 0.4663, 0.3454, 0.1992, 0.3668, 0.2144], [0.2228, 0.2835, 0.4566, 0.4629, 0.39, 0.439, 0.135, 0.4908, 0.451, 0.2894, 0.2871, 0.3652, 0.3529, 0.4572, 0.4152], [0.3887, 0.39, 0.2871, 0.2114, 0.126, 0.2438, 0.3931, 0.1893, 0.1384, 0.1018, 0.4178, 0.3758, 0.2709, 0.1646, 0.3744]]</t>
+          <t>[6,4,8,6,6,7,5,7,5,2,8,1,9,1,6]</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>[[1, 5], [2, 5], [2, 5], [2, 5], [0, 5], [2, 5], [1, 5], [2, 5], [0, 5], [3, 5], [2, 5], [1, 5], [0, 5], [1, 5], [2, 5]]</t>
+          <t>[[0.56,0.54,0.22,0.44,0.47,0.48,0.61,0.57,0.63,0.74,0.77,0.7,0.87,0.21,0.34],[0.21,0.65,0.83,0.37,0.85,0.24,0.85,0.45,0.27,0.54,0.38,0.4,0.42,0.76,0.58],[0.42,0.63,0.7,0.39,0.49,0.29,0.33,0.68,0.33,0.57,0.7,0.27,0.6,0.38,0.87],[0.54,0.76,0.59,0.23,0.64,0.87,0.62,0.77,0.82,0.36,0.35,0.63,0.49,0.79,0.83],[0.45,0.37,0.75,0.39,0.78,0.5,0.67,0.27,0.64,0.52,0.61,0.32,0.72,0.8,0.35],[0.27,0.22,0.65,0.62,0.58,0.36,0.47,0.62,0.55,0.89,0.3,0.69,0.48,0.5,0.7],[0.68,0.89,0.29,0.27,0.71,0.6,0.39,0.26,0.26,0.83,0.33,0.43,0.36,0.45,0.25],[0.56,0.25,0.76,0.36,0.58,0.82,0.66,0.57,0.43,0.43,0.67,0.9,0.66,0.59,0.71],[0.53,0.24,0.59,0.87,0.32,0.68,0.34,0.58,0.27,0.52,0.73,0.44,0.67,0.76,0.85],[0.36,0.48,0.31,0.89,0.85,0.58,0.79,0.56,0.64,0.26,0.73,0.29,0.78,0.75,0.7]]</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[0,5],[2,5],[0,5],[0,5],[0,5],[0,5],[0,5],[2,5],[0,5],[0,5],[0,5],[1,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,2,1,1,1,2,1]</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>[1,2,2,2,1,1,1,1,2,1]</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>[20,70,100,80,70,30,100,70,20,80]</t>
         </is>
       </c>
     </row>
@@ -715,19 +921,37 @@
       <c r="B13" t="n">
         <v>15</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>[4, 9, 10, 5, 6, 9, 6, 5, 7, 5, 6, 7, 8, 8, 6]</t>
-        </is>
+      <c r="C13" t="n">
+        <v>5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>[[0.1735, 0.1376, 0.3697, 0.1297, 0.3716, 0.1884, 0.3268, 0.1351, 0.1932, 0.1617, 0.4462, 0.3411, 0.1482, 0.1713, 0.1011], [0.4116, 0.1843, 0.1177, 0.3458, 0.2478, 0.3485, 0.3272, 0.4163, 0.1784, 0.2011, 0.4649, 0.4822, 0.1309, 0.25, 0.2586], [0.212, 0.2067, 0.1624, 0.3682, 0.4446, 0.2931, 0.2037, 0.4293, 0.1605, 0.4431, 0.4113, 0.2545, 0.395, 0.4506, 0.4495], [0.2774, 0.4522, 0.3094, 0.4824, 0.3348, 0.2185, 0.1619, 0.3248, 0.4737, 0.4276, 0.2276, 0.2496, 0.227, 0.1527, 0.4116], [0.1883, 0.4164, 0.2121, 0.1843, 0.459, 0.2358, 0.2987, 0.4584, 0.4626, 0.3705, 0.3099, 0.4433, 0.4003, 0.4659, 0.3873], [0.4091, 0.4648, 0.2683, 0.1208, 0.2826, 0.4832, 0.3235, 0.1034, 0.3779, 0.2642, 0.3105, 0.346, 0.4459, 0.1898, 0.453], [0.2988, 0.3852, 0.4534, 0.41, 0.1014, 0.321, 0.4031, 0.3041, 0.412, 0.3986, 0.2878, 0.146, 0.3179, 0.2555, 0.4524], [0.4348, 0.4944, 0.4681, 0.177, 0.4222, 0.197, 0.3073, 0.3831, 0.3695, 0.4851, 0.243, 0.1602, 0.1967, 0.3189, 0.294], [0.4311, 0.1068, 0.2771, 0.264, 0.4699, 0.199, 0.1477, 0.4182, 0.4054, 0.2699, 0.2188, 0.2839, 0.2524, 0.4674, 0.1917], [0.1729, 0.2177, 0.235, 0.3192, 0.1548, 0.4562, 0.3381, 0.2844, 0.4793, 0.1383, 0.3086, 0.4772, 0.4435, 0.1416, 0.4801]]</t>
+          <t>[8,2,7,6,8,3,7,3,9,5,10,9,8,8,7]</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>[[1, 5], [3, 5], [1, 5], [1, 5], [3, 5], [0, 5], [3, 5], [3, 5], [2, 5], [2, 5], [2, 5], [0, 5], [3, 5], [2, 5], [0, 5]]</t>
+          <t>[[0.23,0.41,0.38,0.45,0.26,0.86,0.59,0.41,0.48,0.51,0.62,0.56,0.84,0.55,0.89],[0.8,0.35,0.85,0.28,0.77,0.47,0.81,0.81,0.76,0.75,0.41,0.26,0.48,0.32,0.69],[0.44,0.88,0.65,0.78,0.29,0.8,0.85,0.54,0.62,0.74,0.32,0.55,0.48,0.3,0.46],[0.25,0.22,0.29,0.87,0.58,0.88,0.5,0.42,0.55,0.51,0.27,0.65,0.35,0.63,0.66],[0.31,0.24,0.75,0.52,0.24,0.9,0.24,0.69,0.89,0.37,0.3,0.28,0.41,0.27,0.68],[0.24,0.56,0.9,0.77,0.63,0.41,0.64,0.57,0.5,0.29,0.82,0.51,0.34,0.46,0.49],[0.78,0.71,0.74,0.21,0.49,0.54,0.21,0.38,0.73,0.3,0.57,0.35,0.21,0.37,0.88],[0.76,0.87,0.54,0.28,0.58,0.52,0.79,0.27,0.54,0.31,0.43,0.72,0.53,0.46,0.48],[0.52,0.75,0.82,0.87,0.75,0.42,0.68,0.51,0.38,0.79,0.23,0.83,0.52,0.65,0.66],[0.83,0.65,0.63,0.25,0.56,0.31,0.72,0.56,0.68,0.23,0.26,0.7,0.25,0.25,0.21]]</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>[[2,5],[2,5],[1,5],[1,5],[0,5],[0,5],[1,5],[1,5],[0,5],[1,5],[2,5],[2,5],[2,5],[1,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>[1,2,2,1,2,1,2,2,2,2]</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>[2,1,1,1,1,2,2,1,2,2]</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>[90,20,30,60,50,80,50,60,70,90]</t>
         </is>
       </c>
     </row>
@@ -738,19 +962,37 @@
       <c r="B14" t="n">
         <v>15</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>[5, 4, 2, 3, 4, 9, 3, 3, 9, 4, 9, 10, 3, 3, 5]</t>
-        </is>
+      <c r="C14" t="n">
+        <v>5</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>[[0.2198, 0.213, 0.4826, 0.2209, 0.2009, 0.3225, 0.4361, 0.2582, 0.238, 0.2434, 0.3844, 0.1442, 0.4161, 0.3743, 0.1373], [0.4214, 0.3023, 0.2845, 0.1526, 0.2102, 0.3629, 0.2771, 0.235, 0.1855, 0.2108, 0.2833, 0.1615, 0.3707, 0.2512, 0.4911], [0.1875, 0.2221, 0.1994, 0.3497, 0.3825, 0.2856, 0.3229, 0.3467, 0.2796, 0.2657, 0.2186, 0.1081, 0.2265, 0.216, 0.2073], [0.125, 0.3651, 0.2509, 0.1638, 0.1682, 0.4951, 0.4998, 0.3948, 0.1166, 0.3703, 0.1963, 0.1953, 0.2315, 0.3756, 0.1745], [0.3444, 0.3699, 0.4765, 0.1013, 0.1072, 0.3373, 0.3181, 0.4188, 0.1835, 0.2781, 0.2393, 0.4238, 0.3356, 0.395, 0.1383], [0.1005, 0.3594, 0.2222, 0.1859, 0.4432, 0.4422, 0.409, 0.3018, 0.3615, 0.1527, 0.1963, 0.193, 0.2481, 0.4272, 0.2716], [0.2345, 0.266, 0.3048, 0.1813, 0.1126, 0.2166, 0.1313, 0.173, 0.4603, 0.1604, 0.1226, 0.3967, 0.1797, 0.4296, 0.3642], [0.276, 0.2786, 0.336, 0.4943, 0.2857, 0.1489, 0.1117, 0.466, 0.2746, 0.4146, 0.4557, 0.4202, 0.1923, 0.4825, 0.2648], [0.2388, 0.102, 0.2794, 0.25, 0.3395, 0.1317, 0.2175, 0.471, 0.4806, 0.3017, 0.415, 0.2937, 0.4703, 0.4154, 0.2252], [0.425, 0.243, 0.1516, 0.4308, 0.466, 0.4612, 0.3853, 0.3948, 0.2595, 0.3934, 0.3248, 0.3457, 0.3594, 0.1163, 0.246]]</t>
+          <t>[9,9,6,7,9,6,6,8,5,5,5,4,2,4,6]</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>[[2, 5], [3, 5], [1, 5], [2, 5], [3, 5], [1, 5], [3, 5], [0, 5], [1, 5], [0, 5], [0, 5], [2, 5], [0, 5], [1, 5], [0, 5]]</t>
+          <t>[[0.87,0.72,0.45,0.41,0.44,0.74,0.66,0.33,0.32,0.27,0.66,0.74,0.39,0.21,0.26],[0.88,0.41,0.74,0.64,0.47,0.34,0.28,0.63,0.74,0.65,0.57,0.23,0.88,0.76,0.4],[0.89,0.62,0.61,0.72,0.77,0.66,0.29,0.44,0.85,0.36,0.46,0.5,0.51,0.63,0.86],[0.37,0.29,0.34,0.82,0.65,0.4,0.77,0.8,0.79,0.84,0.38,0.73,0.52,0.79,0.71],[0.74,0.66,0.32,0.58,0.89,0.86,0.23,0.32,0.29,0.71,0.77,0.35,0.55,0.79,0.71],[0.58,0.61,0.56,0.41,0.6,0.68,0.81,0.65,0.73,0.31,0.52,0.21,0.37,0.71,0.89],[0.27,0.48,0.76,0.34,0.59,0.71,0.63,0.33,0.45,0.75,0.59,0.2,0.73,0.22,0.72],[0.34,0.87,0.46,0.43,0.3,0.41,0.81,0.9,0.46,0.51,0.71,0.82,0.62,0.47,0.49],[0.69,0.2,0.63,0.45,0.76,0.27,0.61,0.54,0.65,0.25,0.61,0.59,0.59,0.62,0.67],[0.76,0.39,0.78,0.55,0.25,0.24,0.43,0.75,0.7,0.75,0.56,0.51,0.3,0.43,0.5]]</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[2,5],[2,5],[0,5],[0,5],[0,5],[2,5],[1,5],[1,5],[2,5],[2,5],[2,5],[2,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>[1,1,2,1,2,1,2,1,1,2]</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>[1,1,2,1,2,1,1,2,2,2]</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>[90,70,40,20,60,90,30,30,80,90]</t>
         </is>
       </c>
     </row>
@@ -761,19 +1003,37 @@
       <c r="B15" t="n">
         <v>15</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>[4, 6, 2, 1, 8, 6, 6, 10, 5, 3, 7, 4, 1, 9, 1]</t>
-        </is>
+      <c r="C15" t="n">
+        <v>5</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>[[0.2528, 0.1399, 0.1621, 0.2778, 0.3193, 0.1633, 0.1562, 0.1239, 0.3113, 0.143, 0.3922, 0.3302, 0.1871, 0.3073, 0.3669], [0.211, 0.4428, 0.4079, 0.2802, 0.276, 0.1432, 0.2096, 0.1254, 0.1445, 0.4112, 0.2637, 0.1309, 0.4165, 0.218, 0.142], [0.2151, 0.3056, 0.3509, 0.231, 0.3429, 0.1687, 0.2943, 0.1971, 0.212, 0.3162, 0.2996, 0.1743, 0.1514, 0.4029, 0.4487], [0.3455, 0.2971, 0.3185, 0.3519, 0.3753, 0.332, 0.1902, 0.2062, 0.3738, 0.3012, 0.384, 0.4014, 0.4155, 0.2983, 0.2882], [0.1959, 0.2466, 0.4756, 0.3262, 0.132, 0.1974, 0.4367, 0.2234, 0.2592, 0.2735, 0.3228, 0.1186, 0.168, 0.3181, 0.2879], [0.3175, 0.3465, 0.2992, 0.3802, 0.4787, 0.4343, 0.1437, 0.4804, 0.4023, 0.2347, 0.2065, 0.3531, 0.4766, 0.4634, 0.4199], [0.3778, 0.1434, 0.1241, 0.4822, 0.4797, 0.1079, 0.3619, 0.3217, 0.2379, 0.23, 0.4778, 0.4209, 0.3683, 0.496, 0.2897], [0.1435, 0.3348, 0.3367, 0.2464, 0.3372, 0.3395, 0.4597, 0.1068, 0.4585, 0.1375, 0.4512, 0.5, 0.2211, 0.4789, 0.4231], [0.1892, 0.2685, 0.225, 0.1465, 0.4845, 0.407, 0.2291, 0.2562, 0.4548, 0.2858, 0.1898, 0.2577, 0.2995, 0.408, 0.3145], [0.2684, 0.3605, 0.3888, 0.406, 0.4644, 0.4426, 0.1732, 0.2093, 0.3699, 0.4071, 0.313, 0.1565, 0.1967, 0.4054, 0.3552]]</t>
+          <t>[2,10,1,3,3,10,5,2,4,2,9,7,10,10,10]</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>[[1, 5], [3, 5], [3, 5], [0, 5], [3, 5], [0, 5], [3, 5], [3, 5], [1, 5], [1, 5], [3, 5], [1, 5], [0, 5], [1, 5], [0, 5]]</t>
+          <t>[[0.26,0.35,0.62,0.71,0.9,0.85,0.65,0.49,0.65,0.75,0.28,0.49,0.79,0.47,0.6],[0.61,0.33,0.45,0.43,0.22,0.22,0.78,0.39,0.56,0.41,0.86,0.38,0.5,0.81,0.79],[0.33,0.76,0.52,0.54,0.29,0.26,0.71,0.55,0.51,0.71,0.74,0.31,0.63,0.29,0.73],[0.66,0.87,0.25,0.24,0.4,0.38,0.37,0.83,0.37,0.39,0.73,0.51,0.74,0.25,0.54],[0.22,0.24,0.83,0.3,0.57,0.49,0.44,0.83,0.22,0.66,0.87,0.59,0.86,0.24,0.49],[0.38,0.71,0.89,0.38,0.66,0.34,0.6,0.52,0.88,0.63,0.44,0.28,0.31,0.36,0.38],[0.8,0.59,0.57,0.28,0.8,0.71,0.25,0.7,0.58,0.26,0.52,0.54,0.32,0.86,0.79],[0.67,0.52,0.49,0.66,0.58,0.24,0.56,0.76,0.52,0.24,0.75,0.34,0.38,0.32,0.43],[0.73,0.56,0.34,0.81,0.82,0.81,0.37,0.52,0.89,0.74,0.22,0.25,0.52,0.84,0.58],[0.55,0.27,0.66,0.78,0.47,0.74,0.88,0.34,0.57,0.4,0.75,0.6,0.64,0.76,0.48]]</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[1,5],[1,5],[1,5],[1,5],[2,5],[1,5],[1,5],[2,5],[2,5],[0,5],[2,5],[2,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>[1,1,2,1,1,1,1,1,1,1]</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>[2,2,2,2,1,1,2,2,2,1]</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>[50,60,50,80,30,100,50,40,60,40]</t>
         </is>
       </c>
     </row>
@@ -784,19 +1044,37 @@
       <c r="B16" t="n">
         <v>15</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>[5, 2, 8, 6, 9, 4, 6, 7, 9, 2, 9, 7, 6, 5, 7]</t>
-        </is>
+      <c r="C16" t="n">
+        <v>5</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>[[0.1295, 0.3614, 0.1029, 0.1683, 0.3003, 0.1055, 0.2697, 0.3949, 0.3731, 0.267, 0.2004, 0.4542, 0.4908, 0.136, 0.4376], [0.1861, 0.1438, 0.2911, 0.4964, 0.4816, 0.306, 0.4442, 0.2562, 0.1881, 0.4264, 0.3126, 0.2953, 0.1509, 0.3151, 0.1508], [0.4046, 0.2604, 0.4118, 0.3032, 0.3371, 0.282, 0.1334, 0.3991, 0.29, 0.1842, 0.3144, 0.491, 0.3761, 0.3102, 0.143], [0.4522, 0.406, 0.4663, 0.313, 0.332, 0.4977, 0.2825, 0.2427, 0.1177, 0.3688, 0.4466, 0.3083, 0.2815, 0.4429, 0.226], [0.321, 0.1062, 0.319, 0.4459, 0.2486, 0.1613, 0.1783, 0.437, 0.4089, 0.2797, 0.3495, 0.2595, 0.3757, 0.3113, 0.1834], [0.2118, 0.4068, 0.3731, 0.1855, 0.1786, 0.2007, 0.3973, 0.336, 0.459, 0.1988, 0.1196, 0.3136, 0.3335, 0.2233, 0.332], [0.3094, 0.1381, 0.3978, 0.4867, 0.284, 0.2091, 0.1154, 0.3807, 0.1963, 0.3359, 0.1476, 0.2605, 0.2182, 0.4346, 0.3982], [0.2637, 0.2334, 0.4827, 0.1833, 0.345, 0.1675, 0.3506, 0.251, 0.1336, 0.1341, 0.4622, 0.3826, 0.3735, 0.2384, 0.426], [0.1744, 0.3748, 0.4323, 0.1212, 0.4377, 0.1678, 0.1682, 0.4448, 0.225, 0.1404, 0.1929, 0.1386, 0.3536, 0.4866, 0.1404], [0.2404, 0.1131, 0.3893, 0.2528, 0.1027, 0.1986, 0.3713, 0.2665, 0.3066, 0.381, 0.1766, 0.2614, 0.3776, 0.372, 0.1831]]</t>
+          <t>[2,1,3,5,10,10,5,8,2,8,5,7,5,9,9]</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>[[0, 5], [1, 5], [0, 5], [0, 5], [1, 5], [3, 5], [3, 5], [2, 5], [0, 5], [0, 5], [2, 5], [1, 5], [2, 5], [0, 5], [1, 5]]</t>
+          <t>[[0.84,0.57,0.31,0.69,0.76,0.42,0.8,0.83,0.39,0.89,0.3,0.34,0.33,0.83,0.66],[0.31,0.51,0.63,0.26,0.82,0.76,0.55,0.88,0.49,0.89,0.67,0.64,0.32,0.82,0.5],[0.31,0.21,0.59,0.57,0.7,0.82,0.26,0.71,0.33,0.8,0.77,0.58,0.7,0.42,0.53],[0.78,0.52,0.45,0.55,0.78,0.43,0.32,0.7,0.78,0.27,0.37,0.3,0.44,0.52,0.72],[0.66,0.63,0.45,0.79,0.53,0.89,0.64,0.29,0.67,0.43,0.68,0.25,0.32,0.8,0.36],[0.79,0.4,0.65,0.69,0.56,0.41,0.35,0.22,0.41,0.66,0.86,0.81,0.74,0.75,0.67],[0.38,0.84,0.67,0.59,0.28,0.51,0.52,0.81,0.58,0.47,0.88,0.28,0.5,0.23,0.72],[0.84,0.4,0.8,0.4,0.84,0.73,0.76,0.21,0.87,0.71,0.41,0.78,0.4,0.81,0.28],[0.69,0.58,0.27,0.37,0.21,0.53,0.41,0.62,0.41,0.41,0.72,0.23,0.83,0.8,0.67],[0.62,0.82,0.33,0.26,0.37,0.76,0.22,0.61,0.9,0.8,0.57,0.24,0.78,0.62,0.28]]</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>[[1,5],[1,5],[0,5],[2,5],[0,5],[1,5],[2,5],[1,5],[2,5],[1,5],[0,5],[0,5],[0,5],[2,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>[1,2,1,1,2,2,2,1,2,2]</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>[1,2,2,2,2,2,1,1,2,2]</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>[90,60,80,100,20,90,30,70,60,70]</t>
         </is>
       </c>
     </row>
@@ -807,19 +1085,37 @@
       <c r="B17" t="n">
         <v>15</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>[3, 8, 8, 6, 10, 1, 6, 7, 4, 10, 9, 5, 9, 9, 7]</t>
-        </is>
+      <c r="C17" t="n">
+        <v>5</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>[[0.1529, 0.3137, 0.4614, 0.2194, 0.1349, 0.3452, 0.4226, 0.2725, 0.2147, 0.3734, 0.1435, 0.1103, 0.2517, 0.368, 0.4262], [0.4217, 0.2555, 0.4842, 0.169, 0.3183, 0.1848, 0.3101, 0.4804, 0.2041, 0.2156, 0.4058, 0.1566, 0.4088, 0.1203, 0.3734], [0.3863, 0.2992, 0.3967, 0.3394, 0.1831, 0.4756, 0.1399, 0.3353, 0.2226, 0.3636, 0.2339, 0.2062, 0.2775, 0.3126, 0.4083], [0.2603, 0.179, 0.3456, 0.2485, 0.2936, 0.3804, 0.2024, 0.2427, 0.297, 0.179, 0.229, 0.176, 0.4739, 0.2709, 0.204], [0.4279, 0.2685, 0.148, 0.1213, 0.1875, 0.3427, 0.2108, 0.2323, 0.2999, 0.3295, 0.242, 0.381, 0.1337, 0.4321, 0.2029], [0.4885, 0.2742, 0.2792, 0.2908, 0.2954, 0.4556, 0.2884, 0.3328, 0.4023, 0.3012, 0.1452, 0.2618, 0.369, 0.1165, 0.3375], [0.4115, 0.2643, 0.3454, 0.3876, 0.1702, 0.181, 0.3739, 0.1121, 0.2359, 0.1055, 0.1899, 0.1144, 0.2468, 0.4981, 0.3325], [0.3983, 0.1523, 0.4738, 0.1689, 0.4742, 0.3283, 0.1388, 0.4152, 0.1445, 0.3272, 0.1361, 0.3618, 0.2956, 0.1503, 0.1981], [0.2668, 0.4141, 0.3334, 0.1108, 0.3114, 0.3238, 0.2329, 0.3114, 0.4727, 0.4824, 0.3485, 0.2276, 0.1174, 0.4969, 0.3334], [0.4834, 0.4833, 0.3559, 0.1725, 0.1691, 0.3637, 0.1974, 0.1972, 0.3483, 0.4023, 0.4974, 0.4009, 0.2259, 0.3068, 0.1647]]</t>
+          <t>[2,7,9,1,9,8,7,1,4,9,6,10,8,8,1]</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>[[1, 5], [3, 5], [2, 5], [2, 5], [0, 5], [2, 5], [3, 5], [0, 5], [0, 5], [0, 5], [0, 5], [2, 5], [0, 5], [2, 5], [0, 5]]</t>
+          <t>[[0.27,0.84,0.67,0.78,0.82,0.6,0.56,0.5,0.42,0.5,0.74,0.62,0.82,0.51,0.62],[0.64,0.61,0.69,0.37,0.56,0.27,0.47,0.54,0.66,0.87,0.62,0.72,0.55,0.64,0.25],[0.38,0.45,0.53,0.23,0.3,0.39,0.88,0.43,0.54,0.34,0.63,0.4,0.34,0.56,0.2],[0.21,0.35,0.23,0.28,0.44,0.76,0.6,0.56,0.41,0.85,0.48,0.26,0.63,0.28,0.44],[0.56,0.81,0.55,0.69,0.89,0.29,0.39,0.48,0.5,0.49,0.84,0.7,0.63,0.42,0.78],[0.87,0.77,0.2,0.65,0.24,0.38,0.24,0.62,0.68,0.28,0.47,0.52,0.46,0.28,0.49],[0.73,0.25,0.26,0.45,0.86,0.67,0.68,0.45,0.62,0.21,0.65,0.84,0.63,0.81,0.71],[0.28,0.83,0.25,0.57,0.3,0.21,0.5,0.41,0.54,0.6,0.23,0.29,0.59,0.44,0.71],[0.66,0.79,0.68,0.5,0.67,0.39,0.41,0.75,0.51,0.76,0.78,0.8,0.84,0.5,0.42],[0.61,0.46,0.62,0.69,0.68,0.46,0.32,0.5,0.3,0.82,0.44,0.31,0.22,0.65,0.65]]</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>[[0,5],[1,5],[2,5],[0,5],[1,5],[1,5],[2,5],[1,5],[0,5],[0,5],[2,5],[2,5],[0,5],[2,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>[2,1,2,1,1,1,2,1,1,2]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>[2,2,2,2,2,1,2,1,2,1]</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>[100,40,30,60,80,70,100,60,20,60]</t>
         </is>
       </c>
     </row>
@@ -830,19 +1126,37 @@
       <c r="B18" t="n">
         <v>15</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>[7, 5, 10, 7, 7, 9, 2, 10, 7, 9, 3, 5, 8, 7, 8]</t>
-        </is>
+      <c r="C18" t="n">
+        <v>5</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>[[0.4682, 0.2415, 0.1928, 0.3233, 0.4522, 0.102, 0.1487, 0.4198, 0.4578, 0.1591, 0.356, 0.3106, 0.1943, 0.1121, 0.2451], [0.1988, 0.3003, 0.1532, 0.3003, 0.4277, 0.2326, 0.434, 0.4035, 0.4574, 0.3887, 0.1412, 0.3818, 0.198, 0.38, 0.2572], [0.272, 0.1573, 0.1408, 0.2391, 0.325, 0.3562, 0.1249, 0.4979, 0.414, 0.2993, 0.1706, 0.4921, 0.222, 0.4086, 0.1575], [0.3526, 0.3537, 0.202, 0.3157, 0.2723, 0.482, 0.3055, 0.4887, 0.4231, 0.3611, 0.4802, 0.3012, 0.4316, 0.3127, 0.4904], [0.1154, 0.2217, 0.19, 0.3192, 0.4137, 0.4975, 0.1873, 0.3266, 0.1541, 0.3816, 0.2749, 0.4197, 0.2997, 0.4109, 0.3846], [0.4691, 0.4367, 0.1035, 0.1647, 0.1034, 0.3782, 0.3745, 0.2682, 0.2841, 0.2573, 0.3011, 0.226, 0.4867, 0.4021, 0.1606], [0.3802, 0.2627, 0.413, 0.2057, 0.3689, 0.2122, 0.391, 0.3526, 0.4256, 0.3835, 0.2811, 0.1616, 0.3539, 0.4129, 0.217], [0.394, 0.1186, 0.3241, 0.3733, 0.1193, 0.2008, 0.1498, 0.2446, 0.3668, 0.1811, 0.1213, 0.4623, 0.1727, 0.1733, 0.1245], [0.4791, 0.2231, 0.1052, 0.1108, 0.4391, 0.4128, 0.4992, 0.4003, 0.2191, 0.1815, 0.1724, 0.1227, 0.4211, 0.4998, 0.4673], [0.2596, 0.1747, 0.3865, 0.1889, 0.1474, 0.2799, 0.164, 0.3364, 0.391, 0.396, 0.4503, 0.1777, 0.2276, 0.1666, 0.4928]]</t>
+          <t>[5,10,10,8,3,8,9,8,6,6,9,9,7,8,6]</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>[[1, 5], [2, 5], [2, 5], [0, 5], [1, 5], [1, 5], [2, 5], [2, 5], [2, 5], [1, 5], [3, 5], [2, 5], [2, 5], [2, 5], [3, 5]]</t>
+          <t>[[0.44,0.25,0.49,0.42,0.67,0.62,0.46,0.35,0.89,0.52,0.68,0.3,0.54,0.22,0.55],[0.87,0.47,0.23,0.22,0.47,0.31,0.22,0.73,0.52,0.4,0.83,0.28,0.87,0.42,0.82],[0.62,0.78,0.89,0.4,0.87,0.47,0.47,0.44,0.58,0.31,0.59,0.58,0.73,0.78,0.51],[0.41,0.38,0.34,0.24,0.44,0.39,0.88,0.59,0.44,0.61,0.3,0.51,0.64,0.54,0.48],[0.9,0.82,0.64,0.6,0.63,0.34,0.48,0.23,0.53,0.58,0.36,0.87,0.84,0.71,0.57],[0.81,0.29,0.75,0.29,0.76,0.39,0.81,0.86,0.3,0.52,0.89,0.54,0.8,0.61,0.46],[0.4,0.34,0.73,0.47,0.56,0.54,0.6,0.81,0.89,0.49,0.78,0.74,0.6,0.87,0.34],[0.28,0.8,0.51,0.79,0.83,0.24,0.82,0.51,0.56,0.64,0.85,0.21,0.53,0.68,0.71],[0.68,0.29,0.41,0.45,0.76,0.4,0.35,0.87,0.21,0.9,0.67,0.78,0.41,0.21,0.72],[0.78,0.72,0.3,0.73,0.74,0.66,0.74,0.79,0.63,0.26,0.54,0.25,0.49,0.48,0.25]]</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[0,5],[2,5],[1,5],[0,5],[1,5],[0,5],[1,5],[2,5],[1,5],[2,5],[1,5],[1,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>[1,2,1,1,2,1,2,1,2,1]</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>[1,2,1,1,2,2,2,2,1,2]</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>[100,80,70,90,100,20,30,50,60,50]</t>
         </is>
       </c>
     </row>
@@ -853,19 +1167,37 @@
       <c r="B19" t="n">
         <v>15</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>[5, 4, 6, 10, 6, 6, 8, 8, 5, 8, 8, 7, 6, 7, 3]</t>
-        </is>
+      <c r="C19" t="n">
+        <v>5</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>[[0.2739, 0.4326, 0.1166, 0.1444, 0.1104, 0.2748, 0.3244, 0.488, 0.3602, 0.3912, 0.2197, 0.4818, 0.2378, 0.3008, 0.4324], [0.1302, 0.2032, 0.328, 0.3725, 0.4844, 0.4079, 0.4819, 0.3071, 0.2744, 0.1535, 0.1257, 0.1968, 0.3248, 0.1391, 0.259], [0.1172, 0.4101, 0.2141, 0.3858, 0.4275, 0.4504, 0.1959, 0.4162, 0.4267, 0.4658, 0.2104, 0.1574, 0.249, 0.3422, 0.2148], [0.2034, 0.4046, 0.3295, 0.2341, 0.4909, 0.4498, 0.4542, 0.3575, 0.2825, 0.4902, 0.3352, 0.1496, 0.2663, 0.2682, 0.4164], [0.3984, 0.4358, 0.3408, 0.2001, 0.4938, 0.341, 0.4362, 0.1387, 0.2654, 0.2779, 0.3481, 0.4498, 0.4905, 0.241, 0.2568], [0.4718, 0.1301, 0.4089, 0.4894, 0.201, 0.2651, 0.1719, 0.4609, 0.3546, 0.1486, 0.1371, 0.3067, 0.3704, 0.4984, 0.2], [0.278, 0.45, 0.3091, 0.3852, 0.1512, 0.3878, 0.1037, 0.322, 0.2593, 0.3004, 0.4582, 0.3846, 0.4951, 0.4915, 0.3285], [0.4571, 0.444, 0.222, 0.3569, 0.4794, 0.121, 0.243, 0.2247, 0.1669, 0.1554, 0.3752, 0.1523, 0.338, 0.1755, 0.4905], [0.1016, 0.3794, 0.3425, 0.3943, 0.4588, 0.4592, 0.1529, 0.4468, 0.4369, 0.4566, 0.3552, 0.2796, 0.2741, 0.105, 0.4551], [0.2708, 0.4092, 0.311, 0.407, 0.245, 0.1172, 0.2341, 0.1273, 0.2193, 0.241, 0.2168, 0.3757, 0.3004, 0.3148, 0.1494]]</t>
+          <t>[2,7,2,2,8,3,5,1,1,6,1,5,6,6,7]</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>[[3, 5], [0, 5], [1, 5], [2, 5], [3, 5], [0, 5], [0, 5], [1, 5], [2, 5], [0, 5], [1, 5], [2, 5], [0, 5], [1, 5], [0, 5]]</t>
+          <t>[[0.44,0.28,0.77,0.86,0.25,0.87,0.57,0.41,0.25,0.55,0.76,0.69,0.24,0.25,0.48],[0.41,0.36,0.4,0.76,0.85,0.48,0.83,0.43,0.53,0.36,0.65,0.89,0.62,0.45,0.65],[0.29,0.82,0.55,0.51,0.61,0.64,0.25,0.68,0.37,0.7,0.78,0.76,0.59,0.56,0.3],[0.74,0.39,0.55,0.4,0.29,0.64,0.24,0.72,0.42,0.2,0.56,0.23,0.39,0.69,0.24],[0.79,0.2,0.37,0.72,0.42,0.27,0.45,0.39,0.79,0.42,0.75,0.82,0.5,0.84,0.46],[0.87,0.26,0.68,0.55,0.47,0.64,0.69,0.2,0.32,0.7,0.67,0.88,0.73,0.87,0.69],[0.41,0.27,0.75,0.65,0.23,0.45,0.87,0.55,0.5,0.52,0.35,0.46,0.46,0.24,0.74],[0.49,0.78,0.8,0.35,0.66,0.53,0.82,0.35,0.67,0.63,0.41,0.3,0.66,0.72,0.42],[0.65,0.48,0.7,0.34,0.82,0.4,0.46,0.24,0.28,0.56,0.39,0.78,0.21,0.47,0.44],[0.21,0.29,0.49,0.55,0.48,0.57,0.62,0.21,0.52,0.87,0.56,0.67,0.42,0.74,0.74]]</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>[[0,5],[0,5],[2,5],[1,5],[2,5],[2,5],[0,5],[0,5],[0,5],[0,5],[2,5],[1,5],[2,5],[2,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,2,2,2,1,2,2]</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,2,2,2,2,2,1]</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>[80,90,30,50,80,70,60,60,20,80]</t>
         </is>
       </c>
     </row>
@@ -876,19 +1208,37 @@
       <c r="B20" t="n">
         <v>15</v>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>[1, 2, 3, 1, 5, 4, 8, 4, 10, 5, 3, 9, 3, 8, 7]</t>
-        </is>
+      <c r="C20" t="n">
+        <v>5</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>[[0.3551, 0.1178, 0.4025, 0.3378, 0.2485, 0.3036, 0.444, 0.4314, 0.354, 0.4106, 0.4343, 0.4113, 0.3719, 0.2438, 0.2714], [0.4667, 0.2857, 0.3759, 0.366, 0.193, 0.2041, 0.1504, 0.4, 0.3017, 0.4064, 0.2764, 0.3765, 0.1576, 0.4162, 0.2093], [0.3756, 0.377, 0.162, 0.2316, 0.4961, 0.378, 0.1866, 0.3962, 0.3556, 0.3827, 0.3865, 0.4393, 0.2887, 0.3261, 0.116], [0.2601, 0.1663, 0.4121, 0.1917, 0.2922, 0.4659, 0.2787, 0.4366, 0.1575, 0.1217, 0.4453, 0.3289, 0.1426, 0.2463, 0.2749], [0.4511, 0.1347, 0.2702, 0.1835, 0.19, 0.4598, 0.2228, 0.3344, 0.1188, 0.4721, 0.1225, 0.144, 0.1319, 0.1232, 0.1117], [0.2344, 0.2459, 0.1463, 0.2644, 0.2631, 0.3535, 0.153, 0.1985, 0.2273, 0.1208, 0.4596, 0.249, 0.3978, 0.2947, 0.4224], [0.2323, 0.2368, 0.1374, 0.1472, 0.4006, 0.3071, 0.3508, 0.3167, 0.4098, 0.274, 0.2464, 0.2826, 0.4985, 0.444, 0.3772], [0.3641, 0.4527, 0.4606, 0.2149, 0.1174, 0.312, 0.144, 0.1101, 0.3146, 0.2029, 0.1531, 0.245, 0.4493, 0.3386, 0.4212], [0.4485, 0.3965, 0.2663, 0.1917, 0.3105, 0.3067, 0.3472, 0.1408, 0.2273, 0.1303, 0.1905, 0.1257, 0.3256, 0.4985, 0.3778], [0.1148, 0.2993, 0.4856, 0.3769, 0.4369, 0.4602, 0.4312, 0.4214, 0.3307, 0.4495, 0.1948, 0.2109, 0.3241, 0.3787, 0.2714]]</t>
+          <t>[5,1,10,1,10,8,5,4,10,6,4,4,10,5,3]</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>[[3, 5], [0, 5], [2, 5], [2, 5], [2, 5], [0, 5], [2, 5], [1, 5], [3, 5], [1, 5], [1, 5], [0, 5], [3, 5], [0, 5], [2, 5]]</t>
+          <t>[[0.56,0.88,0.29,0.21,0.74,0.77,0.28,0.39,0.21,0.41,0.74,0.56,0.44,0.46,0.2],[0.41,0.65,0.88,0.79,0.22,0.83,0.75,0.75,0.52,0.48,0.41,0.25,0.36,0.37,0.54],[0.72,0.53,0.24,0.87,0.86,0.75,0.89,0.58,0.87,0.25,0.46,0.36,0.34,0.3,0.64],[0.75,0.6,0.3,0.77,0.65,0.47,0.67,0.38,0.44,0.84,0.4,0.53,0.82,0.7,0.24],[0.3,0.21,0.64,0.51,0.29,0.87,0.57,0.37,0.55,0.68,0.25,0.39,0.76,0.52,0.58],[0.5,0.23,0.32,0.51,0.35,0.23,0.79,0.89,0.76,0.8,0.37,0.87,0.34,0.87,0.9],[0.7,0.89,0.6,0.38,0.51,0.62,0.25,0.64,0.89,0.33,0.75,0.84,0.86,0.87,0.57],[0.88,0.73,0.31,0.53,0.7,0.37,0.65,0.67,0.31,0.6,0.74,0.55,0.21,0.21,0.45],[0.85,0.36,0.64,0.36,0.43,0.79,0.71,0.27,0.5,0.22,0.54,0.66,0.28,0.4,0.48],[0.84,0.9,0.23,0.73,0.46,0.47,0.73,0.84,0.87,0.6,0.45,0.75,0.38,0.59,0.45]]</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>[[2,5],[0,5],[2,5],[2,5],[0,5],[1,5],[1,5],[0,5],[2,5],[1,5],[2,5],[0,5],[0,5],[1,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>[2,1,1,1,2,2,1,2,2,2]</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>[2,1,2,1,1,1,2,2,1,2]</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>[20,60,100,30,90,70,60,80,70,30]</t>
         </is>
       </c>
     </row>
@@ -899,19 +1249,37 @@
       <c r="B21" t="n">
         <v>15</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>[9, 10, 4, 5, 6, 6, 10, 9, 2, 6, 10, 2, 3, 7, 2]</t>
-        </is>
+      <c r="C21" t="n">
+        <v>5</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>[[0.3483, 0.4892, 0.2317, 0.3143, 0.4967, 0.4434, 0.4115, 0.4271, 0.4739, 0.1582, 0.3094, 0.1436, 0.129, 0.3879, 0.1086], [0.211, 0.4626, 0.4544, 0.1477, 0.3035, 0.3124, 0.2298, 0.265, 0.2614, 0.21, 0.1682, 0.3762, 0.4568, 0.2205, 0.2659], [0.2703, 0.3283, 0.4541, 0.1477, 0.4256, 0.2341, 0.4508, 0.1251, 0.3326, 0.2768, 0.1697, 0.3785, 0.2877, 0.3637, 0.3772], [0.1527, 0.2498, 0.2484, 0.4031, 0.4264, 0.3666, 0.1422, 0.1822, 0.449, 0.1568, 0.467, 0.2176, 0.2093, 0.2382, 0.1311], [0.1756, 0.1209, 0.316, 0.1028, 0.2588, 0.4369, 0.1242, 0.4641, 0.3814, 0.4522, 0.4955, 0.1467, 0.3027, 0.296, 0.2007], [0.2806, 0.3234, 0.1735, 0.4143, 0.199, 0.3017, 0.329, 0.3482, 0.4225, 0.3906, 0.2661, 0.2906, 0.4431, 0.4267, 0.3603], [0.204, 0.4118, 0.1035, 0.4397, 0.3494, 0.1972, 0.3047, 0.183, 0.1117, 0.128, 0.3838, 0.3813, 0.2501, 0.4461, 0.4237], [0.3889, 0.1666, 0.378, 0.3321, 0.2829, 0.2953, 0.2305, 0.1156, 0.43, 0.4871, 0.3544, 0.4811, 0.4428, 0.167, 0.4176], [0.3981, 0.3115, 0.3024, 0.2198, 0.3116, 0.2987, 0.3618, 0.3832, 0.2906, 0.1048, 0.2392, 0.2051, 0.3092, 0.3056, 0.1734], [0.1779, 0.3343, 0.4383, 0.4241, 0.3272, 0.4117, 0.479, 0.2015, 0.4351, 0.4593, 0.3096, 0.2036, 0.1513, 0.268, 0.135]]</t>
+          <t>[4,8,1,10,9,6,10,4,2,8,5,7,2,3,1]</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>[[0, 5], [2, 5], [0, 5], [1, 5], [2, 5], [0, 5], [2, 5], [3, 5], [1, 5], [1, 5], [2, 5], [3, 5], [3, 5], [1, 5], [2, 5]]</t>
+          <t>[[0.66,0.37,0.33,0.84,0.27,0.55,0.35,0.23,0.23,0.32,0.81,0.4,0.87,0.61,0.51],[0.61,0.56,0.73,0.4,0.45,0.83,0.86,0.82,0.49,0.75,0.53,0.55,0.34,0.61,0.33],[0.43,0.8,0.34,0.25,0.25,0.86,0.55,0.49,0.77,0.79,0.43,0.69,0.74,0.66,0.31],[0.81,0.58,0.4,0.5,0.23,0.29,0.74,0.2,0.49,0.57,0.24,0.88,0.36,0.41,0.41],[0.36,0.2,0.71,0.88,0.36,0.66,0.72,0.79,0.5,0.41,0.43,0.7,0.77,0.33,0.46],[0.83,0.76,0.89,0.73,0.48,0.61,0.66,0.25,0.58,0.7,0.32,0.75,0.61,0.87,0.23],[0.39,0.62,0.41,0.7,0.73,0.27,0.56,0.56,0.46,0.85,0.78,0.69,0.7,0.52,0.84],[0.69,0.71,0.8,0.39,0.76,0.34,0.44,0.43,0.88,0.8,0.69,0.71,0.59,0.86,0.55],[0.47,0.31,0.75,0.71,0.47,0.22,0.79,0.21,0.69,0.88,0.51,0.36,0.69,0.77,0.58],[0.88,0.24,0.55,0.7,0.8,0.33,0.76,0.59,0.48,0.29,0.81,0.31,0.42,0.4,0.81]]</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>[[0,5],[1,5],[1,5],[0,5],[0,5],[0,5],[2,5],[0,5],[1,5],[1,5],[1,5],[2,5],[2,5],[2,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>[2,1,2,1,2,2,2,1,2,1]</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>[2,2,1,2,1,2,2,1,2,2]</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>[50,30,90,30,50,20,20,70,50,40]</t>
         </is>
       </c>
     </row>
@@ -922,19 +1290,37 @@
       <c r="B22" t="n">
         <v>15</v>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>[7, 5, 1, 4, 10, 2, 9, 9, 2, 1, 2, 3, 2, 6, 8]</t>
-        </is>
+      <c r="C22" t="n">
+        <v>5</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>[[0.3782, 0.463, 0.2448, 0.4319, 0.4218, 0.2807, 0.4284, 0.3073, 0.318, 0.2916, 0.2068, 0.193, 0.4223, 0.1372, 0.4485], [0.3994, 0.3738, 0.2322, 0.4574, 0.3471, 0.1569, 0.1753, 0.3552, 0.2082, 0.4381, 0.1779, 0.4358, 0.4866, 0.2942, 0.4643], [0.1245, 0.3369, 0.3986, 0.2532, 0.2642, 0.1815, 0.3917, 0.448, 0.2134, 0.4589, 0.1638, 0.462, 0.4662, 0.3686, 0.3849], [0.2645, 0.1808, 0.2183, 0.1735, 0.3379, 0.3433, 0.1022, 0.384, 0.3057, 0.3648, 0.1141, 0.163, 0.3647, 0.3491, 0.4598], [0.1339, 0.4288, 0.4097, 0.1518, 0.2481, 0.2765, 0.316, 0.1771, 0.2127, 0.1357, 0.1761, 0.26, 0.3459, 0.183, 0.4489], [0.303, 0.4594, 0.2394, 0.2659, 0.2585, 0.2295, 0.3779, 0.1636, 0.393, 0.4267, 0.3276, 0.2855, 0.4062, 0.1059, 0.4972], [0.4204, 0.1087, 0.4467, 0.2675, 0.4424, 0.2801, 0.1886, 0.3092, 0.1745, 0.1518, 0.48, 0.1245, 0.4878, 0.3013, 0.2888], [0.3941, 0.1546, 0.1996, 0.1681, 0.1044, 0.3412, 0.19, 0.4848, 0.2017, 0.2159, 0.1029, 0.248, 0.2586, 0.2439, 0.3884], [0.2336, 0.2648, 0.4209, 0.124, 0.1075, 0.1936, 0.1708, 0.1363, 0.1696, 0.3438, 0.3637, 0.2724, 0.2291, 0.1692, 0.4159], [0.4245, 0.2482, 0.1198, 0.3232, 0.2873, 0.4445, 0.4426, 0.42, 0.2019, 0.4357, 0.3575, 0.3242, 0.4278, 0.4318, 0.438]]</t>
+          <t>[10,4,2,9,4,10,4,4,6,3,10,1,5,3,3]</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>[[1, 5], [1, 5], [0, 5], [2, 5], [0, 5], [1, 5], [3, 5], [3, 5], [3, 5], [2, 5], [1, 5], [3, 5], [2, 5], [0, 5], [2, 5]]</t>
+          <t>[[0.67,0.76,0.38,0.64,0.6,0.78,0.83,0.21,0.67,0.24,0.58,0.4,0.41,0.45,0.63],[0.43,0.71,0.48,0.25,0.75,0.4,0.5,0.68,0.43,0.24,0.46,0.86,0.65,0.67,0.64],[0.34,0.49,0.73,0.27,0.39,0.39,0.5,0.89,0.25,0.56,0.33,0.88,0.28,0.48,0.72],[0.69,0.5,0.44,0.48,0.38,0.34,0.54,0.39,0.4,0.66,0.88,0.62,0.25,0.25,0.87],[0.41,0.26,0.62,0.64,0.65,0.39,0.21,0.88,0.38,0.67,0.69,0.63,0.42,0.39,0.62],[0.81,0.86,0.27,0.31,0.86,0.72,0.82,0.34,0.61,0.69,0.68,0.49,0.21,0.61,0.38],[0.52,0.87,0.48,0.79,0.33,0.67,0.88,0.27,0.21,0.5,0.26,0.72,0.84,0.5,0.38],[0.5,0.71,0.21,0.61,0.63,0.65,0.37,0.7,0.26,0.34,0.81,0.72,0.21,0.37,0.35],[0.39,0.37,0.24,0.52,0.71,0.62,0.67,0.26,0.87,0.79,0.76,0.78,0.85,0.58,0.34],[0.63,0.72,0.72,0.57,0.25,0.46,0.84,0.61,0.58,0.39,0.46,0.83,0.67,0.75,0.52]]</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>[[2,5],[1,5],[0,5],[0,5],[2,5],[0,5],[0,5],[0,5],[1,5],[0,5],[2,5],[1,5],[0,5],[0,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>[1,1,2,1,1,2,2,2,1,2]</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,1,1,2,2,2,1]</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>[90,90,30,30,70,40,30,40,60,100]</t>
         </is>
       </c>
     </row>
@@ -945,19 +1331,37 @@
       <c r="B23" t="n">
         <v>15</v>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>[5, 7, 8, 7, 5, 9, 3, 10, 1, 10, 4, 8, 7, 4, 8]</t>
-        </is>
+      <c r="C23" t="n">
+        <v>5</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>[[0.4762, 0.1656, 0.2664, 0.2509, 0.2601, 0.2794, 0.4395, 0.1939, 0.224, 0.4633, 0.2244, 0.4719, 0.3836, 0.4366, 0.1215], [0.1445, 0.3356, 0.2397, 0.2845, 0.2513, 0.1628, 0.2411, 0.3773, 0.4809, 0.4409, 0.3655, 0.4434, 0.4087, 0.4357, 0.1233], [0.2049, 0.1296, 0.1391, 0.4046, 0.4318, 0.4788, 0.4727, 0.3325, 0.2559, 0.1226, 0.3118, 0.2008, 0.4296, 0.414, 0.1752], [0.3414, 0.3059, 0.3655, 0.2691, 0.3024, 0.1255, 0.3477, 0.3433, 0.2876, 0.1944, 0.4536, 0.4066, 0.3278, 0.4621, 0.2129], [0.1803, 0.3699, 0.1435, 0.2265, 0.2453, 0.2885, 0.3539, 0.2742, 0.4387, 0.1275, 0.1531, 0.374, 0.3018, 0.4157, 0.1821], [0.4415, 0.4966, 0.4985, 0.3925, 0.2, 0.4746, 0.2773, 0.1837, 0.2504, 0.1654, 0.4119, 0.3007, 0.136, 0.3607, 0.2068], [0.2481, 0.4665, 0.1822, 0.4894, 0.2576, 0.4026, 0.4944, 0.2964, 0.2855, 0.3238, 0.3987, 0.4288, 0.2899, 0.3414, 0.3749], [0.257, 0.202, 0.3051, 0.2857, 0.2175, 0.1499, 0.1477, 0.4162, 0.2326, 0.4935, 0.4813, 0.1036, 0.3219, 0.1711, 0.3254], [0.2808, 0.4614, 0.2871, 0.1128, 0.1754, 0.4059, 0.2772, 0.3366, 0.1436, 0.4674, 0.4533, 0.1062, 0.3326, 0.2327, 0.4279], [0.359, 0.1594, 0.3889, 0.4511, 0.1262, 0.1434, 0.103, 0.2916, 0.3909, 0.4388, 0.3825, 0.3844, 0.2199, 0.446, 0.4499]]</t>
+          <t>[6,7,10,9,5,8,9,10,7,2,2,9,4,7,8]</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>[[0, 5], [3, 5], [2, 5], [0, 5], [1, 5], [0, 5], [3, 5], [3, 5], [2, 5], [0, 5], [0, 5], [1, 5], [0, 5], [2, 5], [3, 5]]</t>
+          <t>[[0.64,0.37,0.69,0.5,0.51,0.65,0.86,0.24,0.78,0.4,0.51,0.22,0.41,0.55,0.24],[0.54,0.85,0.27,0.74,0.49,0.66,0.38,0.31,0.31,0.25,0.33,0.66,0.82,0.77,0.68],[0.28,0.4,0.42,0.37,0.56,0.57,0.45,0.45,0.78,0.75,0.42,0.84,0.87,0.43,0.45],[0.55,0.86,0.81,0.27,0.47,0.59,0.55,0.34,0.8,0.67,0.79,0.8,0.72,0.51,0.63],[0.31,0.67,0.33,0.69,0.36,0.28,0.32,0.2,0.7,0.71,0.56,0.31,0.26,0.21,0.32],[0.82,0.37,0.45,0.27,0.36,0.56,0.63,0.37,0.24,0.47,0.36,0.35,0.87,0.63,0.59],[0.49,0.5,0.58,0.69,0.69,0.32,0.55,0.49,0.81,0.64,0.57,0.28,0.62,0.28,0.44],[0.3,0.68,0.34,0.47,0.83,0.34,0.56,0.49,0.21,0.75,0.25,0.53,0.59,0.64,0.68],[0.38,0.21,0.71,0.57,0.79,0.77,0.79,0.54,0.43,0.75,0.52,0.33,0.8,0.82,0.53],[0.25,0.47,0.76,0.83,0.34,0.25,0.81,0.47,0.58,0.88,0.25,0.65,0.25,0.46,0.76]]</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>[[0,5],[1,5],[1,5],[1,5],[1,5],[1,5],[2,5],[0,5],[1,5],[1,5],[1,5],[2,5],[1,5],[1,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>[2,1,1,1,1,2,1,2,1,1]</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>[2,1,2,2,2,1,2,2,2,1]</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>[100,50,40,90,50,30,70,100,70,30]</t>
         </is>
       </c>
     </row>
@@ -968,19 +1372,37 @@
       <c r="B24" t="n">
         <v>15</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>[9, 7, 4, 5, 8, 1, 3, 8, 3, 1, 8, 8, 2, 4, 2]</t>
-        </is>
+      <c r="C24" t="n">
+        <v>5</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>[[0.1419, 0.4489, 0.4857, 0.4866, 0.443, 0.2793, 0.2732, 0.4353, 0.284, 0.2554, 0.3145, 0.372, 0.3012, 0.1235, 0.2911], [0.1392, 0.4016, 0.2599, 0.2013, 0.1063, 0.1916, 0.3103, 0.1282, 0.1601, 0.4754, 0.1895, 0.3685, 0.4898, 0.3746, 0.4965], [0.3554, 0.2095, 0.1692, 0.4992, 0.2308, 0.2393, 0.2521, 0.2378, 0.492, 0.1849, 0.1424, 0.4512, 0.3768, 0.305, 0.2255], [0.1977, 0.2029, 0.3928, 0.192, 0.2243, 0.4198, 0.1316, 0.4818, 0.2358, 0.2153, 0.1906, 0.3253, 0.4983, 0.3647, 0.239], [0.4898, 0.2271, 0.4368, 0.4395, 0.2009, 0.405, 0.2243, 0.2355, 0.1295, 0.1441, 0.4299, 0.2914, 0.2551, 0.4692, 0.2182], [0.2304, 0.3651, 0.2485, 0.368, 0.3657, 0.3657, 0.4799, 0.3797, 0.3957, 0.1873, 0.3382, 0.2204, 0.3374, 0.3858, 0.1382], [0.442, 0.1066, 0.2625, 0.1429, 0.4631, 0.1039, 0.1722, 0.4824, 0.3473, 0.1261, 0.3772, 0.3602, 0.2838, 0.2673, 0.4765], [0.1213, 0.3292, 0.1052, 0.1436, 0.1494, 0.3294, 0.1559, 0.2737, 0.1666, 0.3703, 0.136, 0.2102, 0.4292, 0.2264, 0.4606], [0.3472, 0.3034, 0.4262, 0.1343, 0.4027, 0.1499, 0.4678, 0.1164, 0.2935, 0.1109, 0.4635, 0.2684, 0.1842, 0.1385, 0.4166], [0.1677, 0.2715, 0.2268, 0.4686, 0.4443, 0.2676, 0.3098, 0.4568, 0.3718, 0.305, 0.1628, 0.2903, 0.1836, 0.2702, 0.3368]]</t>
+          <t>[5,10,4,7,9,10,10,9,1,10,5,1,3,5,5]</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>[[2, 5], [3, 5], [2, 5], [0, 5], [2, 5], [0, 5], [3, 5], [2, 5], [1, 5], [2, 5], [0, 5], [1, 5], [2, 5], [2, 5], [1, 5]]</t>
+          <t>[[0.5,0.9,0.59,0.42,0.35,0.45,0.46,0.25,0.46,0.52,0.71,0.66,0.7,0.21,0.35],[0.66,0.54,0.2,0.76,0.74,0.58,0.25,0.74,0.61,0.75,0.73,0.76,0.56,0.3,0.67],[0.63,0.72,0.32,0.34,0.82,0.72,0.84,0.73,0.62,0.66,0.82,0.61,0.64,0.31,0.53],[0.7,0.39,0.34,0.42,0.37,0.35,0.5,0.84,0.55,0.33,0.25,0.69,0.47,0.78,0.66],[0.76,0.39,0.68,0.38,0.86,0.65,0.43,0.39,0.33,0.69,0.35,0.62,0.39,0.66,0.77],[0.74,0.73,0.33,0.26,0.69,0.46,0.5,0.22,0.38,0.22,0.82,0.37,0.59,0.23,0.67],[0.43,0.83,0.82,0.43,0.83,0.9,0.78,0.79,0.37,0.6,0.25,0.27,0.9,0.43,0.72],[0.76,0.8,0.9,0.37,0.23,0.49,0.29,0.22,0.45,0.75,0.6,0.42,0.66,0.36,0.21],[0.74,0.64,0.73,0.23,0.79,0.63,0.59,0.64,0.81,0.61,0.61,0.89,0.73,0.51,0.7],[0.47,0.36,0.62,0.85,0.85,0.44,0.57,0.35,0.9,0.89,0.65,0.76,0.7,0.62,0.24]]</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>[[1,5],[1,5],[0,5],[0,5],[0,5],[2,5],[2,5],[1,5],[0,5],[0,5],[2,5],[2,5],[0,5],[0,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>[1,2,2,2,2,1,2,2,2,1]</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>[1,1,1,1,1,2,2,2,2,2]</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>[80,60,50,100,30,70,80,30,60,90]</t>
         </is>
       </c>
     </row>
@@ -991,19 +1413,37 @@
       <c r="B25" t="n">
         <v>15</v>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>[7, 10, 6, 9, 8, 2, 7, 9, 5, 5, 8, 5, 4, 7, 10]</t>
-        </is>
+      <c r="C25" t="n">
+        <v>5</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>[[0.1791, 0.353, 0.1136, 0.414, 0.4489, 0.236, 0.4834, 0.3464, 0.2229, 0.2057, 0.1427, 0.2215, 0.3171, 0.2704, 0.4751], [0.2414, 0.2471, 0.2875, 0.2721, 0.4656, 0.452, 0.3778, 0.2599, 0.4201, 0.4138, 0.3672, 0.4956, 0.4264, 0.4542, 0.1996], [0.3999, 0.1984, 0.43, 0.359, 0.2285, 0.4995, 0.3714, 0.2381, 0.1375, 0.2057, 0.4251, 0.4534, 0.4406, 0.3252, 0.358], [0.4745, 0.3049, 0.1603, 0.4186, 0.4014, 0.1153, 0.2755, 0.2949, 0.3851, 0.1666, 0.1827, 0.1785, 0.4421, 0.4243, 0.2089], [0.161, 0.2601, 0.2997, 0.115, 0.4116, 0.3675, 0.2188, 0.3192, 0.37, 0.3639, 0.3822, 0.2309, 0.3187, 0.3716, 0.292], [0.1578, 0.1878, 0.3429, 0.1918, 0.1668, 0.2308, 0.3706, 0.2607, 0.1087, 0.4573, 0.3516, 0.1254, 0.1559, 0.4835, 0.3131], [0.2522, 0.1122, 0.2165, 0.3306, 0.4376, 0.4853, 0.2825, 0.4799, 0.378, 0.3622, 0.3177, 0.1358, 0.1035, 0.474, 0.3283], [0.3662, 0.2816, 0.4154, 0.3486, 0.1687, 0.488, 0.169, 0.127, 0.3835, 0.4399, 0.4875, 0.4794, 0.4906, 0.1521, 0.3241], [0.2956, 0.3693, 0.1795, 0.4724, 0.1467, 0.2212, 0.1669, 0.3327, 0.1912, 0.4227, 0.2095, 0.4503, 0.3964, 0.4354, 0.3623], [0.1031, 0.2166, 0.3503, 0.3061, 0.4665, 0.1708, 0.104, 0.4666, 0.4012, 0.1412, 0.1683, 0.1061, 0.4291, 0.1459, 0.1229]]</t>
+          <t>[9,5,1,4,7,10,1,1,4,5,4,3,5,5,6]</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>[[2, 5], [3, 5], [2, 5], [0, 5], [1, 5], [1, 5], [0, 5], [0, 5], [1, 5], [1, 5], [1, 5], [0, 5], [1, 5], [2, 5], [3, 5]]</t>
+          <t>[[0.52,0.67,0.67,0.46,0.86,0.32,0.55,0.68,0.69,0.65,0.39,0.31,0.65,0.62,0.33],[0.69,0.52,0.67,0.79,0.32,0.21,0.75,0.63,0.69,0.79,0.76,0.87,0.58,0.54,0.48],[0.31,0.6,0.39,0.84,0.61,0.61,0.45,0.24,0.22,0.5,0.26,0.62,0.82,0.82,0.66],[0.35,0.8,0.82,0.34,0.72,0.4,0.76,0.9,0.22,0.83,0.64,0.88,0.53,0.79,0.24],[0.43,0.25,0.88,0.77,0.8,0.86,0.26,0.47,0.25,0.35,0.36,0.53,0.39,0.27,0.32],[0.3,0.88,0.73,0.88,0.51,0.39,0.76,0.43,0.41,0.36,0.29,0.38,0.45,0.67,0.24],[0.35,0.77,0.3,0.44,0.81,0.31,0.26,0.54,0.41,0.59,0.76,0.3,0.61,0.55,0.3],[0.64,0.39,0.54,0.26,0.52,0.41,0.78,0.24,0.49,0.52,0.71,0.6,0.67,0.74,0.8],[0.42,0.58,0.79,0.89,0.82,0.46,0.34,0.54,0.72,0.54,0.54,0.79,0.45,0.8,0.48],[0.43,0.52,0.73,0.29,0.34,0.87,0.32,0.6,0.61,0.54,0.65,0.36,0.59,0.46,0.66]]</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>[[0,5],[0,5],[1,5],[2,5],[1,5],[0,5],[0,5],[1,5],[2,5],[2,5],[0,5],[2,5],[2,5],[2,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>[1,2,1,2,1,2,1,2,2,2]</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>[2,2,1,2,1,2,1,2,2,1]</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>[80,30,50,80,80,100,30,80,60,70]</t>
         </is>
       </c>
     </row>
@@ -1014,19 +1454,37 @@
       <c r="B26" t="n">
         <v>15</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>[1, 1, 8, 3, 1, 7, 2, 9, 7, 7, 9, 4, 4, 10, 1]</t>
-        </is>
+      <c r="C26" t="n">
+        <v>5</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>[[0.3272, 0.1482, 0.1794, 0.4378, 0.2163, 0.3873, 0.1424, 0.3648, 0.1012, 0.251, 0.1205, 0.2244, 0.2257, 0.2592, 0.3974], [0.1042, 0.4076, 0.114, 0.4826, 0.3532, 0.4281, 0.4366, 0.1998, 0.4713, 0.4512, 0.4257, 0.4713, 0.1338, 0.1773, 0.289], [0.3937, 0.1364, 0.4697, 0.3167, 0.1873, 0.3907, 0.3923, 0.2948, 0.3074, 0.3668, 0.1558, 0.2823, 0.4546, 0.4841, 0.2475], [0.4755, 0.4457, 0.3171, 0.3627, 0.1749, 0.2054, 0.3193, 0.4894, 0.4227, 0.2744, 0.394, 0.4394, 0.4259, 0.3016, 0.3467], [0.2676, 0.2272, 0.1445, 0.248, 0.4773, 0.3722, 0.1467, 0.2039, 0.2202, 0.4296, 0.1498, 0.2914, 0.136, 0.2216, 0.3893], [0.2625, 0.3933, 0.4283, 0.3435, 0.2833, 0.2074, 0.1141, 0.1883, 0.4235, 0.3602, 0.2101, 0.3713, 0.3428, 0.4656, 0.1719], [0.4654, 0.3626, 0.4288, 0.397, 0.3706, 0.2575, 0.2685, 0.2067, 0.1013, 0.1258, 0.2129, 0.3582, 0.1193, 0.4316, 0.2954], [0.2932, 0.4802, 0.1021, 0.4766, 0.4742, 0.1803, 0.2269, 0.29, 0.1054, 0.4105, 0.2665, 0.4802, 0.3132, 0.1882, 0.1916], [0.1862, 0.2147, 0.4972, 0.1931, 0.1203, 0.238, 0.3476, 0.1269, 0.1329, 0.2718, 0.1901, 0.1487, 0.1303, 0.3011, 0.3005], [0.1573, 0.4918, 0.2931, 0.2035, 0.3324, 0.4745, 0.2364, 0.2091, 0.2944, 0.2447, 0.1492, 0.1356, 0.471, 0.2509, 0.217]]</t>
+          <t>[4,6,3,2,9,2,9,9,4,6,6,3,4,2,3]</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>[[1, 5], [2, 5], [0, 5], [3, 5], [1, 5], [3, 5], [2, 5], [3, 5], [0, 5], [2, 5], [3, 5], [2, 5], [1, 5], [0, 5], [1, 5]]</t>
+          <t>[[0.3,0.6,0.33,0.4,0.35,0.33,0.78,0.4,0.85,0.88,0.6,0.3,0.46,0.76,0.46],[0.26,0.59,0.79,0.76,0.32,0.67,0.35,0.35,0.81,0.37,0.38,0.2,0.81,0.75,0.64],[0.73,0.31,0.52,0.45,0.27,0.54,0.84,0.23,0.4,0.35,0.37,0.84,0.53,0.53,0.73],[0.31,0.54,0.5,0.62,0.9,0.74,0.48,0.78,0.32,0.22,0.34,0.44,0.56,0.63,0.84],[0.56,0.55,0.24,0.22,0.59,0.51,0.79,0.31,0.22,0.51,0.37,0.23,0.71,0.28,0.63],[0.4,0.32,0.47,0.76,0.47,0.73,0.29,0.74,0.37,0.67,0.6,0.85,0.47,0.25,0.21],[0.78,0.57,0.74,0.36,0.44,0.22,0.87,0.67,0.85,0.39,0.63,0.67,0.42,0.79,0.86],[0.82,0.72,0.39,0.4,0.87,0.21,0.7,0.69,0.64,0.89,0.42,0.44,0.26,0.51,0.38],[0.44,0.78,0.85,0.33,0.46,0.85,0.24,0.26,0.31,0.62,0.31,0.88,0.51,0.55,0.37],[0.53,0.66,0.73,0.73,0.6,0.83,0.77,0.73,0.24,0.2,0.35,0.66,0.49,0.48,0.82]]</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>[[1,5],[0,5],[0,5],[2,5],[0,5],[2,5],[0,5],[0,5],[2,5],[1,5],[1,5],[2,5],[2,5],[1,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>[2,2,1,2,1,2,2,2,2,1]</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>[2,1,2,2,2,1,1,2,2,1]</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>[30,100,80,90,100,20,90,50,70,90]</t>
         </is>
       </c>
     </row>
@@ -1037,19 +1495,37 @@
       <c r="B27" t="n">
         <v>15</v>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>[4, 4, 5, 5, 7, 5, 10, 4, 2, 6, 9, 2, 9, 8, 7]</t>
-        </is>
+      <c r="C27" t="n">
+        <v>5</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>[[0.4245, 0.4621, 0.1425, 0.3859, 0.4961, 0.1117, 0.1047, 0.3157, 0.4172, 0.4483, 0.2298, 0.2584, 0.1645, 0.4764, 0.2629], [0.1215, 0.2342, 0.2569, 0.3546, 0.4987, 0.2616, 0.2816, 0.3556, 0.4872, 0.267, 0.3654, 0.1627, 0.2607, 0.3971, 0.1383], [0.1426, 0.1953, 0.2472, 0.2294, 0.1382, 0.4959, 0.2256, 0.3911, 0.3088, 0.3088, 0.1002, 0.1868, 0.3794, 0.391, 0.2803], [0.3945, 0.2428, 0.3279, 0.457, 0.4662, 0.3644, 0.2472, 0.2287, 0.1252, 0.316, 0.2142, 0.2132, 0.3038, 0.1675, 0.1022], [0.3213, 0.2724, 0.3871, 0.1613, 0.4618, 0.448, 0.1307, 0.1392, 0.4854, 0.2145, 0.3719, 0.1533, 0.3927, 0.191, 0.4163], [0.4186, 0.3075, 0.4161, 0.157, 0.1008, 0.4662, 0.3757, 0.1548, 0.2484, 0.1636, 0.3825, 0.4031, 0.497, 0.1739, 0.4073], [0.1008, 0.3997, 0.3926, 0.3484, 0.1624, 0.3666, 0.188, 0.3914, 0.3654, 0.1721, 0.2418, 0.1347, 0.4992, 0.3224, 0.2296], [0.43, 0.4467, 0.1074, 0.2448, 0.2497, 0.3149, 0.129, 0.4436, 0.2943, 0.4949, 0.2412, 0.4264, 0.4179, 0.3806, 0.256], [0.4102, 0.402, 0.2124, 0.2331, 0.326, 0.19, 0.4537, 0.2069, 0.2802, 0.4872, 0.3982, 0.3348, 0.3855, 0.3919, 0.3587], [0.4528, 0.3905, 0.2228, 0.238, 0.227, 0.1139, 0.4389, 0.4278, 0.1742, 0.278, 0.1118, 0.2492, 0.2261, 0.281, 0.1669]]</t>
+          <t>[9,3,1,8,2,6,2,9,3,1,4,8,8,9,9]</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>[[3, 5], [3, 5], [3, 5], [2, 5], [0, 5], [0, 5], [2, 5], [2, 5], [3, 5], [0, 5], [0, 5], [1, 5], [2, 5], [3, 5], [1, 5]]</t>
+          <t>[[0.83,0.84,0.42,0.68,0.39,0.33,0.33,0.44,0.5,0.78,0.28,0.71,0.57,0.4,0.54],[0.41,0.62,0.5,0.32,0.28,0.58,0.83,0.44,0.71,0.66,0.85,0.77,0.6,0.66,0.83],[0.48,0.43,0.21,0.78,0.76,0.27,0.6,0.52,0.28,0.89,0.35,0.25,0.62,0.72,0.22],[0.66,0.57,0.27,0.32,0.6,0.41,0.86,0.77,0.89,0.38,0.88,0.5,0.44,0.24,0.24],[0.68,0.52,0.36,0.63,0.38,0.6,0.45,0.78,0.77,0.53,0.45,0.45,0.76,0.43,0.35],[0.26,0.53,0.54,0.79,0.35,0.47,0.77,0.78,0.47,0.52,0.41,0.85,0.28,0.85,0.68],[0.57,0.22,0.53,0.49,0.31,0.66,0.88,0.59,0.7,0.25,0.49,0.28,0.63,0.86,0.66],[0.25,0.45,0.59,0.48,0.78,0.77,0.63,0.46,0.38,0.27,0.45,0.49,0.67,0.66,0.25],[0.48,0.33,0.31,0.78,0.23,0.49,0.32,0.82,0.59,0.36,0.55,0.71,0.87,0.35,0.82],[0.85,0.84,0.64,0.64,0.48,0.73,0.57,0.67,0.5,0.71,0.78,0.3,0.78,0.58,0.79]]</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>[[2,5],[0,5],[1,5],[1,5],[1,5],[1,5],[1,5],[1,5],[2,5],[2,5],[0,5],[2,5],[2,5],[1,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>[2,1,2,2,2,1,2,1,1,2]</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>[2,2,1,1,2,2,2,1,1,2]</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>[100,70,20,70,60,40,50,70,90,50]</t>
         </is>
       </c>
     </row>
@@ -1060,19 +1536,37 @@
       <c r="B28" t="n">
         <v>15</v>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>[7, 3, 10, 7, 1, 10, 5, 3, 4, 8, 10, 7, 10, 3, 8]</t>
-        </is>
+      <c r="C28" t="n">
+        <v>5</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>[[0.1999, 0.4802, 0.2378, 0.2035, 0.4681, 0.2376, 0.2223, 0.4014, 0.2252, 0.3212, 0.1659, 0.4197, 0.1068, 0.4961, 0.1012], [0.2608, 0.2937, 0.4442, 0.4082, 0.3536, 0.4035, 0.4163, 0.3958, 0.2925, 0.1135, 0.1351, 0.4909, 0.2575, 0.1337, 0.2109], [0.4777, 0.4969, 0.1585, 0.3274, 0.1311, 0.1307, 0.2624, 0.2006, 0.4353, 0.3709, 0.4667, 0.4465, 0.1025, 0.1373, 0.3835], [0.4351, 0.4262, 0.4312, 0.498, 0.1463, 0.4876, 0.2968, 0.3471, 0.4783, 0.3425, 0.2964, 0.2485, 0.1409, 0.1847, 0.3105], [0.4545, 0.4138, 0.4808, 0.2471, 0.1523, 0.1914, 0.1519, 0.1828, 0.3484, 0.3514, 0.1322, 0.1733, 0.1523, 0.4691, 0.1045], [0.3829, 0.3155, 0.496, 0.3837, 0.4413, 0.2545, 0.1382, 0.1532, 0.1471, 0.124, 0.1501, 0.2133, 0.2643, 0.1955, 0.3887], [0.2827, 0.3939, 0.3101, 0.3392, 0.3879, 0.4656, 0.2278, 0.391, 0.3558, 0.3166, 0.211, 0.1364, 0.1042, 0.4772, 0.2763], [0.4489, 0.2441, 0.2511, 0.2108, 0.2511, 0.188, 0.3611, 0.2015, 0.1782, 0.2767, 0.3929, 0.2596, 0.2128, 0.4922, 0.4292], [0.1798, 0.2048, 0.3595, 0.2384, 0.3199, 0.3506, 0.3053, 0.1576, 0.3669, 0.2, 0.1035, 0.3345, 0.2181, 0.1014, 0.2663], [0.4054, 0.3944, 0.1785, 0.3221, 0.2552, 0.4306, 0.1944, 0.2153, 0.3935, 0.2098, 0.1746, 0.265, 0.4442, 0.4323, 0.3806]]</t>
+          <t>[4,3,3,2,5,2,9,9,9,1,6,10,3,10,7]</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>[[3, 5], [0, 5], [0, 5], [0, 5], [0, 5], [3, 5], [1, 5], [1, 5], [3, 5], [2, 5], [2, 5], [0, 5], [0, 5], [0, 5], [2, 5]]</t>
+          <t>[[0.5,0.47,0.84,0.38,0.79,0.54,0.56,0.42,0.6,0.43,0.23,0.39,0.2,0.88,0.88],[0.48,0.71,0.44,0.67,0.76,0.86,0.48,0.75,0.39,0.89,0.22,0.62,0.66,0.68,0.28],[0.86,0.33,0.64,0.36,0.42,0.58,0.49,0.31,0.32,0.49,0.73,0.83,0.26,0.48,0.27],[0.21,0.66,0.62,0.31,0.36,0.22,0.78,0.88,0.29,0.36,0.81,0.85,0.49,0.24,0.23],[0.6,0.48,0.22,0.61,0.21,0.75,0.41,0.23,0.61,0.48,0.88,0.58,0.39,0.7,0.39],[0.83,0.46,0.58,0.24,0.5,0.78,0.76,0.36,0.36,0.77,0.85,0.27,0.52,0.44,0.81],[0.26,0.35,0.73,0.24,0.54,0.51,0.43,0.48,0.57,0.31,0.6,0.76,0.73,0.31,0.3],[0.39,0.45,0.49,0.68,0.24,0.22,0.47,0.69,0.34,0.65,0.38,0.82,0.83,0.41,0.36],[0.49,0.37,0.67,0.78,0.67,0.78,0.48,0.31,0.72,0.45,0.67,0.39,0.26,0.89,0.31],[0.89,0.88,0.76,0.66,0.6,0.81,0.4,0.53,0.63,0.49,0.5,0.43,0.59,0.8,0.34]]</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>[[0,5],[0,5],[0,5],[2,5],[2,5],[0,5],[2,5],[1,5],[0,5],[1,5],[1,5],[2,5],[2,5],[0,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>[2,2,1,1,2,2,1,2,2,2]</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>[2,2,2,1,1,1,2,1,2,2]</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>[100,30,100,30,60,30,40,60,90,100]</t>
         </is>
       </c>
     </row>
@@ -1083,19 +1577,37 @@
       <c r="B29" t="n">
         <v>15</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>[2, 7, 1, 10, 8, 5, 2, 3, 7, 5, 7, 9, 6, 3, 5]</t>
-        </is>
+      <c r="C29" t="n">
+        <v>5</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>[[0.4836, 0.168, 0.3255, 0.4289, 0.2845, 0.2567, 0.4609, 0.4387, 0.176, 0.4957, 0.425, 0.1346, 0.1921, 0.3275, 0.49], [0.3183, 0.193, 0.2827, 0.3824, 0.4291, 0.2628, 0.4236, 0.4292, 0.4063, 0.4665, 0.3478, 0.3538, 0.2891, 0.2186, 0.3559], [0.4821, 0.3095, 0.4306, 0.2571, 0.4481, 0.3225, 0.2324, 0.4307, 0.2042, 0.2172, 0.1357, 0.2359, 0.3867, 0.2198, 0.2546], [0.2756, 0.27, 0.2663, 0.3371, 0.127, 0.2946, 0.4087, 0.1062, 0.171, 0.3087, 0.4585, 0.4942, 0.2733, 0.3734, 0.2321], [0.4898, 0.2833, 0.1813, 0.1835, 0.3329, 0.2731, 0.3894, 0.3607, 0.4656, 0.1858, 0.2466, 0.4331, 0.422, 0.2166, 0.1402], [0.4923, 0.1487, 0.4861, 0.4282, 0.3359, 0.2525, 0.336, 0.1994, 0.3131, 0.2766, 0.1243, 0.1987, 0.279, 0.4658, 0.3957], [0.2553, 0.4682, 0.4688, 0.2121, 0.1976, 0.3347, 0.4147, 0.4267, 0.3231, 0.4704, 0.2747, 0.3713, 0.2506, 0.2327, 0.3084], [0.3241, 0.4678, 0.236, 0.2105, 0.4579, 0.4479, 0.3074, 0.4931, 0.194, 0.3621, 0.3995, 0.1002, 0.3501, 0.3217, 0.3951], [0.1967, 0.4448, 0.317, 0.3524, 0.4977, 0.3953, 0.4045, 0.3769, 0.2012, 0.1022, 0.4112, 0.3888, 0.2728, 0.2447, 0.457], [0.4568, 0.166, 0.456, 0.4498, 0.4024, 0.2778, 0.1691, 0.3982, 0.3002, 0.1929, 0.1921, 0.1734, 0.3931, 0.2448, 0.4207]]</t>
+          <t>[3,7,2,4,8,6,1,7,1,7,9,6,4,7,2]</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>[[0, 5], [3, 5], [0, 5], [2, 5], [2, 5], [2, 5], [0, 5], [1, 5], [1, 5], [2, 5], [3, 5], [2, 5], [0, 5], [0, 5], [2, 5]]</t>
+          <t>[[0.85,0.68,0.78,0.59,0.75,0.21,0.77,0.23,0.82,0.89,0.41,0.35,0.74,0.38,0.81],[0.27,0.29,0.89,0.67,0.79,0.43,0.67,0.62,0.62,0.68,0.6,0.5,0.39,0.74,0.36],[0.68,0.36,0.64,0.72,0.35,0.24,0.29,0.62,0.79,0.23,0.71,0.44,0.53,0.85,0.43],[0.53,0.21,0.26,0.38,0.22,0.64,0.5,0.58,0.32,0.41,0.66,0.88,0.24,0.82,0.6],[0.59,0.55,0.25,0.26,0.62,0.44,0.84,0.48,0.3,0.7,0.41,0.57,0.69,0.83,0.75],[0.67,0.68,0.86,0.41,0.2,0.39,0.35,0.66,0.64,0.62,0.21,0.71,0.43,0.67,0.59],[0.44,0.29,0.27,0.78,0.84,0.65,0.27,0.48,0.71,0.75,0.28,0.2,0.7,0.45,0.38],[0.21,0.58,0.8,0.87,0.6,0.56,0.26,0.58,0.47,0.62,0.47,0.37,0.27,0.42,0.27],[0.32,0.89,0.51,0.57,0.81,0.9,0.61,0.77,0.43,0.41,0.48,0.67,0.68,0.42,0.29],[0.64,0.29,0.6,0.69,0.69,0.73,0.81,0.55,0.71,0.63,0.33,0.22,0.4,0.51,0.63]]</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>[[1,5],[0,5],[0,5],[1,5],[0,5],[2,5],[2,5],[1,5],[0,5],[0,5],[0,5],[1,5],[1,5],[2,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>[2,2,1,1,1,2,1,1,2,1]</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>[2,1,2,1,1,1,2,2,1,1]</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>[90,100,20,100,50,40,60,80,20,70]</t>
         </is>
       </c>
     </row>
@@ -1106,19 +1618,37 @@
       <c r="B30" t="n">
         <v>15</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>[3, 1, 9, 4, 7, 4, 9, 10, 3, 6, 7, 7, 10, 7, 5]</t>
-        </is>
+      <c r="C30" t="n">
+        <v>5</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>[[0.1978, 0.1864, 0.4522, 0.1015, 0.359, 0.3188, 0.491, 0.297, 0.1351, 0.2738, 0.2363, 0.3749, 0.2203, 0.1905, 0.4684], [0.4802, 0.2261, 0.1598, 0.1847, 0.1807, 0.4632, 0.3936, 0.1694, 0.464, 0.2226, 0.2803, 0.25, 0.1282, 0.2574, 0.2198], [0.2409, 0.4439, 0.4895, 0.472, 0.2321, 0.1453, 0.418, 0.1768, 0.3211, 0.4641, 0.2365, 0.3236, 0.3562, 0.172, 0.1449], [0.2167, 0.1018, 0.261, 0.171, 0.3771, 0.4548, 0.1448, 0.3485, 0.1842, 0.3243, 0.3281, 0.1646, 0.4516, 0.4817, 0.2452], [0.1912, 0.2825, 0.212, 0.4234, 0.2611, 0.3486, 0.4978, 0.4201, 0.3287, 0.3825, 0.2217, 0.2448, 0.3027, 0.3581, 0.2868], [0.3991, 0.2125, 0.4436, 0.2307, 0.469, 0.4628, 0.128, 0.3907, 0.3553, 0.4831, 0.2142, 0.4402, 0.4295, 0.1155, 0.4454], [0.3222, 0.4795, 0.226, 0.1098, 0.3547, 0.2103, 0.1076, 0.1691, 0.3501, 0.1396, 0.3681, 0.2663, 0.3237, 0.3369, 0.3823], [0.2493, 0.2861, 0.4212, 0.1337, 0.1621, 0.3213, 0.4251, 0.4018, 0.4377, 0.1741, 0.3052, 0.4528, 0.3854, 0.1377, 0.4185], [0.4508, 0.1115, 0.3193, 0.2031, 0.4166, 0.2011, 0.4517, 0.2468, 0.227, 0.2386, 0.3654, 0.2154, 0.2301, 0.4405, 0.1992], [0.3326, 0.3423, 0.228, 0.3345, 0.205, 0.2785, 0.377, 0.4604, 0.3448, 0.4157, 0.3778, 0.4509, 0.3727, 0.129, 0.1274]]</t>
+          <t>[4,10,7,3,2,9,6,2,9,9,9,9,9,1,7]</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>[[0, 5], [1, 5], [2, 5], [1, 5], [0, 5], [1, 5], [2, 5], [2, 5], [3, 5], [1, 5], [0, 5], [1, 5], [3, 5], [2, 5], [3, 5]]</t>
+          <t>[[0.79,0.34,0.29,0.87,0.28,0.53,0.61,0.58,0.26,0.24,0.27,0.61,0.58,0.36,0.65],[0.77,0.23,0.55,0.68,0.38,0.42,0.63,0.83,0.77,0.61,0.71,0.46,0.65,0.53,0.33],[0.69,0.59,0.45,0.84,0.21,0.42,0.24,0.74,0.69,0.43,0.67,0.48,0.73,0.52,0.49],[0.85,0.38,0.28,0.61,0.88,0.46,0.24,0.44,0.55,0.31,0.66,0.9,0.52,0.45,0.48],[0.28,0.82,0.49,0.47,0.66,0.51,0.65,0.24,0.77,0.86,0.65,0.87,0.31,0.53,0.62],[0.61,0.48,0.44,0.29,0.47,0.31,0.71,0.35,0.24,0.59,0.62,0.81,0.6,0.44,0.76],[0.58,0.26,0.6,0.84,0.48,0.41,0.3,0.31,0.5,0.62,0.26,0.86,0.73,0.61,0.78],[0.26,0.53,0.64,0.78,0.75,0.39,0.86,0.29,0.81,0.88,0.32,0.71,0.23,0.48,0.56],[0.61,0.86,0.67,0.54,0.77,0.87,0.22,0.89,0.26,0.77,0.4,0.29,0.51,0.65,0.47],[0.24,0.62,0.83,0.47,0.35,0.51,0.23,0.77,0.78,0.61,0.45,0.76,0.59,0.78,0.64]]</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>[[1,5],[0,5],[2,5],[1,5],[1,5],[1,5],[2,5],[0,5],[1,5],[0,5],[1,5],[0,5],[2,5],[2,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>[1,2,1,1,2,2,1,2,2,1]</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>[1,1,2,1,2,1,1,1,1,2]</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>[60,100,80,100,90,60,20,50,60,70]</t>
         </is>
       </c>
     </row>
@@ -1129,19 +1659,37 @@
       <c r="B31" t="n">
         <v>15</v>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>[6, 3, 1, 5, 2, 8, 10, 6, 3, 10, 4, 6, 2, 8, 4]</t>
-        </is>
+      <c r="C31" t="n">
+        <v>5</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>[[0.4984, 0.2333, 0.4206, 0.4219, 0.3462, 0.3426, 0.4444, 0.4842, 0.1031, 0.4584, 0.2607, 0.2555, 0.3891, 0.4502, 0.3489], [0.4561, 0.1955, 0.3551, 0.4421, 0.2725, 0.4809, 0.4669, 0.4932, 0.2617, 0.2215, 0.4497, 0.1373, 0.2383, 0.3628, 0.3582], [0.272, 0.4886, 0.3515, 0.161, 0.1625, 0.1612, 0.1378, 0.4685, 0.2186, 0.3443, 0.2341, 0.2943, 0.4299, 0.4796, 0.3013], [0.2859, 0.1464, 0.3842, 0.3725, 0.3459, 0.2785, 0.2507, 0.241, 0.2032, 0.1078, 0.2243, 0.1325, 0.3298, 0.3932, 0.4772], [0.1741, 0.415, 0.2141, 0.1896, 0.3949, 0.1299, 0.4859, 0.4316, 0.4767, 0.1878, 0.2977, 0.2477, 0.4048, 0.3865, 0.465], [0.1168, 0.2263, 0.2914, 0.1848, 0.4588, 0.3824, 0.3806, 0.3188, 0.2292, 0.3648, 0.371, 0.2591, 0.2342, 0.1603, 0.135], [0.4626, 0.136, 0.1332, 0.1689, 0.3626, 0.3833, 0.3478, 0.1884, 0.3306, 0.475, 0.2594, 0.4305, 0.3429, 0.404, 0.1306], [0.1058, 0.4589, 0.3565, 0.4533, 0.4671, 0.1186, 0.3651, 0.3499, 0.3021, 0.4175, 0.2674, 0.2527, 0.2951, 0.4149, 0.194], [0.1291, 0.1079, 0.1132, 0.166, 0.385, 0.169, 0.1765, 0.1096, 0.2452, 0.2506, 0.2851, 0.3629, 0.2605, 0.2628, 0.4988], [0.3463, 0.1086, 0.48, 0.3437, 0.1747, 0.4184, 0.131, 0.4008, 0.3311, 0.1378, 0.2571, 0.3912, 0.4012, 0.3886, 0.2292]]</t>
+          <t>[1,6,5,2,6,7,7,8,7,6,3,8,8,6,9]</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>[[1, 5], [3, 5], [2, 5], [3, 5], [1, 5], [3, 5], [0, 5], [0, 5], [0, 5], [1, 5], [2, 5], [0, 5], [3, 5], [3, 5], [3, 5]]</t>
+          <t>[[0.75,0.62,0.49,0.87,0.58,0.62,0.35,0.64,0.6,0.33,0.24,0.62,0.73,0.57,0.36],[0.67,0.26,0.51,0.31,0.33,0.34,0.47,0.24,0.48,0.56,0.54,0.47,0.79,0.3,0.55],[0.24,0.25,0.6,0.6,0.81,0.59,0.87,0.23,0.27,0.23,0.33,0.58,0.65,0.23,0.86],[0.79,0.41,0.25,0.32,0.29,0.29,0.56,0.37,0.45,0.89,0.68,0.86,0.3,0.47,0.59],[0.25,0.2,0.67,0.65,0.49,0.54,0.49,0.22,0.43,0.32,0.27,0.87,0.62,0.71,0.42],[0.48,0.37,0.27,0.33,0.76,0.67,0.58,0.53,0.85,0.25,0.4,0.44,0.75,0.89,0.37],[0.81,0.78,0.36,0.48,0.49,0.88,0.33,0.76,0.43,0.71,0.49,0.6,0.78,0.76,0.81],[0.24,0.68,0.3,0.49,0.58,0.48,0.56,0.9,0.29,0.67,0.48,0.29,0.31,0.86,0.82],[0.83,0.89,0.35,0.45,0.67,0.54,0.49,0.45,0.62,0.6,0.31,0.53,0.59,0.6,0.35],[0.72,0.22,0.45,0.75,0.59,0.38,0.69,0.6,0.76,0.71,0.63,0.54,0.29,0.38,0.49]]</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>[[1,5],[0,5],[2,5],[1,5],[0,5],[1,5],[2,5],[0,5],[2,5],[1,5],[1,5],[0,5],[0,5],[1,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>[2,2,2,2,1,2,2,2,1,2]</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>[2,2,1,1,2,2,1,1,1,2]</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>[20,40,30,50,70,70,80,20,40,90]</t>
         </is>
       </c>
     </row>
@@ -1152,19 +1700,37 @@
       <c r="B32" t="n">
         <v>15</v>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>[3, 6, 2, 3, 10, 6, 9, 8, 7, 2, 5, 6, 10, 5, 10]</t>
-        </is>
+      <c r="C32" t="n">
+        <v>5</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>[[0.3971, 0.1133, 0.348, 0.4426, 0.2428, 0.1375, 0.3941, 0.415, 0.2304, 0.3767, 0.214, 0.3562, 0.189, 0.2596, 0.3818], [0.4798, 0.3391, 0.3327, 0.3984, 0.2043, 0.2581, 0.1775, 0.3266, 0.1355, 0.3995, 0.1787, 0.3768, 0.2322, 0.4757, 0.4477], [0.229, 0.3216, 0.2051, 0.1593, 0.1996, 0.1872, 0.1954, 0.4577, 0.3535, 0.1052, 0.4753, 0.1587, 0.1856, 0.2074, 0.3389], [0.1914, 0.1987, 0.2461, 0.3905, 0.1357, 0.4966, 0.384, 0.2481, 0.2874, 0.4979, 0.1326, 0.3955, 0.4309, 0.3854, 0.2332], [0.4677, 0.1649, 0.2106, 0.1021, 0.4024, 0.1322, 0.2395, 0.4177, 0.3841, 0.4376, 0.2787, 0.1214, 0.4226, 0.3672, 0.3671], [0.492, 0.1351, 0.1705, 0.2032, 0.4798, 0.1409, 0.3274, 0.1746, 0.2274, 0.2776, 0.1244, 0.3855, 0.2834, 0.3473, 0.4712], [0.3654, 0.3908, 0.2143, 0.2868, 0.3684, 0.3701, 0.3032, 0.4569, 0.388, 0.4872, 0.3722, 0.2887, 0.3247, 0.4437, 0.1798], [0.136, 0.4746, 0.4639, 0.1283, 0.4087, 0.273, 0.202, 0.2995, 0.1744, 0.2824, 0.2594, 0.3524, 0.3092, 0.2981, 0.2457], [0.3445, 0.2327, 0.229, 0.1286, 0.3719, 0.1151, 0.4878, 0.3261, 0.3656, 0.277, 0.2097, 0.1404, 0.3035, 0.2302, 0.2437], [0.201, 0.2186, 0.2753, 0.2362, 0.492, 0.3398, 0.1961, 0.3874, 0.329, 0.4498, 0.1175, 0.4142, 0.2169, 0.4297, 0.2166]]</t>
+          <t>[6,6,8,2,10,3,9,6,7,6,5,4,2,1,3]</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>[[2, 5], [2, 5], [0, 5], [0, 5], [3, 5], [1, 5], [0, 5], [3, 5], [2, 5], [3, 5], [1, 5], [2, 5], [2, 5], [0, 5], [0, 5]]</t>
+          <t>[[0.62,0.56,0.4,0.2,0.55,0.4,0.71,0.22,0.61,0.86,0.32,0.53,0.26,0.64,0.59],[0.49,0.56,0.83,0.34,0.22,0.8,0.6,0.82,0.62,0.77,0.5,0.72,0.84,0.6,0.33],[0.39,0.34,0.37,0.41,0.59,0.61,0.5,0.63,0.26,0.26,0.32,0.56,0.35,0.4,0.48],[0.77,0.21,0.65,0.67,0.76,0.85,0.21,0.31,0.82,0.52,0.6,0.66,0.68,0.85,0.9],[0.7,0.4,0.82,0.23,0.36,0.83,0.38,0.35,0.3,0.8,0.55,0.67,0.37,0.73,0.73],[0.42,0.49,0.35,0.88,0.65,0.85,0.41,0.75,0.74,0.68,0.88,0.48,0.29,0.67,0.71],[0.6,0.34,0.55,0.42,0.5,0.65,0.72,0.36,0.48,0.39,0.34,0.75,0.84,0.46,0.73],[0.83,0.79,0.33,0.87,0.46,0.44,0.24,0.54,0.28,0.37,0.42,0.77,0.81,0.41,0.8],[0.8,0.74,0.3,0.68,0.86,0.68,0.43,0.55,0.65,0.56,0.28,0.42,0.76,0.8,0.3],[0.87,0.43,0.66,0.73,0.77,0.86,0.42,0.8,0.29,0.69,0.72,0.67,0.38,0.81,0.32]]</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>[[1,5],[2,5],[1,5],[2,5],[0,5],[1,5],[1,5],[2,5],[1,5],[0,5],[2,5],[1,5],[2,5],[1,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>[1,1,1,2,1,2,1,2,2,1]</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>[2,2,1,1,2,1,1,1,1,1]</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>[90,20,70,100,70,90,100,40,30,30]</t>
         </is>
       </c>
     </row>
@@ -1175,19 +1741,37 @@
       <c r="B33" t="n">
         <v>15</v>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>[5, 8, 6, 8, 8, 1, 1, 10, 8, 5, 7, 10, 7, 3, 10]</t>
-        </is>
+      <c r="C33" t="n">
+        <v>5</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>[[0.3937, 0.1708, 0.2054, 0.4069, 0.3929, 0.4801, 0.44, 0.3338, 0.2827, 0.3765, 0.1005, 0.2734, 0.4161, 0.4233, 0.201], [0.3154, 0.2829, 0.1904, 0.4361, 0.253, 0.1423, 0.3816, 0.2242, 0.2188, 0.3934, 0.13, 0.3049, 0.4882, 0.2481, 0.1469], [0.3688, 0.2782, 0.1717, 0.2943, 0.1585, 0.1967, 0.2512, 0.3747, 0.2192, 0.2379, 0.3844, 0.2152, 0.2482, 0.2106, 0.3983], [0.3861, 0.1432, 0.2919, 0.1232, 0.3489, 0.3706, 0.4791, 0.2106, 0.4179, 0.3211, 0.1899, 0.1828, 0.4506, 0.4835, 0.3466], [0.2005, 0.2708, 0.3504, 0.4585, 0.1205, 0.1702, 0.3313, 0.2066, 0.4765, 0.2314, 0.1231, 0.4226, 0.4388, 0.4828, 0.1247], [0.2712, 0.4973, 0.1977, 0.4521, 0.3133, 0.1459, 0.3922, 0.4217, 0.3534, 0.3695, 0.4486, 0.1205, 0.466, 0.223, 0.2577], [0.1816, 0.324, 0.2373, 0.2357, 0.2789, 0.1421, 0.4472, 0.2378, 0.4417, 0.3907, 0.3403, 0.238, 0.1413, 0.2429, 0.3519], [0.1555, 0.3558, 0.3005, 0.3755, 0.2853, 0.3136, 0.1028, 0.1214, 0.3748, 0.1367, 0.391, 0.4147, 0.1152, 0.4682, 0.1266], [0.1697, 0.3439, 0.4385, 0.124, 0.2055, 0.1346, 0.4773, 0.1443, 0.4172, 0.1726, 0.2332, 0.4855, 0.4959, 0.115, 0.2691], [0.4028, 0.3271, 0.2517, 0.3716, 0.2366, 0.3371, 0.2228, 0.202, 0.2418, 0.1346, 0.3181, 0.2597, 0.1311, 0.1749, 0.3624]]</t>
+          <t>[5,7,8,9,7,7,10,2,3,6,2,8,8,9,6]</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>[[3, 5], [0, 5], [0, 5], [0, 5], [1, 5], [2, 5], [0, 5], [2, 5], [0, 5], [2, 5], [3, 5], [0, 5], [1, 5], [0, 5], [3, 5]]</t>
+          <t>[[0.24,0.7,0.53,0.79,0.47,0.32,0.79,0.58,0.33,0.7,0.56,0.62,0.52,0.78,0.78],[0.7,0.27,0.79,0.67,0.69,0.45,0.82,0.71,0.28,0.49,0.82,0.23,0.87,0.68,0.64],[0.39,0.37,0.86,0.41,0.74,0.48,0.3,0.21,0.58,0.88,0.46,0.45,0.44,0.56,0.51],[0.82,0.55,0.56,0.3,0.89,0.37,0.25,0.66,0.62,0.49,0.5,0.75,0.34,0.77,0.65],[0.49,0.52,0.38,0.73,0.56,0.42,0.62,0.9,0.5,0.84,0.44,0.24,0.34,0.49,0.35],[0.2,0.84,0.79,0.72,0.32,0.28,0.25,0.71,0.85,0.5,0.28,0.56,0.44,0.46,0.63],[0.7,0.28,0.22,0.9,0.36,0.24,0.33,0.23,0.47,0.76,0.44,0.51,0.67,0.56,0.8],[0.81,0.21,0.74,0.52,0.89,0.54,0.89,0.73,0.37,0.58,0.89,0.8,0.27,0.69,0.44],[0.2,0.48,0.36,0.77,0.44,0.78,0.2,0.42,0.37,0.36,0.25,0.33,0.59,0.4,0.49],[0.46,0.81,0.83,0.55,0.43,0.27,0.87,0.24,0.41,0.41,0.42,0.32,0.75,0.29,0.64]]</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[2,5],[2,5],[0,5],[0,5],[1,5],[2,5],[0,5],[0,5],[2,5],[0,5],[1,5],[0,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>[2,1,2,2,1,2,1,2,1,2]</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>[1,1,1,1,2,1,1,1,1,2]</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>[50,80,20,90,100,60,60,90,50,80]</t>
         </is>
       </c>
     </row>
@@ -1198,19 +1782,37 @@
       <c r="B34" t="n">
         <v>15</v>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>[2, 1, 8, 10, 9, 5, 10, 7, 10, 5, 10, 5, 4, 8, 5]</t>
-        </is>
+      <c r="C34" t="n">
+        <v>5</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>[[0.4353, 0.1224, 0.293, 0.1624, 0.2025, 0.3431, 0.3985, 0.394, 0.3655, 0.4845, 0.2758, 0.2196, 0.2388, 0.2945, 0.4375], [0.3378, 0.3244, 0.4654, 0.1529, 0.3737, 0.3507, 0.4843, 0.2646, 0.4461, 0.3934, 0.2383, 0.1237, 0.2394, 0.4004, 0.2695], [0.3863, 0.1109, 0.4665, 0.4669, 0.1148, 0.3314, 0.1968, 0.4158, 0.4875, 0.1693, 0.182, 0.299, 0.3503, 0.4141, 0.4652], [0.1939, 0.2312, 0.1946, 0.3308, 0.1336, 0.243, 0.4787, 0.2706, 0.279, 0.2633, 0.1649, 0.4883, 0.429, 0.2584, 0.4532], [0.4333, 0.4687, 0.1149, 0.2891, 0.2226, 0.2684, 0.1645, 0.3033, 0.168, 0.1385, 0.2725, 0.313, 0.4682, 0.104, 0.3148], [0.201, 0.2468, 0.3348, 0.1143, 0.4257, 0.3081, 0.3582, 0.3193, 0.3761, 0.1438, 0.3905, 0.4967, 0.1685, 0.351, 0.4824], [0.1541, 0.495, 0.2648, 0.1035, 0.3921, 0.2885, 0.1419, 0.1099, 0.1414, 0.2089, 0.1464, 0.4507, 0.4844, 0.2515, 0.2513], [0.4167, 0.1949, 0.2627, 0.1626, 0.2539, 0.427, 0.1673, 0.261, 0.2375, 0.1032, 0.4338, 0.1785, 0.4611, 0.4779, 0.4099], [0.3532, 0.3732, 0.4031, 0.1088, 0.2182, 0.3587, 0.4416, 0.3608, 0.2516, 0.493, 0.3608, 0.1962, 0.1745, 0.4714, 0.4469], [0.1463, 0.1639, 0.3048, 0.2102, 0.2409, 0.1822, 0.4401, 0.1408, 0.1739, 0.1204, 0.4252, 0.2909, 0.1465, 0.1076, 0.329]]</t>
+          <t>[5,8,2,1,3,8,7,8,8,4,6,10,3,6,6]</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>[[1, 5], [0, 5], [0, 5], [1, 5], [1, 5], [2, 5], [2, 5], [3, 5], [1, 5], [2, 5], [0, 5], [1, 5], [1, 5], [2, 5], [3, 5]]</t>
+          <t>[[0.29,0.25,0.84,0.33,0.77,0.58,0.25,0.87,0.37,0.8,0.32,0.8,0.21,0.56,0.74],[0.85,0.84,0.77,0.82,0.34,0.4,0.4,0.46,0.48,0.58,0.31,0.68,0.32,0.42,0.55],[0.76,0.72,0.65,0.31,0.58,0.26,0.46,0.49,0.23,0.39,0.87,0.87,0.45,0.23,0.33],[0.47,0.86,0.3,0.73,0.28,0.89,0.47,0.74,0.44,0.64,0.33,0.3,0.86,0.84,0.82],[0.64,0.77,0.25,0.43,0.42,0.64,0.45,0.3,0.62,0.77,0.47,0.29,0.34,0.37,0.41],[0.65,0.62,0.69,0.45,0.78,0.34,0.53,0.76,0.33,0.28,0.82,0.44,0.68,0.22,0.68],[0.42,0.24,0.63,0.37,0.47,0.26,0.3,0.41,0.26,0.84,0.2,0.54,0.29,0.42,0.85],[0.31,0.88,0.34,0.72,0.58,0.82,0.59,0.57,0.34,0.32,0.84,0.43,0.46,0.73,0.44],[0.87,0.72,0.62,0.82,0.23,0.38,0.53,0.36,0.72,0.84,0.5,0.44,0.87,0.51,0.54],[0.45,0.84,0.6,0.73,0.77,0.44,0.5,0.79,0.45,0.76,0.86,0.64,0.72,0.76,0.79]]</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>[[2,5],[1,5],[1,5],[0,5],[1,5],[2,5],[2,5],[0,5],[1,5],[0,5],[1,5],[0,5],[1,5],[1,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>[1,1,1,2,2,2,1,1,2,2]</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,2,2,2,1,1,2]</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>[100,90,50,50,70,20,20,60,90,90]</t>
         </is>
       </c>
     </row>
@@ -1221,19 +1823,37 @@
       <c r="B35" t="n">
         <v>15</v>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>[2, 3, 4, 4, 2, 5, 6, 6, 5, 10, 7, 2, 9, 8, 2]</t>
-        </is>
+      <c r="C35" t="n">
+        <v>5</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>[[0.272, 0.326, 0.1311, 0.2794, 0.4093, 0.1271, 0.1084, 0.3486, 0.287, 0.1339, 0.4814, 0.168, 0.2957, 0.2019, 0.1297], [0.294, 0.38, 0.4153, 0.2881, 0.4368, 0.2334, 0.2894, 0.3872, 0.4004, 0.4464, 0.2774, 0.2929, 0.2332, 0.292, 0.246], [0.4766, 0.3507, 0.2266, 0.3416, 0.2508, 0.2343, 0.3658, 0.4264, 0.1987, 0.1802, 0.1302, 0.2358, 0.1426, 0.3856, 0.1196], [0.1063, 0.1089, 0.4261, 0.3898, 0.2039, 0.1238, 0.1682, 0.4263, 0.2758, 0.132, 0.358, 0.3353, 0.4013, 0.3691, 0.4214], [0.2932, 0.3486, 0.2664, 0.3309, 0.1435, 0.4075, 0.1877, 0.315, 0.3069, 0.2949, 0.3914, 0.4716, 0.3439, 0.1134, 0.1988], [0.4151, 0.2035, 0.2405, 0.25, 0.103, 0.1049, 0.153, 0.1895, 0.1106, 0.43, 0.4709, 0.4189, 0.1179, 0.3301, 0.2599], [0.1081, 0.2691, 0.1769, 0.4325, 0.3615, 0.3715, 0.2503, 0.2665, 0.3769, 0.2954, 0.2158, 0.361, 0.2612, 0.1594, 0.4554], [0.4665, 0.3986, 0.2726, 0.3102, 0.3455, 0.105, 0.1867, 0.3816, 0.2587, 0.4891, 0.1384, 0.3382, 0.3457, 0.4899, 0.1925], [0.3501, 0.3403, 0.4194, 0.404, 0.2242, 0.4749, 0.2233, 0.4166, 0.1314, 0.2887, 0.2202, 0.1855, 0.4638, 0.4759, 0.1852], [0.1173, 0.1679, 0.1106, 0.4619, 0.2608, 0.173, 0.2597, 0.3036, 0.1731, 0.2448, 0.4802, 0.2727, 0.1249, 0.495, 0.2248]]</t>
+          <t>[5,9,1,2,7,3,5,6,7,6,1,7,1,10,9]</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>[[1, 5], [1, 5], [0, 5], [3, 5], [3, 5], [1, 5], [0, 5], [1, 5], [2, 5], [1, 5], [0, 5], [0, 5], [0, 5], [0, 5], [2, 5]]</t>
+          <t>[[0.48,0.24,0.48,0.67,0.52,0.72,0.45,0.64,0.33,0.72,0.58,0.34,0.4,0.72,0.54],[0.35,0.88,0.7,0.87,0.5,0.53,0.83,0.57,0.7,0.38,0.51,0.29,0.34,0.2,0.23],[0.88,0.37,0.66,0.79,0.59,0.31,0.71,0.62,0.71,0.74,0.88,0.6,0.44,0.65,0.25],[0.83,0.28,0.43,0.77,0.62,0.48,0.53,0.8,0.44,0.81,0.26,0.74,0.79,0.33,0.5],[0.32,0.69,0.57,0.64,0.34,0.35,0.23,0.43,0.59,0.8,0.67,0.5,0.87,0.7,0.85],[0.57,0.38,0.24,0.71,0.28,0.41,0.57,0.6,0.62,0.32,0.47,0.63,0.88,0.71,0.85],[0.73,0.61,0.33,0.67,0.64,0.62,0.54,0.57,0.43,0.56,0.34,0.76,0.33,0.26,0.51],[0.66,0.51,0.39,0.59,0.44,0.85,0.85,0.55,0.43,0.72,0.23,0.53,0.44,0.84,0.21],[0.59,0.72,0.54,0.26,0.88,0.56,0.63,0.37,0.54,0.5,0.25,0.27,0.79,0.37,0.34],[0.55,0.74,0.24,0.6,0.28,0.23,0.24,0.78,0.28,0.23,0.51,0.79,0.38,0.5,0.23]]</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>[[0,5],[1,5],[2,5],[1,5],[0,5],[1,5],[2,5],[1,5],[2,5],[1,5],[2,5],[2,5],[2,5],[0,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>[1,2,2,2,2,1,1,2,1,1]</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,2,1,1,2,2,1]</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>[80,60,70,100,100,100,90,60,90,20]</t>
         </is>
       </c>
     </row>
@@ -1244,19 +1864,37 @@
       <c r="B36" t="n">
         <v>15</v>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>[8, 6, 8, 4, 7, 6, 5, 4, 3, 3, 3, 5, 8, 9, 4]</t>
-        </is>
+      <c r="C36" t="n">
+        <v>5</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>[[0.4529, 0.2862, 0.4702, 0.4957, 0.2875, 0.172, 0.2983, 0.1835, 0.4664, 0.4114, 0.3448, 0.2547, 0.1232, 0.1162, 0.4612], [0.4417, 0.1459, 0.4885, 0.2817, 0.2889, 0.1891, 0.2564, 0.1895, 0.3898, 0.3589, 0.387, 0.4356, 0.4133, 0.2942, 0.2668], [0.3253, 0.122, 0.4944, 0.2057, 0.3803, 0.4761, 0.4397, 0.3483, 0.4696, 0.1493, 0.312, 0.1474, 0.2493, 0.4985, 0.2792], [0.3604, 0.4093, 0.3443, 0.4048, 0.2319, 0.1304, 0.4086, 0.3119, 0.2462, 0.3498, 0.376, 0.3402, 0.4013, 0.1963, 0.4316], [0.1005, 0.3496, 0.4688, 0.4299, 0.2839, 0.2387, 0.2483, 0.3472, 0.1535, 0.2896, 0.4938, 0.3266, 0.4458, 0.3258, 0.438], [0.2039, 0.1299, 0.1494, 0.3973, 0.2796, 0.1406, 0.1534, 0.131, 0.4425, 0.1773, 0.4011, 0.4554, 0.3603, 0.4387, 0.2213], [0.1001, 0.4274, 0.2943, 0.4448, 0.1773, 0.2846, 0.106, 0.4444, 0.2806, 0.2615, 0.237, 0.2012, 0.3128, 0.1739, 0.2415], [0.4404, 0.1256, 0.1704, 0.2547, 0.2252, 0.288, 0.4419, 0.4219, 0.2649, 0.4505, 0.3523, 0.3793, 0.3903, 0.4955, 0.1627], [0.1542, 0.476, 0.3395, 0.3402, 0.2971, 0.1624, 0.3652, 0.1439, 0.1215, 0.1681, 0.1582, 0.1673, 0.4307, 0.4392, 0.3007], [0.4694, 0.1625, 0.1208, 0.4149, 0.491, 0.3291, 0.4438, 0.1282, 0.2003, 0.4877, 0.3581, 0.1191, 0.1718, 0.3847, 0.3702]]</t>
+          <t>[6,6,2,7,10,5,1,10,8,5,10,10,4,1,10]</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>[[3, 5], [0, 5], [2, 5], [1, 5], [0, 5], [1, 5], [1, 5], [2, 5], [1, 5], [3, 5], [2, 5], [3, 5], [1, 5], [3, 5], [2, 5]]</t>
+          <t>[[0.51,0.6,0.6,0.43,0.42,0.27,0.46,0.27,0.74,0.88,0.88,0.81,0.62,0.69,0.4],[0.64,0.52,0.54,0.73,0.4,0.42,0.85,0.24,0.54,0.84,0.63,0.58,0.37,0.44,0.8],[0.59,0.56,0.27,0.21,0.87,0.46,0.62,0.26,0.68,0.85,0.6,0.29,0.61,0.74,0.48],[0.82,0.65,0.83,0.64,0.29,0.42,0.34,0.84,0.73,0.67,0.41,0.33,0.73,0.53,0.36],[0.63,0.23,0.43,0.53,0.3,0.89,0.35,0.29,0.34,0.74,0.5,0.6,0.21,0.22,0.51],[0.77,0.82,0.26,0.58,0.84,0.47,0.78,0.29,0.85,0.73,0.86,0.67,0.45,0.86,0.39],[0.43,0.69,0.74,0.85,0.34,0.76,0.72,0.24,0.47,0.4,0.41,0.89,0.65,0.7,0.88],[0.46,0.76,0.5,0.81,0.33,0.86,0.35,0.43,0.73,0.48,0.63,0.51,0.72,0.36,0.24],[0.41,0.53,0.32,0.45,0.48,0.24,0.61,0.82,0.31,0.62,0.67,0.49,0.69,0.49,0.55],[0.21,0.68,0.66,0.23,0.46,0.89,0.49,0.55,0.84,0.7,0.61,0.76,0.81,0.52,0.53]]</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>[[1,5],[0,5],[2,5],[2,5],[2,5],[2,5],[1,5],[0,5],[2,5],[0,5],[0,5],[2,5],[2,5],[0,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>[1,2,2,2,1,2,1,2,2,1]</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,2,2,1,2,2,2]</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>[60,90,50,50,60,100,60,50,60,60]</t>
         </is>
       </c>
     </row>
@@ -1267,19 +1905,37 @@
       <c r="B37" t="n">
         <v>15</v>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>[9, 10, 6, 10, 6, 10, 5, 9, 1, 2, 5, 6, 3, 10, 7]</t>
-        </is>
+      <c r="C37" t="n">
+        <v>5</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>[[0.1726, 0.4033, 0.1377, 0.4803, 0.4814, 0.2973, 0.4892, 0.1639, 0.1638, 0.3585, 0.2666, 0.1606, 0.1972, 0.2722, 0.4867], [0.3034, 0.4577, 0.274, 0.4446, 0.333, 0.1581, 0.4879, 0.4692, 0.3687, 0.4458, 0.3757, 0.3282, 0.2914, 0.3345, 0.4986], [0.2336, 0.3643, 0.2962, 0.1048, 0.1052, 0.2917, 0.3073, 0.3307, 0.4344, 0.1685, 0.3152, 0.4168, 0.3377, 0.1181, 0.4371], [0.4328, 0.4764, 0.1956, 0.3872, 0.1739, 0.2452, 0.115, 0.4858, 0.3191, 0.4906, 0.216, 0.3188, 0.3075, 0.3611, 0.2701], [0.239, 0.4242, 0.2056, 0.2471, 0.4738, 0.3052, 0.2601, 0.3775, 0.1806, 0.4796, 0.2102, 0.4883, 0.3035, 0.1608, 0.3582], [0.4422, 0.4986, 0.4298, 0.4562, 0.4268, 0.3945, 0.4035, 0.3218, 0.1845, 0.2665, 0.4422, 0.1139, 0.1756, 0.2993, 0.2], [0.4888, 0.1279, 0.397, 0.1277, 0.2913, 0.4389, 0.4507, 0.1467, 0.2437, 0.4048, 0.4808, 0.4805, 0.139, 0.2771, 0.1101], [0.2178, 0.2962, 0.439, 0.4407, 0.1457, 0.2594, 0.3639, 0.2691, 0.4061, 0.3421, 0.3634, 0.4912, 0.2151, 0.4988, 0.4206], [0.2051, 0.1144, 0.2143, 0.2613, 0.2195, 0.4624, 0.2114, 0.2112, 0.2957, 0.1584, 0.3979, 0.3875, 0.4409, 0.3935, 0.3328], [0.1576, 0.2034, 0.2905, 0.4333, 0.3199, 0.1732, 0.1172, 0.27, 0.3373, 0.2513, 0.2042, 0.177, 0.3792, 0.1573, 0.2495]]</t>
+          <t>[4,8,6,8,6,9,5,5,2,10,9,7,7,6,3]</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>[[0, 5], [1, 5], [3, 5], [0, 5], [3, 5], [1, 5], [3, 5], [0, 5], [2, 5], [2, 5], [1, 5], [1, 5], [1, 5], [1, 5], [0, 5]]</t>
+          <t>[[0.47,0.88,0.69,0.26,0.8,0.54,0.25,0.58,0.49,0.81,0.34,0.78,0.59,0.24,0.88],[0.56,0.4,0.53,0.8,0.41,0.33,0.29,0.41,0.75,0.53,0.36,0.32,0.43,0.86,0.44],[0.89,0.54,0.33,0.82,0.52,0.7,0.89,0.24,0.27,0.7,0.4,0.33,0.23,0.22,0.74],[0.29,0.53,0.62,0.5,0.22,0.75,0.21,0.73,0.83,0.5,0.57,0.53,0.47,0.82,0.83],[0.44,0.63,0.85,0.87,0.56,0.52,0.4,0.87,0.3,0.61,0.4,0.4,0.48,0.9,0.24],[0.6,0.26,0.31,0.51,0.56,0.38,0.42,0.26,0.41,0.88,0.86,0.43,0.6,0.84,0.2],[0.77,0.86,0.26,0.31,0.87,0.58,0.21,0.38,0.51,0.69,0.71,0.9,0.4,0.58,0.57],[0.48,0.32,0.88,0.8,0.55,0.62,0.36,0.58,0.69,0.56,0.89,0.63,0.46,0.74,0.32],[0.47,0.44,0.5,0.75,0.54,0.76,0.6,0.44,0.77,0.37,0.36,0.55,0.38,0.21,0.65],[0.56,0.51,0.88,0.6,0.8,0.3,0.6,0.81,0.61,0.7,0.46,0.26,0.52,0.48,0.81]]</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>[[1,5],[0,5],[1,5],[2,5],[0,5],[1,5],[1,5],[2,5],[1,5],[2,5],[1,5],[0,5],[0,5],[2,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>[2,1,1,1,1,1,1,1,1,1]</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>[2,2,2,1,1,1,1,2,2,2]</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>[50,60,70,60,20,30,50,100,20,40]</t>
         </is>
       </c>
     </row>
@@ -1290,19 +1946,37 @@
       <c r="B38" t="n">
         <v>15</v>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>[8, 3, 5, 5, 6, 7, 5, 6, 1, 9, 8, 10, 3, 8, 1]</t>
-        </is>
+      <c r="C38" t="n">
+        <v>5</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>[[0.2129, 0.1008, 0.2587, 0.3751, 0.4884, 0.1891, 0.4916, 0.2451, 0.4187, 0.4011, 0.4365, 0.4045, 0.489, 0.281, 0.2379], [0.3861, 0.2951, 0.4589, 0.3712, 0.2484, 0.4583, 0.2463, 0.3492, 0.1553, 0.2335, 0.3904, 0.3723, 0.4586, 0.1272, 0.2258], [0.3012, 0.4882, 0.2093, 0.3986, 0.1023, 0.4983, 0.3247, 0.4381, 0.3896, 0.1416, 0.4569, 0.378, 0.2338, 0.2754, 0.2801], [0.1297, 0.4949, 0.2337, 0.2207, 0.3446, 0.1197, 0.1804, 0.4359, 0.4432, 0.1194, 0.2066, 0.3556, 0.1682, 0.1129, 0.2603], [0.276, 0.1853, 0.4071, 0.398, 0.4619, 0.2877, 0.3654, 0.3674, 0.2833, 0.1284, 0.4573, 0.2443, 0.4936, 0.4863, 0.1647], [0.2239, 0.2158, 0.307, 0.1124, 0.2319, 0.1681, 0.3565, 0.2147, 0.1718, 0.467, 0.2485, 0.2679, 0.2216, 0.3055, 0.1495], [0.2093, 0.215, 0.1333, 0.4452, 0.4526, 0.3307, 0.4493, 0.1816, 0.337, 0.3911, 0.3377, 0.4607, 0.1469, 0.1208, 0.1256], [0.3413, 0.4965, 0.4957, 0.3164, 0.282, 0.2452, 0.3791, 0.3814, 0.1863, 0.4101, 0.3628, 0.4917, 0.4434, 0.4352, 0.3305], [0.2819, 0.2115, 0.1275, 0.2439, 0.3718, 0.2459, 0.1905, 0.4703, 0.2449, 0.127, 0.2631, 0.132, 0.188, 0.4049, 0.4751], [0.4577, 0.4863, 0.4338, 0.1246, 0.3873, 0.3118, 0.3981, 0.3436, 0.2181, 0.3988, 0.1551, 0.1532, 0.4582, 0.2178, 0.3985]]</t>
+          <t>[7,3,1,7,8,3,5,1,1,5,10,10,2,6,5]</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>[[2, 5], [3, 5], [3, 5], [1, 5], [1, 5], [3, 5], [0, 5], [0, 5], [2, 5], [3, 5], [0, 5], [0, 5], [0, 5], [2, 5], [1, 5]]</t>
+          <t>[[0.37,0.88,0.87,0.37,0.44,0.83,0.88,0.51,0.42,0.57,0.68,0.39,0.72,0.24,0.23],[0.47,0.45,0.42,0.54,0.42,0.33,0.42,0.88,0.49,0.51,0.6,0.89,0.37,0.68,0.7],[0.63,0.26,0.67,0.24,0.62,0.72,0.35,0.79,0.22,0.79,0.52,0.35,0.29,0.87,0.25],[0.34,0.44,0.63,0.58,0.29,0.4,0.37,0.35,0.49,0.69,0.35,0.46,0.47,0.88,0.87],[0.76,0.37,0.25,0.42,0.39,0.55,0.74,0.8,0.79,0.45,0.68,0.42,0.24,0.69,0.21],[0.49,0.43,0.69,0.74,0.41,0.77,0.41,0.51,0.71,0.69,0.89,0.36,0.66,0.63,0.84],[0.31,0.73,0.6,0.39,0.53,0.43,0.61,0.82,0.6,0.64,0.56,0.24,0.36,0.54,0.42],[0.33,0.55,0.43,0.38,0.52,0.29,0.85,0.81,0.7,0.27,0.74,0.77,0.74,0.28,0.65],[0.78,0.6,0.65,0.52,0.57,0.22,0.65,0.26,0.5,0.4,0.58,0.29,0.68,0.76,0.31],[0.27,0.3,0.81,0.57,0.53,0.27,0.65,0.81,0.78,0.64,0.25,0.28,0.23,0.38,0.29]]</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>[[1,5],[2,5],[2,5],[2,5],[1,5],[0,5],[2,5],[1,5],[1,5],[0,5],[0,5],[1,5],[0,5],[2,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,2,1,1,2,2,2]</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>[1,2,1,1,1,2,2,1,1,2]</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>[80,50,90,60,70,60,20,60,70,50]</t>
         </is>
       </c>
     </row>
@@ -1313,19 +1987,37 @@
       <c r="B39" t="n">
         <v>15</v>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>[8, 10, 3, 2, 3, 10, 3, 7, 5, 1, 8, 9, 10, 6, 6]</t>
-        </is>
+      <c r="C39" t="n">
+        <v>5</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>[[0.1312, 0.1113, 0.4118, 0.4359, 0.398, 0.3134, 0.3953, 0.3088, 0.1459, 0.4791, 0.195, 0.4081, 0.3104, 0.4429, 0.25], [0.2781, 0.4839, 0.3283, 0.3066, 0.2066, 0.2408, 0.1295, 0.1964, 0.2735, 0.4066, 0.4877, 0.4215, 0.3353, 0.489, 0.2706], [0.4288, 0.3916, 0.4308, 0.4058, 0.1355, 0.1344, 0.4537, 0.4796, 0.4776, 0.2999, 0.4018, 0.4057, 0.4883, 0.3095, 0.1948], [0.4934, 0.4743, 0.2901, 0.1889, 0.1014, 0.1504, 0.1765, 0.2999, 0.3277, 0.1369, 0.4328, 0.1234, 0.3447, 0.3611, 0.1075], [0.2421, 0.2378, 0.1593, 0.1151, 0.3729, 0.2545, 0.4368, 0.436, 0.456, 0.3393, 0.4091, 0.2551, 0.2956, 0.2424, 0.11], [0.247, 0.2615, 0.15, 0.405, 0.1898, 0.4146, 0.1339, 0.1663, 0.4693, 0.2188, 0.1985, 0.1224, 0.4131, 0.2516, 0.3624], [0.4011, 0.4101, 0.4584, 0.3952, 0.2835, 0.196, 0.4444, 0.3539, 0.1049, 0.148, 0.3069, 0.1509, 0.3371, 0.3828, 0.1454], [0.3537, 0.1813, 0.2418, 0.1806, 0.2141, 0.1446, 0.2655, 0.4418, 0.2909, 0.376, 0.2877, 0.2786, 0.1133, 0.2497, 0.3819], [0.4844, 0.1147, 0.137, 0.3769, 0.2688, 0.2231, 0.4576, 0.4729, 0.2972, 0.3173, 0.2264, 0.2777, 0.2714, 0.1735, 0.2864], [0.2371, 0.2439, 0.4789, 0.1194, 0.263, 0.3333, 0.3888, 0.1385, 0.3507, 0.3355, 0.4096, 0.3945, 0.342, 0.1023, 0.1019]]</t>
+          <t>[1,2,8,5,3,7,9,5,2,5,6,10,4,4,3]</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>[[0, 5], [0, 5], [0, 5], [0, 5], [1, 5], [3, 5], [0, 5], [1, 5], [1, 5], [2, 5], [0, 5], [2, 5], [1, 5], [0, 5], [3, 5]]</t>
+          <t>[[0.38,0.47,0.86,0.63,0.78,0.7,0.28,0.72,0.39,0.65,0.44,0.9,0.38,0.4,0.85],[0.22,0.69,0.71,0.79,0.88,0.88,0.25,0.78,0.65,0.65,0.29,0.66,0.89,0.84,0.51],[0.23,0.45,0.78,0.69,0.52,0.24,0.5,0.53,0.85,0.65,0.42,0.57,0.25,0.88,0.45],[0.53,0.45,0.68,0.66,0.7,0.39,0.42,0.29,0.66,0.23,0.62,0.81,0.82,0.51,0.52],[0.25,0.67,0.77,0.37,0.49,0.79,0.81,0.37,0.59,0.33,0.27,0.84,0.77,0.73,0.23],[0.79,0.51,0.44,0.58,0.26,0.73,0.61,0.33,0.33,0.33,0.24,0.61,0.79,0.21,0.23],[0.6,0.77,0.43,0.44,0.62,0.39,0.22,0.71,0.64,0.61,0.72,0.67,0.34,0.45,0.29],[0.29,0.67,0.8,0.87,0.64,0.33,0.27,0.77,0.61,0.63,0.75,0.69,0.78,0.24,0.72],[0.8,0.4,0.65,0.42,0.87,0.22,0.61,0.32,0.7,0.32,0.36,0.55,0.84,0.35,0.3],[0.73,0.55,0.84,0.3,0.65,0.36,0.31,0.68,0.62,0.73,0.42,0.51,0.48,0.89,0.4]]</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>[[1,5],[0,5],[1,5],[2,5],[2,5],[1,5],[1,5],[2,5],[2,5],[1,5],[2,5],[2,5],[0,5],[0,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>[1,2,2,1,1,1,1,1,1,2]</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,1,2,1,2,1,2]</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>[90,20,100,90,60,20,80,60,20,50]</t>
         </is>
       </c>
     </row>
@@ -1336,19 +2028,37 @@
       <c r="B40" t="n">
         <v>15</v>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>[4, 7, 1, 5, 6, 2, 4, 5, 7, 7, 4, 8, 10, 3, 3]</t>
-        </is>
+      <c r="C40" t="n">
+        <v>5</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>[[0.2321, 0.3139, 0.3361, 0.2652, 0.3196, 0.3639, 0.2888, 0.3213, 0.3173, 0.2945, 0.2223, 0.2997, 0.1377, 0.4247, 0.2492], [0.3405, 0.2354, 0.4742, 0.1314, 0.4238, 0.2374, 0.3566, 0.3384, 0.3299, 0.3065, 0.2049, 0.2654, 0.142, 0.2638, 0.4408], [0.1785, 0.4177, 0.3597, 0.3631, 0.3372, 0.2709, 0.468, 0.3695, 0.1055, 0.38, 0.498, 0.4829, 0.1674, 0.2615, 0.4576], [0.3795, 0.1922, 0.1871, 0.3035, 0.4145, 0.484, 0.4903, 0.4494, 0.3344, 0.2507, 0.4812, 0.2185, 0.3883, 0.2894, 0.2885], [0.3128, 0.3693, 0.3941, 0.3227, 0.1033, 0.3249, 0.397, 0.4143, 0.4967, 0.469, 0.2608, 0.3159, 0.4275, 0.2842, 0.461], [0.1899, 0.2087, 0.3897, 0.3855, 0.4494, 0.1107, 0.3058, 0.4121, 0.3532, 0.4049, 0.1442, 0.1633, 0.2404, 0.2102, 0.1937], [0.1274, 0.3822, 0.1029, 0.3821, 0.2858, 0.1273, 0.1685, 0.225, 0.3403, 0.3072, 0.3029, 0.353, 0.4505, 0.4645, 0.2879], [0.1241, 0.1001, 0.3862, 0.287, 0.1805, 0.262, 0.3111, 0.4039, 0.3171, 0.295, 0.4134, 0.3763, 0.3619, 0.2209, 0.2739], [0.2602, 0.2263, 0.2701, 0.3835, 0.3157, 0.176, 0.3426, 0.1203, 0.2153, 0.1869, 0.3183, 0.2106, 0.3204, 0.2095, 0.3144], [0.3704, 0.3734, 0.269, 0.4479, 0.4969, 0.1197, 0.2317, 0.1128, 0.3994, 0.1229, 0.3093, 0.2921, 0.3919, 0.3936, 0.2159]]</t>
+          <t>[10,2,1,7,6,2,9,1,2,8,1,5,7,3,3]</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>[[2, 5], [3, 5], [2, 5], [0, 5], [1, 5], [1, 5], [3, 5], [3, 5], [0, 5], [2, 5], [3, 5], [1, 5], [0, 5], [3, 5], [3, 5]]</t>
+          <t>[[0.41,0.45,0.6,0.38,0.84,0.39,0.83,0.27,0.66,0.83,0.32,0.88,0.52,0.86,0.67],[0.41,0.33,0.41,0.27,0.3,0.27,0.5,0.76,0.3,0.29,0.65,0.34,0.27,0.32,0.85],[0.78,0.45,0.66,0.58,0.67,0.68,0.64,0.39,0.23,0.52,0.82,0.6,0.78,0.89,0.31],[0.68,0.67,0.89,0.89,0.68,0.37,0.76,0.27,0.75,0.84,0.47,0.64,0.5,0.51,0.42],[0.73,0.86,0.86,0.32,0.81,0.72,0.38,0.25,0.39,0.84,0.64,0.7,0.38,0.7,0.22],[0.46,0.64,0.3,0.78,0.36,0.66,0.48,0.62,0.28,0.21,0.84,0.39,0.77,0.9,0.35],[0.39,0.66,0.88,0.84,0.55,0.76,0.3,0.88,0.88,0.31,0.41,0.27,0.39,0.77,0.46],[0.26,0.44,0.89,0.64,0.49,0.32,0.89,0.77,0.4,0.25,0.24,0.28,0.61,0.85,0.55],[0.79,0.51,0.7,0.71,0.32,0.45,0.65,0.25,0.45,0.57,0.9,0.53,0.77,0.5,0.76],[0.62,0.82,0.49,0.62,0.64,0.49,0.3,0.27,0.21,0.81,0.37,0.35,0.72,0.42,0.55]]</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>[[2,5],[2,5],[2,5],[1,5],[1,5],[1,5],[1,5],[1,5],[1,5],[0,5],[2,5],[2,5],[2,5],[0,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,1,1,1,1,2,2]</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>[2,2,1,1,2,2,1,2,1,1]</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>[20,80,20,50,50,30,30,20,90,20]</t>
         </is>
       </c>
     </row>
@@ -1359,19 +2069,37 @@
       <c r="B41" t="n">
         <v>15</v>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>[3, 2, 8, 8, 2, 10, 3, 1, 3, 4, 7, 6, 9, 3, 5]</t>
-        </is>
+      <c r="C41" t="n">
+        <v>5</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>[[0.391, 0.1346, 0.1217, 0.1145, 0.2107, 0.1391, 0.1773, 0.3983, 0.4797, 0.4732, 0.2414, 0.1574, 0.3604, 0.1349, 0.1583], [0.2087, 0.2959, 0.4244, 0.4254, 0.2265, 0.2127, 0.2425, 0.2468, 0.4038, 0.1015, 0.2195, 0.4579, 0.1936, 0.3049, 0.3373], [0.4904, 0.2868, 0.3931, 0.1672, 0.2863, 0.4976, 0.1465, 0.4684, 0.115, 0.3932, 0.2774, 0.2371, 0.3332, 0.2967, 0.3642], [0.3824, 0.1549, 0.3146, 0.4325, 0.2895, 0.2266, 0.4913, 0.2335, 0.239, 0.1468, 0.2133, 0.41, 0.2181, 0.121, 0.2532], [0.4172, 0.4733, 0.1438, 0.4518, 0.1023, 0.2113, 0.1076, 0.3759, 0.2707, 0.2128, 0.3534, 0.3844, 0.4859, 0.401, 0.2183], [0.4689, 0.4209, 0.3975, 0.2696, 0.2558, 0.2529, 0.2669, 0.4444, 0.3943, 0.3155, 0.3473, 0.3079, 0.264, 0.1259, 0.4657], [0.3354, 0.4878, 0.2734, 0.1912, 0.1603, 0.2886, 0.3478, 0.4659, 0.1667, 0.4148, 0.422, 0.4708, 0.4236, 0.3552, 0.1659], [0.1915, 0.2497, 0.2506, 0.2885, 0.1619, 0.472, 0.3026, 0.2059, 0.1132, 0.45, 0.3036, 0.2999, 0.3546, 0.3551, 0.4299], [0.2147, 0.4272, 0.2424, 0.377, 0.1402, 0.2072, 0.4621, 0.4749, 0.3304, 0.1509, 0.3306, 0.1884, 0.2853, 0.4379, 0.3122], [0.4831, 0.3833, 0.4627, 0.1007, 0.1114, 0.4512, 0.1835, 0.2793, 0.2424, 0.3517, 0.3067, 0.4896, 0.2247, 0.2692, 0.3304]]</t>
+          <t>[4,1,7,8,4,9,4,1,3,9,5,4,10,6,10]</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>[[3, 5], [3, 5], [0, 5], [1, 5], [2, 5], [3, 5], [3, 5], [2, 5], [0, 5], [0, 5], [1, 5], [2, 5], [3, 5], [1, 5], [2, 5]]</t>
+          <t>[[0.31,0.87,0.8,0.8,0.48,0.73,0.3,0.21,0.21,0.61,0.52,0.56,0.21,0.5,0.7],[0.51,0.71,0.36,0.77,0.61,0.35,0.37,0.64,0.78,0.49,0.38,0.81,0.67,0.51,0.54],[0.34,0.64,0.45,0.9,0.54,0.54,0.6,0.84,0.76,0.52,0.7,0.61,0.54,0.33,0.52],[0.37,0.84,0.43,0.87,0.57,0.64,0.58,0.29,0.46,0.27,0.64,0.51,0.74,0.35,0.32],[0.48,0.85,0.7,0.49,0.56,0.26,0.89,0.67,0.4,0.61,0.28,0.88,0.32,0.65,0.37],[0.7,0.74,0.67,0.63,0.82,0.26,0.43,0.37,0.89,0.47,0.71,0.68,0.35,0.37,0.4],[0.49,0.36,0.21,0.82,0.88,0.44,0.44,0.2,0.68,0.78,0.3,0.31,0.75,0.63,0.23],[0.64,0.42,0.46,0.74,0.77,0.48,0.86,0.48,0.74,0.54,0.83,0.84,0.26,0.86,0.78],[0.75,0.34,0.76,0.8,0.4,0.87,0.23,0.3,0.58,0.6,0.65,0.21,0.87,0.23,0.3],[0.21,0.6,0.85,0.67,0.78,0.21,0.58,0.52,0.55,0.25,0.68,0.55,0.74,0.54,0.3]]</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>[[2,5],[2,5],[1,5],[0,5],[1,5],[0,5],[2,5],[2,5],[0,5],[1,5],[1,5],[1,5],[0,5],[2,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>[1,2,2,1,2,2,2,2,2,1]</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>[2,2,1,2,1,1,2,1,2,1]</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>[100,80,80,100,100,40,80,50,60,50]</t>
         </is>
       </c>
     </row>
@@ -1382,19 +2110,37 @@
       <c r="B42" t="n">
         <v>15</v>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>[10, 2, 3, 4, 3, 2, 1, 4, 10, 10, 10, 4, 6, 2, 5]</t>
-        </is>
+      <c r="C42" t="n">
+        <v>5</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>[[0.4723, 0.3404, 0.3626, 0.3082, 0.4427, 0.1475, 0.182, 0.4357, 0.2669, 0.4409, 0.1847, 0.4004, 0.2467, 0.4266, 0.2049], [0.489, 0.2094, 0.1998, 0.3279, 0.2356, 0.2853, 0.2863, 0.3017, 0.4221, 0.1142, 0.3602, 0.1323, 0.4681, 0.1493, 0.3714], [0.2922, 0.3674, 0.2866, 0.4303, 0.2811, 0.1985, 0.3225, 0.1829, 0.4228, 0.4832, 0.4117, 0.2406, 0.1562, 0.2941, 0.1281], [0.182, 0.2212, 0.1759, 0.2357, 0.1712, 0.1427, 0.2047, 0.4493, 0.2233, 0.4446, 0.238, 0.2038, 0.2914, 0.4186, 0.4587], [0.1637, 0.4537, 0.3633, 0.3404, 0.4745, 0.1135, 0.1842, 0.1348, 0.4744, 0.1179, 0.458, 0.2795, 0.4241, 0.4279, 0.2026], [0.4449, 0.2045, 0.1213, 0.1813, 0.4239, 0.3555, 0.281, 0.335, 0.274, 0.4257, 0.498, 0.3835, 0.2734, 0.3791, 0.4901], [0.4742, 0.1429, 0.3923, 0.3284, 0.4223, 0.3306, 0.2062, 0.3045, 0.4757, 0.1969, 0.3743, 0.1362, 0.3305, 0.2406, 0.4398], [0.1324, 0.4835, 0.3026, 0.4788, 0.406, 0.1164, 0.3435, 0.4991, 0.15, 0.4553, 0.1754, 0.3676, 0.1225, 0.3743, 0.3118], [0.3896, 0.364, 0.1841, 0.3823, 0.4872, 0.2402, 0.3673, 0.2259, 0.2513, 0.4495, 0.3159, 0.4124, 0.4843, 0.3022, 0.4218], [0.2269, 0.4991, 0.4787, 0.166, 0.4658, 0.2972, 0.3373, 0.3097, 0.4141, 0.4949, 0.3691, 0.164, 0.1597, 0.3478, 0.274]]</t>
+          <t>[6,2,8,6,2,9,4,1,5,7,10,10,1,2,4]</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>[[1, 5], [2, 5], [1, 5], [0, 5], [1, 5], [1, 5], [1, 5], [3, 5], [1, 5], [0, 5], [2, 5], [2, 5], [2, 5], [1, 5], [0, 5]]</t>
+          <t>[[0.65,0.32,0.81,0.63,0.31,0.87,0.56,0.25,0.64,0.38,0.76,0.77,0.89,0.55,0.52],[0.73,0.29,0.58,0.58,0.26,0.49,0.8,0.8,0.27,0.26,0.38,0.81,0.29,0.7,0.27],[0.64,0.45,0.75,0.36,0.65,0.36,0.7,0.81,0.29,0.81,0.62,0.29,0.5,0.31,0.69],[0.73,0.27,0.55,0.77,0.86,0.56,0.87,0.57,0.48,0.79,0.55,0.53,0.54,0.79,0.78],[0.48,0.43,0.54,0.6,0.37,0.76,0.54,0.43,0.27,0.37,0.86,0.41,0.32,0.52,0.41],[0.22,0.43,0.58,0.59,0.45,0.51,0.88,0.46,0.38,0.37,0.52,0.73,0.34,0.7,0.21],[0.49,0.74,0.44,0.59,0.34,0.72,0.24,0.8,0.34,0.81,0.45,0.71,0.42,0.83,0.29],[0.32,0.55,0.26,0.34,0.86,0.88,0.46,0.85,0.58,0.39,0.69,0.66,0.89,0.39,0.67],[0.24,0.28,0.2,0.9,0.76,0.75,0.56,0.41,0.31,0.4,0.46,0.73,0.58,0.25,0.21],[0.27,0.49,0.85,0.65,0.76,0.53,0.45,0.28,0.81,0.75,0.32,0.56,0.54,0.64,0.86]]</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>[[2,5],[2,5],[2,5],[2,5],[0,5],[1,5],[0,5],[1,5],[1,5],[0,5],[0,5],[0,5],[2,5],[0,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,1,2,2,2,2,2]</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>[2,2,2,2,2,1,2,2,1,2]</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>[70,80,20,50,40,20,60,100,80,60]</t>
         </is>
       </c>
     </row>
@@ -1405,19 +2151,37 @@
       <c r="B43" t="n">
         <v>15</v>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>[4, 5, 10, 6, 7, 10, 5, 7, 5, 2, 4, 9, 2, 7, 1]</t>
-        </is>
+      <c r="C43" t="n">
+        <v>5</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>[[0.281, 0.4327, 0.3573, 0.319, 0.1701, 0.4392, 0.438, 0.2578, 0.3669, 0.2716, 0.2885, 0.4499, 0.3139, 0.3336, 0.2466], [0.4775, 0.1937, 0.2873, 0.4297, 0.2076, 0.2407, 0.163, 0.4577, 0.2078, 0.4833, 0.4887, 0.3992, 0.1788, 0.1818, 0.3583], [0.181, 0.1397, 0.1508, 0.2872, 0.118, 0.2775, 0.2967, 0.1905, 0.4544, 0.1825, 0.3961, 0.3909, 0.3428, 0.2916, 0.1908], [0.441, 0.4593, 0.4357, 0.1248, 0.4684, 0.3471, 0.1021, 0.1322, 0.454, 0.455, 0.4979, 0.3656, 0.2762, 0.1929, 0.2337], [0.4616, 0.1624, 0.3669, 0.369, 0.2178, 0.3112, 0.2274, 0.3171, 0.4868, 0.3355, 0.3131, 0.3993, 0.4333, 0.2625, 0.4122], [0.1178, 0.4285, 0.1039, 0.3359, 0.2228, 0.1791, 0.1097, 0.3688, 0.293, 0.4765, 0.4125, 0.4724, 0.419, 0.1777, 0.1669], [0.2817, 0.1235, 0.3325, 0.3852, 0.3215, 0.2073, 0.3094, 0.4899, 0.1332, 0.152, 0.2073, 0.1984, 0.3091, 0.4144, 0.3501], [0.3081, 0.338, 0.4143, 0.1741, 0.3264, 0.2447, 0.3802, 0.3845, 0.2143, 0.3996, 0.1389, 0.4305, 0.3657, 0.2597, 0.3963], [0.293, 0.1283, 0.2323, 0.4868, 0.2052, 0.4702, 0.3527, 0.2102, 0.4851, 0.3277, 0.3835, 0.4605, 0.1798, 0.1413, 0.1752], [0.201, 0.3001, 0.1463, 0.4797, 0.2449, 0.1309, 0.3668, 0.3583, 0.2601, 0.1433, 0.1669, 0.467, 0.1324, 0.1932, 0.2185]]</t>
+          <t>[3,4,6,4,7,10,4,8,9,6,5,8,8,8,3]</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>[[2, 5], [0, 5], [1, 5], [0, 5], [2, 5], [2, 5], [0, 5], [3, 5], [2, 5], [1, 5], [2, 5], [3, 5], [0, 5], [3, 5], [1, 5]]</t>
+          <t>[[0.61,0.58,0.24,0.24,0.33,0.22,0.72,0.71,0.3,0.79,0.31,0.41,0.37,0.46,0.38],[0.54,0.49,0.89,0.24,0.3,0.24,0.64,0.24,0.79,0.56,0.57,0.59,0.32,0.34,0.42],[0.62,0.35,0.28,0.88,0.22,0.76,0.75,0.41,0.29,0.3,0.69,0.65,0.75,0.86,0.68],[0.31,0.37,0.79,0.35,0.25,0.69,0.48,0.84,0.66,0.26,0.86,0.38,0.44,0.48,0.24],[0.55,0.29,0.48,0.45,0.74,0.76,0.31,0.46,0.46,0.31,0.76,0.7,0.33,0.46,0.27],[0.64,0.28,0.89,0.75,0.47,0.6,0.84,0.59,0.32,0.47,0.79,0.65,0.66,0.81,0.83],[0.84,0.27,0.58,0.72,0.73,0.62,0.32,0.76,0.7,0.26,0.52,0.32,0.44,0.21,0.48],[0.58,0.63,0.66,0.79,0.35,0.28,0.8,0.31,0.88,0.79,0.55,0.89,0.27,0.41,0.65],[0.45,0.85,0.25,0.58,0.61,0.66,0.38,0.46,0.79,0.34,0.78,0.59,0.73,0.7,0.35],[0.6,0.81,0.5,0.88,0.52,0.3,0.47,0.87,0.42,0.81,0.82,0.45,0.26,0.71,0.42]]</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>[[2,5],[1,5],[0,5],[0,5],[2,5],[2,5],[1,5],[0,5],[2,5],[2,5],[0,5],[2,5],[0,5],[0,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>[1,1,2,1,1,1,1,1,1,2]</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>[2,1,2,2,1,1,2,1,1,2]</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>[100,60,20,100,80,40,30,30,100,40]</t>
         </is>
       </c>
     </row>
@@ -1428,19 +2192,37 @@
       <c r="B44" t="n">
         <v>15</v>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>[9, 9, 5, 6, 4, 5, 7, 7, 7, 6, 6, 4, 4, 5, 10]</t>
-        </is>
+      <c r="C44" t="n">
+        <v>5</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>[[0.213, 0.3971, 0.2513, 0.3712, 0.4666, 0.1676, 0.3674, 0.3111, 0.2745, 0.4924, 0.3995, 0.2211, 0.2639, 0.1915, 0.1626], [0.1667, 0.2707, 0.325, 0.134, 0.3127, 0.2084, 0.4606, 0.3066, 0.2629, 0.384, 0.1277, 0.2126, 0.4776, 0.21, 0.2409], [0.4778, 0.2012, 0.2921, 0.3266, 0.2334, 0.1827, 0.2319, 0.4471, 0.1616, 0.3183, 0.1085, 0.2415, 0.4316, 0.1715, 0.4301], [0.4914, 0.3853, 0.2086, 0.2902, 0.2775, 0.2699, 0.4744, 0.4279, 0.1595, 0.4439, 0.224, 0.1671, 0.4619, 0.4151, 0.1868], [0.2837, 0.3103, 0.359, 0.3982, 0.2604, 0.1506, 0.13, 0.2853, 0.1406, 0.1283, 0.2212, 0.1993, 0.2567, 0.338, 0.3679], [0.4447, 0.4381, 0.1193, 0.3466, 0.4482, 0.181, 0.2156, 0.1755, 0.2686, 0.2766, 0.2603, 0.1901, 0.2984, 0.2082, 0.2356], [0.4386, 0.4859, 0.2303, 0.4163, 0.4247, 0.1305, 0.128, 0.1338, 0.1217, 0.1146, 0.3572, 0.4264, 0.332, 0.1514, 0.4113], [0.431, 0.3661, 0.3329, 0.2733, 0.1164, 0.4129, 0.2925, 0.4199, 0.1835, 0.437, 0.2893, 0.2085, 0.4771, 0.4848, 0.376], [0.4777, 0.2458, 0.1483, 0.4137, 0.3869, 0.2045, 0.2346, 0.1889, 0.2427, 0.3117, 0.494, 0.2089, 0.2687, 0.2057, 0.2065], [0.1032, 0.339, 0.1488, 0.2964, 0.4635, 0.4114, 0.2115, 0.2796, 0.3452, 0.4146, 0.3954, 0.1216, 0.2323, 0.4927, 0.3379]]</t>
+          <t>[4,4,10,9,5,6,5,7,2,6,7,8,10,4,4]</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>[[0, 5], [1, 5], [2, 5], [1, 5], [2, 5], [3, 5], [2, 5], [3, 5], [1, 5], [3, 5], [0, 5], [1, 5], [2, 5], [3, 5], [0, 5]]</t>
+          <t>[[0.75,0.51,0.54,0.74,0.47,0.51,0.46,0.46,0.57,0.77,0.45,0.57,0.67,0.39,0.39],[0.85,0.71,0.6,0.65,0.22,0.63,0.56,0.58,0.45,0.26,0.34,0.87,0.49,0.53,0.24],[0.23,0.7,0.58,0.56,0.37,0.72,0.32,0.33,0.52,0.4,0.37,0.65,0.66,0.78,0.49],[0.25,0.39,0.89,0.62,0.7,0.21,0.56,0.23,0.6,0.84,0.88,0.58,0.52,0.86,0.67],[0.25,0.53,0.37,0.53,0.52,0.61,0.45,0.31,0.55,0.78,0.66,0.44,0.85,0.84,0.35],[0.23,0.72,0.78,0.88,0.82,0.62,0.57,0.22,0.37,0.52,0.64,0.59,0.72,0.4,0.6],[0.26,0.49,0.73,0.69,0.89,0.39,0.55,0.43,0.51,0.8,0.68,0.82,0.34,0.81,0.24],[0.82,0.43,0.42,0.56,0.86,0.23,0.45,0.8,0.48,0.34,0.5,0.47,0.84,0.73,0.55],[0.89,0.53,0.24,0.38,0.51,0.31,0.86,0.74,0.39,0.61,0.71,0.86,0.82,0.56,0.74],[0.59,0.59,0.28,0.29,0.57,0.39,0.21,0.71,0.22,0.62,0.58,0.88,0.54,0.24,0.59]]</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>[[1,5],[2,5],[0,5],[2,5],[2,5],[0,5],[0,5],[1,5],[1,5],[1,5],[2,5],[1,5],[0,5],[2,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,2,1,1,1,1,2]</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,1,1,2,1,1,1]</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>[80,30,60,40,50,80,100,70,80,40]</t>
         </is>
       </c>
     </row>
@@ -1451,19 +2233,37 @@
       <c r="B45" t="n">
         <v>15</v>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>[3, 3, 5, 3, 3, 3, 3, 7, 3, 2, 3, 3, 10, 2, 2]</t>
-        </is>
+      <c r="C45" t="n">
+        <v>5</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>[[0.3912, 0.3077, 0.3556, 0.4767, 0.1482, 0.2219, 0.2988, 0.2749, 0.3555, 0.19, 0.1929, 0.3436, 0.2325, 0.2346, 0.431], [0.3912, 0.2167, 0.3878, 0.4694, 0.1019, 0.2502, 0.483, 0.438, 0.2672, 0.3168, 0.1769, 0.1234, 0.2679, 0.1499, 0.2236], [0.4289, 0.3306, 0.1818, 0.1861, 0.2852, 0.3277, 0.1056, 0.4119, 0.1367, 0.4252, 0.3607, 0.3732, 0.3444, 0.267, 0.4403], [0.3506, 0.3609, 0.4172, 0.1213, 0.1439, 0.3578, 0.1975, 0.1013, 0.3989, 0.1237, 0.287, 0.2765, 0.3343, 0.4892, 0.3613], [0.4707, 0.2393, 0.2221, 0.1996, 0.3366, 0.2691, 0.2759, 0.4671, 0.412, 0.4645, 0.3505, 0.2872, 0.2117, 0.2508, 0.4159], [0.1037, 0.4216, 0.3255, 0.1101, 0.2969, 0.1029, 0.2485, 0.2678, 0.1735, 0.3274, 0.2339, 0.3369, 0.4599, 0.2491, 0.2389], [0.1506, 0.2509, 0.1171, 0.3537, 0.2684, 0.2428, 0.4686, 0.3057, 0.1363, 0.2194, 0.1551, 0.4538, 0.204, 0.1436, 0.127], [0.2862, 0.2757, 0.3134, 0.1803, 0.3226, 0.2523, 0.252, 0.1568, 0.3537, 0.1675, 0.2853, 0.3202, 0.2699, 0.2447, 0.179], [0.2912, 0.3483, 0.2998, 0.2016, 0.3582, 0.3331, 0.1576, 0.208, 0.1714, 0.365, 0.4842, 0.4134, 0.2192, 0.2312, 0.1663], [0.1688, 0.2103, 0.3331, 0.4793, 0.2999, 0.371, 0.4897, 0.4313, 0.3452, 0.2552, 0.1797, 0.4145, 0.2858, 0.409, 0.3568]]</t>
+          <t>[2,9,6,1,2,7,4,2,6,10,10,10,7,6,1]</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>[[0, 5], [1, 5], [2, 5], [1, 5], [3, 5], [3, 5], [1, 5], [2, 5], [2, 5], [3, 5], [0, 5], [1, 5], [0, 5], [1, 5], [3, 5]]</t>
+          <t>[[0.79,0.9,0.5,0.42,0.83,0.33,0.63,0.48,0.23,0.44,0.39,0.68,0.86,0.39,0.77],[0.24,0.58,0.25,0.85,0.74,0.66,0.78,0.65,0.88,0.7,0.85,0.56,0.28,0.57,0.29],[0.61,0.54,0.64,0.21,0.34,0.54,0.87,0.47,0.5,0.7,0.62,0.41,0.49,0.35,0.88],[0.29,0.46,0.22,0.36,0.75,0.34,0.26,0.53,0.21,0.26,0.77,0.74,0.84,0.8,0.68],[0.24,0.75,0.79,0.76,0.56,0.36,0.79,0.71,0.89,0.31,0.36,0.35,0.75,0.33,0.25],[0.9,0.22,0.78,0.46,0.79,0.59,0.83,0.85,0.21,0.25,0.38,0.67,0.82,0.52,0.62],[0.33,0.76,0.88,0.39,0.55,0.26,0.59,0.55,0.3,0.51,0.43,0.57,0.61,0.21,0.73],[0.7,0.46,0.24,0.73,0.87,0.37,0.43,0.33,0.6,0.31,0.45,0.69,0.59,0.47,0.49],[0.59,0.2,0.25,0.82,0.25,0.69,0.84,0.39,0.46,0.6,0.82,0.86,0.72,0.26,0.67],[0.49,0.53,0.23,0.33,0.75,0.52,0.41,0.47,0.8,0.72,0.39,0.28,0.38,0.84,0.61]]</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>[[2,5],[1,5],[1,5],[1,5],[0,5],[1,5],[2,5],[1,5],[1,5],[0,5],[2,5],[2,5],[2,5],[1,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>[2,1,1,1,2,1,2,1,2,2]</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>[2,1,1,1,2,2,2,2,1,1]</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>[30,40,80,90,100,100,100,80,30,20]</t>
         </is>
       </c>
     </row>
@@ -1474,19 +2274,37 @@
       <c r="B46" t="n">
         <v>15</v>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>[4, 1, 8, 1, 5, 6, 10, 2, 5, 1, 1, 7, 8, 4, 4]</t>
-        </is>
+      <c r="C46" t="n">
+        <v>5</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>[[0.1738, 0.1024, 0.1495, 0.3168, 0.4792, 0.4758, 0.4701, 0.4551, 0.4686, 0.4825, 0.3561, 0.4187, 0.4237, 0.1979, 0.4924], [0.2039, 0.4437, 0.4587, 0.2446, 0.1554, 0.3031, 0.1979, 0.402, 0.4804, 0.4071, 0.3756, 0.408, 0.2205, 0.1886, 0.2256], [0.3666, 0.3348, 0.1204, 0.446, 0.4902, 0.4334, 0.4886, 0.3776, 0.4025, 0.4986, 0.1274, 0.4943, 0.4781, 0.3522, 0.335], [0.352, 0.2852, 0.4831, 0.1297, 0.4483, 0.2435, 0.4354, 0.3231, 0.345, 0.227, 0.2024, 0.1265, 0.1148, 0.2377, 0.2762], [0.1011, 0.1577, 0.3605, 0.4971, 0.4341, 0.3579, 0.3604, 0.467, 0.4254, 0.2975, 0.3701, 0.4252, 0.1592, 0.435, 0.3535], [0.3975, 0.4151, 0.2576, 0.3655, 0.1711, 0.4528, 0.122, 0.2577, 0.2192, 0.1779, 0.1631, 0.2638, 0.2735, 0.4417, 0.2954], [0.1881, 0.4206, 0.2068, 0.2292, 0.4495, 0.2021, 0.2448, 0.3009, 0.3263, 0.3083, 0.4863, 0.1901, 0.4806, 0.1485, 0.445], [0.4418, 0.4159, 0.2516, 0.196, 0.1067, 0.2614, 0.22, 0.4623, 0.2255, 0.1564, 0.3008, 0.2316, 0.283, 0.4382, 0.1046], [0.1573, 0.3433, 0.2994, 0.2468, 0.4159, 0.2173, 0.2512, 0.167, 0.4702, 0.3882, 0.2235, 0.1768, 0.4346, 0.3599, 0.2714], [0.1369, 0.3548, 0.2199, 0.4541, 0.3694, 0.2997, 0.1045, 0.1303, 0.2734, 0.1534, 0.1461, 0.3886, 0.2427, 0.2815, 0.3868]]</t>
+          <t>[2,6,9,2,10,10,6,7,1,5,7,7,2,9,4]</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>[[3, 5], [0, 5], [3, 5], [3, 5], [0, 5], [3, 5], [2, 5], [2, 5], [0, 5], [3, 5], [2, 5], [0, 5], [0, 5], [3, 5], [1, 5]]</t>
+          <t>[[0.57,0.62,0.46,0.76,0.57,0.28,0.29,0.58,0.86,0.42,0.81,0.73,0.37,0.23,0.27],[0.71,0.34,0.46,0.55,0.71,0.28,0.48,0.54,0.58,0.77,0.32,0.77,0.69,0.59,0.69],[0.49,0.3,0.67,0.57,0.65,0.44,0.83,0.61,0.26,0.51,0.73,0.76,0.55,0.83,0.39],[0.49,0.83,0.83,0.68,0.8,0.26,0.81,0.42,0.32,0.37,0.49,0.38,0.42,0.29,0.41],[0.6,0.51,0.44,0.72,0.83,0.73,0.43,0.72,0.31,0.29,0.44,0.77,0.37,0.24,0.29],[0.8,0.64,0.38,0.59,0.57,0.66,0.36,0.81,0.42,0.69,0.21,0.46,0.45,0.58,0.25],[0.75,0.35,0.67,0.76,0.59,0.72,0.66,0.45,0.77,0.41,0.6,0.72,0.47,0.41,0.52],[0.77,0.85,0.58,0.66,0.83,0.27,0.36,0.7,0.78,0.8,0.49,0.26,0.51,0.36,0.4],[0.74,0.25,0.78,0.5,0.62,0.26,0.44,0.26,0.87,0.77,0.52,0.36,0.85,0.44,0.31],[0.59,0.86,0.2,0.37,0.86,0.32,0.28,0.6,0.8,0.53,0.9,0.68,0.25,0.89,0.49]]</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>[[2,5],[2,5],[0,5],[2,5],[1,5],[0,5],[0,5],[1,5],[1,5],[1,5],[1,5],[0,5],[0,5],[0,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>[2,2,2,2,1,2,2,1,2,1]</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,1,2,2,2,2,2]</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>[70,80,40,60,70,50,90,70,40,80]</t>
         </is>
       </c>
     </row>
@@ -1497,19 +2315,37 @@
       <c r="B47" t="n">
         <v>15</v>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>[4, 7, 3, 6, 4, 5, 10, 4, 6, 2, 10, 7, 5, 7, 9]</t>
-        </is>
+      <c r="C47" t="n">
+        <v>5</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>[[0.2626, 0.2978, 0.4362, 0.1206, 0.3108, 0.3419, 0.4587, 0.3131, 0.2409, 0.3353, 0.2622, 0.3147, 0.371, 0.2844, 0.1093], [0.455, 0.3126, 0.1088, 0.4933, 0.4094, 0.3016, 0.1004, 0.2215, 0.2571, 0.1148, 0.3326, 0.4705, 0.1983, 0.272, 0.4504], [0.3872, 0.3308, 0.1973, 0.4733, 0.232, 0.1114, 0.1926, 0.1479, 0.1989, 0.4031, 0.4309, 0.3577, 0.4934, 0.2592, 0.3973], [0.192, 0.2661, 0.2278, 0.4261, 0.3375, 0.3283, 0.1924, 0.419, 0.2881, 0.2783, 0.4418, 0.4168, 0.159, 0.2307, 0.3268], [0.3212, 0.3386, 0.4531, 0.1198, 0.4013, 0.3275, 0.4569, 0.1964, 0.1838, 0.4926, 0.2839, 0.2946, 0.1066, 0.4582, 0.3321], [0.3915, 0.1778, 0.2434, 0.1607, 0.2429, 0.119, 0.4745, 0.2084, 0.1564, 0.1414, 0.442, 0.3892, 0.4786, 0.2489, 0.1432], [0.158, 0.476, 0.3491, 0.2263, 0.2533, 0.2062, 0.3758, 0.2574, 0.1289, 0.1015, 0.4981, 0.4848, 0.2878, 0.4223, 0.3867], [0.4062, 0.486, 0.3713, 0.3426, 0.4728, 0.1841, 0.4196, 0.4154, 0.3326, 0.4638, 0.1686, 0.2473, 0.2177, 0.4096, 0.1005], [0.2113, 0.3294, 0.193, 0.4492, 0.4594, 0.1079, 0.3531, 0.1003, 0.1109, 0.3314, 0.3841, 0.1843, 0.1779, 0.4253, 0.2562], [0.132, 0.329, 0.4947, 0.3976, 0.4833, 0.4054, 0.3091, 0.3909, 0.4759, 0.1403, 0.3555, 0.3114, 0.2703, 0.4366, 0.4457]]</t>
+          <t>[6,5,8,10,4,6,7,5,7,6,2,10,4,10,9]</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>[[2, 5], [2, 5], [0, 5], [0, 5], [2, 5], [0, 5], [3, 5], [1, 5], [3, 5], [2, 5], [3, 5], [0, 5], [2, 5], [3, 5], [3, 5]]</t>
+          <t>[[0.4,0.59,0.41,0.26,0.2,0.51,0.79,0.6,0.9,0.4,0.4,0.31,0.31,0.4,0.75],[0.83,0.88,0.36,0.82,0.43,0.28,0.81,0.65,0.32,0.5,0.4,0.72,0.52,0.89,0.24],[0.45,0.54,0.55,0.42,0.71,0.81,0.86,0.76,0.8,0.59,0.78,0.41,0.48,0.42,0.53],[0.4,0.87,0.42,0.27,0.57,0.24,0.28,0.35,0.53,0.5,0.76,0.72,0.5,0.43,0.42],[0.74,0.24,0.21,0.76,0.53,0.29,0.36,0.85,0.8,0.7,0.54,0.56,0.88,0.88,0.35],[0.77,0.34,0.35,0.67,0.48,0.85,0.26,0.56,0.84,0.83,0.31,0.46,0.63,0.31,0.88],[0.84,0.32,0.28,0.26,0.84,0.34,0.49,0.51,0.62,0.25,0.36,0.85,0.84,0.75,0.21],[0.43,0.64,0.39,0.84,0.64,0.25,0.84,0.87,0.25,0.57,0.41,0.47,0.33,0.6,0.87],[0.55,0.26,0.63,0.44,0.8,0.5,0.33,0.33,0.74,0.39,0.74,0.34,0.43,0.53,0.86],[0.85,0.34,0.45,0.3,0.56,0.52,0.83,0.85,0.47,0.54,0.83,0.76,0.2,0.42,0.5]]</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[2,5],[0,5],[2,5],[1,5],[2,5],[0,5],[1,5],[1,5],[2,5],[0,5],[1,5],[2,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>[1,2,1,2,1,2,2,1,2,2]</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>[2,2,1,2,1,1,1,2,1,1]</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>[80,70,80,30,20,30,60,50,100,100]</t>
         </is>
       </c>
     </row>
@@ -1520,19 +2356,37 @@
       <c r="B48" t="n">
         <v>15</v>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>[10, 5, 1, 2, 8, 4, 4, 7, 3, 3, 10, 10, 10, 5, 7]</t>
-        </is>
+      <c r="C48" t="n">
+        <v>5</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>[[0.1472, 0.4458, 0.4314, 0.3355, 0.3484, 0.1431, 0.3379, 0.3333, 0.161, 0.2383, 0.2829, 0.3628, 0.1167, 0.2426, 0.3464], [0.4904, 0.2838, 0.2877, 0.2403, 0.4524, 0.3329, 0.1959, 0.358, 0.1513, 0.289, 0.4689, 0.4127, 0.4177, 0.3842, 0.1757], [0.1363, 0.4138, 0.1665, 0.3448, 0.3808, 0.134, 0.2857, 0.492, 0.3744, 0.2637, 0.3383, 0.4991, 0.1858, 0.4874, 0.1451], [0.4242, 0.1384, 0.4449, 0.1762, 0.3138, 0.4926, 0.208, 0.2227, 0.2391, 0.4076, 0.4046, 0.1112, 0.2753, 0.2845, 0.462], [0.3251, 0.2412, 0.3315, 0.2643, 0.2906, 0.135, 0.4559, 0.2221, 0.426, 0.3245, 0.3629, 0.2336, 0.2838, 0.3213, 0.2135], [0.3561, 0.3432, 0.1191, 0.142, 0.1302, 0.4723, 0.4953, 0.3058, 0.3454, 0.2551, 0.1749, 0.2486, 0.326, 0.2714, 0.4552], [0.2804, 0.1914, 0.3987, 0.2585, 0.1943, 0.1095, 0.1271, 0.3287, 0.3678, 0.251, 0.2508, 0.4063, 0.3689, 0.2992, 0.254], [0.2585, 0.4025, 0.1802, 0.3662, 0.1833, 0.337, 0.3778, 0.1288, 0.2873, 0.3485, 0.4514, 0.4337, 0.301, 0.2421, 0.4426], [0.4859, 0.226, 0.4334, 0.4083, 0.3328, 0.1586, 0.4195, 0.1968, 0.2866, 0.4984, 0.2744, 0.3258, 0.1604, 0.3688, 0.2757], [0.2108, 0.419, 0.3496, 0.4548, 0.4414, 0.399, 0.2736, 0.2623, 0.2915, 0.218, 0.2113, 0.3653, 0.3127, 0.2211, 0.3615]]</t>
+          <t>[9,10,10,4,8,6,7,8,10,9,3,6,1,8,2]</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>[[0, 5], [3, 5], [3, 5], [3, 5], [2, 5], [0, 5], [3, 5], [0, 5], [0, 5], [3, 5], [0, 5], [2, 5], [2, 5], [2, 5], [2, 5]]</t>
+          <t>[[0.36,0.34,0.23,0.65,0.38,0.24,0.36,0.76,0.8,0.54,0.49,0.88,0.34,0.35,0.4],[0.32,0.47,0.84,0.63,0.49,0.85,0.23,0.35,0.6,0.63,0.23,0.48,0.65,0.69,0.65],[0.42,0.27,0.5,0.29,0.86,0.53,0.42,0.74,0.55,0.42,0.77,0.81,0.67,0.23,0.6],[0.73,0.3,0.36,0.82,0.21,0.73,0.53,0.51,0.2,0.77,0.45,0.58,0.67,0.69,0.87],[0.57,0.48,0.87,0.65,0.41,0.29,0.79,0.45,0.66,0.53,0.34,0.62,0.24,0.49,0.58],[0.51,0.72,0.78,0.74,0.23,0.34,0.58,0.85,0.78,0.79,0.41,0.5,0.53,0.31,0.22],[0.86,0.37,0.37,0.26,0.85,0.61,0.67,0.84,0.44,0.64,0.23,0.33,0.78,0.74,0.45],[0.46,0.57,0.2,0.37,0.35,0.38,0.76,0.4,0.33,0.55,0.81,0.37,0.25,0.45,0.72],[0.59,0.77,0.87,0.75,0.62,0.55,0.23,0.89,0.47,0.31,0.67,0.4,0.61,0.61,0.51],[0.79,0.39,0.51,0.58,0.66,0.75,0.48,0.65,0.31,0.85,0.47,0.71,0.21,0.34,0.54]]</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>[[1,5],[1,5],[0,5],[0,5],[2,5],[0,5],[1,5],[1,5],[1,5],[1,5],[0,5],[2,5],[1,5],[1,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>[1,2,2,2,1,2,1,1,1,2]</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>[1,1,1,1,1,2,2,2,1,2]</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>[40,40,80,80,20,50,90,80,80,20]</t>
         </is>
       </c>
     </row>
@@ -1543,19 +2397,37 @@
       <c r="B49" t="n">
         <v>15</v>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>[3, 7, 3, 8, 5, 1, 4, 8, 4, 2, 5, 9, 3, 6, 2]</t>
-        </is>
+      <c r="C49" t="n">
+        <v>5</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>[[0.3083, 0.367, 0.1969, 0.1613, 0.3385, 0.2586, 0.1412, 0.3694, 0.4234, 0.4711, 0.4632, 0.1493, 0.2741, 0.2838, 0.4242], [0.3568, 0.3204, 0.357, 0.2473, 0.3848, 0.1914, 0.2048, 0.2639, 0.4217, 0.1139, 0.2293, 0.4954, 0.1477, 0.2709, 0.3864], [0.2148, 0.2148, 0.4183, 0.4898, 0.3651, 0.2253, 0.3949, 0.2627, 0.1985, 0.1296, 0.3882, 0.3184, 0.2363, 0.348, 0.3079], [0.2594, 0.4307, 0.3614, 0.431, 0.2047, 0.4521, 0.1025, 0.3828, 0.1066, 0.2607, 0.237, 0.477, 0.2524, 0.4721, 0.4108], [0.2388, 0.4093, 0.1812, 0.369, 0.321, 0.3212, 0.3621, 0.1369, 0.3085, 0.2633, 0.4572, 0.2393, 0.1053, 0.2729, 0.2823], [0.2853, 0.2309, 0.1247, 0.4143, 0.4806, 0.2669, 0.4796, 0.192, 0.2901, 0.4715, 0.3458, 0.3267, 0.1696, 0.4803, 0.4018], [0.1709, 0.1069, 0.4971, 0.4511, 0.2347, 0.1731, 0.1765, 0.4591, 0.2226, 0.4465, 0.1694, 0.1284, 0.4988, 0.4696, 0.299], [0.2191, 0.3021, 0.282, 0.3114, 0.3337, 0.2452, 0.28, 0.2771, 0.1275, 0.245, 0.2825, 0.3353, 0.123, 0.1985, 0.1956], [0.3755, 0.1886, 0.4081, 0.1056, 0.4518, 0.4366, 0.3901, 0.4424, 0.4791, 0.1071, 0.3885, 0.4417, 0.4604, 0.2233, 0.2877], [0.3878, 0.2704, 0.4208, 0.1258, 0.3592, 0.3441, 0.1453, 0.3513, 0.4925, 0.3485, 0.1389, 0.3829, 0.2037, 0.1625, 0.2106]]</t>
+          <t>[4,4,5,2,10,2,9,3,6,6,4,8,2,5,8]</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>[[2, 5], [2, 5], [2, 5], [3, 5], [3, 5], [0, 5], [3, 5], [1, 5], [0, 5], [1, 5], [2, 5], [2, 5], [1, 5], [0, 5], [2, 5]]</t>
+          <t>[[0.81,0.57,0.85,0.54,0.54,0.28,0.76,0.37,0.83,0.84,0.86,0.56,0.67,0.74,0.29],[0.62,0.22,0.55,0.31,0.33,0.46,0.5,0.64,0.25,0.55,0.33,0.6,0.65,0.59,0.72],[0.43,0.74,0.5,0.54,0.65,0.21,0.66,0.63,0.42,0.26,0.26,0.85,0.68,0.29,0.45],[0.61,0.78,0.23,0.37,0.82,0.21,0.34,0.87,0.63,0.38,0.25,0.22,0.37,0.82,0.49],[0.7,0.84,0.49,0.33,0.56,0.84,0.76,0.25,0.68,0.6,0.84,0.29,0.57,0.82,0.49],[0.54,0.25,0.39,0.43,0.86,0.4,0.52,0.67,0.31,0.54,0.72,0.81,0.64,0.67,0.29],[0.86,0.29,0.74,0.39,0.85,0.7,0.73,0.35,0.51,0.63,0.74,0.27,0.87,0.82,0.39],[0.78,0.56,0.52,0.42,0.61,0.71,0.49,0.64,0.69,0.7,0.24,0.8,0.52,0.38,0.37],[0.54,0.82,0.46,0.72,0.27,0.53,0.89,0.74,0.35,0.55,0.36,0.49,0.75,0.74,0.36],[0.85,0.61,0.47,0.55,0.62,0.59,0.54,0.55,0.32,0.77,0.58,0.29,0.74,0.85,0.86]]</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>[[2,5],[2,5],[1,5],[2,5],[1,5],[2,5],[1,5],[2,5],[0,5],[1,5],[1,5],[1,5],[2,5],[0,5],[2,5]]</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>[2,1,1,2,1,1,2,1,1,2]</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>[1,2,2,1,2,2,1,2,1,1]</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>[90,60,40,40,70,90,20,70,20,90]</t>
         </is>
       </c>
     </row>
@@ -1566,19 +2438,37 @@
       <c r="B50" t="n">
         <v>15</v>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>[9, 10, 6, 8, 8, 8, 3, 1, 5, 5, 5, 7, 8, 8, 8]</t>
-        </is>
+      <c r="C50" t="n">
+        <v>5</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>[[0.4082, 0.3872, 0.4733, 0.1282, 0.3348, 0.1563, 0.2536, 0.301, 0.2279, 0.3889, 0.296, 0.4274, 0.1553, 0.4103, 0.3115], [0.2133, 0.2654, 0.2661, 0.1303, 0.4771, 0.1352, 0.3208, 0.3749, 0.409, 0.193, 0.1084, 0.2112, 0.4985, 0.3133, 0.1684], [0.363, 0.4002, 0.4664, 0.2224, 0.4979, 0.4359, 0.1651, 0.1359, 0.2848, 0.1506, 0.232, 0.3829, 0.4148, 0.4131, 0.3785], [0.2102, 0.3199, 0.3221, 0.2983, 0.1413, 0.3284, 0.4251, 0.401, 0.2614, 0.4215, 0.4856, 0.4047, 0.4337, 0.1042, 0.3835], [0.1051, 0.135, 0.4843, 0.1083, 0.3695, 0.39, 0.1841, 0.3994, 0.1497, 0.2469, 0.3232, 0.2139, 0.2607, 0.3025, 0.4478], [0.3993, 0.1717, 0.3185, 0.1876, 0.4253, 0.2038, 0.308, 0.4496, 0.2838, 0.3474, 0.1487, 0.1405, 0.3607, 0.1046, 0.2776], [0.1158, 0.2966, 0.3108, 0.4536, 0.1903, 0.384, 0.1689, 0.3975, 0.1297, 0.3617, 0.178, 0.1341, 0.4013, 0.1305, 0.4624], [0.3369, 0.102, 0.1529, 0.2064, 0.1579, 0.4682, 0.4208, 0.2686, 0.2479, 0.1292, 0.1548, 0.3336, 0.1821, 0.2401, 0.4473], [0.3746, 0.4415, 0.3321, 0.2456, 0.2821, 0.2205, 0.4735, 0.2991, 0.299, 0.1114, 0.4919, 0.2018, 0.3839, 0.1166, 0.3199], [0.3623, 0.4871, 0.2018, 0.2333, 0.4598, 0.4685, 0.2633, 0.3034, 0.2523, 0.3261, 0.4832, 0.1141, 0.1716, 0.4024, 0.1808]]</t>
+          <t>[3,4,7,9,9,8,7,8,7,8,8,3,2,10,1]</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>[[0, 5], [1, 5], [3, 5], [2, 5], [2, 5], [1, 5], [2, 5], [3, 5], [0, 5], [0, 5], [1, 5], [3, 5], [2, 5], [3, 5], [0, 5]]</t>
+          <t>[[0.46,0.29,0.56,0.28,0.85,0.33,0.38,0.48,0.47,0.76,0.52,0.32,0.39,0.56,0.3],[0.63,0.6,0.7,0.86,0.84,0.86,0.37,0.29,0.41,0.83,0.88,0.8,0.28,0.86,0.5],[0.21,0.51,0.23,0.58,0.44,0.53,0.63,0.81,0.66,0.5,0.77,0.83,0.28,0.57,0.4],[0.23,0.67,0.8,0.31,0.77,0.8,0.84,0.39,0.83,0.42,0.59,0.24,0.23,0.7,0.51],[0.38,0.33,0.67,0.2,0.76,0.26,0.33,0.47,0.54,0.45,0.42,0.87,0.65,0.22,0.5],[0.81,0.41,0.27,0.73,0.62,0.6,0.24,0.3,0.64,0.35,0.55,0.58,0.4,0.86,0.79],[0.71,0.25,0.27,0.54,0.31,0.88,0.31,0.54,0.45,0.65,0.29,0.5,0.39,0.82,0.23],[0.84,0.78,0.41,0.75,0.22,0.88,0.57,0.41,0.45,0.25,0.89,0.23,0.66,0.51,0.86],[0.37,0.57,0.54,0.69,0.25,0.34,0.35,0.72,0.33,0.6,0.35,0.8,0.86,0.56,0.45],[0.36,0.23,0.39,0.66,0.57,0.86,0.48,0.69,0.54,0.56,0.39,0.52,0.53,0.69,0.86]]</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>[[0,5],[1,5],[0,5],[1,5],[0,5],[2,5],[1,5],[0,5],[1,5],[2,5],[2,5],[1,5],[2,5],[2,5],[0,5]]</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>[1,2,2,1,2,1,2,1,1,2]</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>[1,2,2,2,1,2,1,1,1,2]</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>[80,40,40,50,50,20,70,100,60,100]</t>
         </is>
       </c>
     </row>
@@ -1589,19 +2479,37 @@
       <c r="B51" t="n">
         <v>15</v>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>[5, 5, 2, 4, 6, 9, 1, 3, 2, 5, 7, 8, 5, 7, 4]</t>
-        </is>
+      <c r="C51" t="n">
+        <v>5</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>[[0.1953, 0.2933, 0.2092, 0.1782, 0.121, 0.2418, 0.2857, 0.1868, 0.3471, 0.2102, 0.1714, 0.4819, 0.3045, 0.3758, 0.2343], [0.3517, 0.436, 0.2713, 0.4852, 0.4112, 0.4558, 0.459, 0.1939, 0.2825, 0.3336, 0.4984, 0.3163, 0.3867, 0.1268, 0.2976], [0.1376, 0.2687, 0.2774, 0.1331, 0.4891, 0.4946, 0.1489, 0.2723, 0.3386, 0.3708, 0.3352, 0.3328, 0.308, 0.2936, 0.1991], [0.2442, 0.1346, 0.3171, 0.218, 0.3749, 0.4207, 0.3126, 0.4771, 0.2882, 0.1704, 0.1676, 0.1696, 0.1731, 0.146, 0.4349], [0.2488, 0.1058, 0.2894, 0.4025, 0.3088, 0.1141, 0.242, 0.4712, 0.3198, 0.2987, 0.2681, 0.2022, 0.2009, 0.3997, 0.2454], [0.1531, 0.3795, 0.4193, 0.3918, 0.4475, 0.3871, 0.4194, 0.1034, 0.109, 0.2221, 0.2172, 0.4653, 0.4406, 0.3669, 0.4546], [0.2207, 0.3073, 0.2261, 0.1407, 0.2849, 0.3042, 0.1904, 0.3094, 0.4615, 0.2074, 0.3805, 0.3419, 0.2512, 0.1199, 0.4146], [0.1601, 0.2827, 0.1375, 0.2994, 0.4379, 0.2767, 0.4331, 0.216, 0.4148, 0.2462, 0.3209, 0.4959, 0.2734, 0.111, 0.4149], [0.4536, 0.2076, 0.3903, 0.382, 0.1768, 0.392, 0.2237, 0.18, 0.2542, 0.1525, 0.403, 0.3577, 0.4028, 0.3723, 0.1166], [0.2663, 0.3829, 0.1165, 0.1483, 0.2076, 0.1694, 0.2756, 0.1803, 0.1498, 0.1201, 0.1207, 0.4114, 0.3259, 0.1126, 0.4526]]</t>
+          <t>[3,6,5,5,10,5,9,2,3,7,1,5,3,3,4]</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>[[0, 5], [0, 5], [0, 5], [2, 5], [0, 5], [0, 5], [2, 5], [3, 5], [3, 5], [3, 5], [1, 5], [0, 5], [2, 5], [1, 5], [2, 5]]</t>
+          <t>[[0.43,0.23,0.55,0.58,0.32,0.73,0.89,0.86,0.34,0.81,0.69,0.52,0.58,0.79,0.54],[0.46,0.55,0.61,0.33,0.83,0.67,0.64,0.27,0.62,0.28,0.26,0.57,0.48,0.61,0.26],[0.5,0.32,0.89,0.59,0.68,0.43,0.27,0.88,0.4,0.5,0.65,0.22,0.77,0.58,0.39],[0.24,0.31,0.83,0.68,0.37,0.25,0.68,0.6,0.48,0.45,0.35,0.67,0.88,0.32,0.62],[0.5,0.51,0.38,0.78,0.54,0.58,0.41,0.33,0.26,0.7,0.34,0.68,0.47,0.49,0.53],[0.46,0.27,0.42,0.66,0.67,0.4,0.52,0.34,0.35,0.22,0.83,0.35,0.36,0.4,0.29],[0.65,0.25,0.29,0.65,0.44,0.7,0.59,0.38,0.66,0.28,0.58,0.51,0.39,0.62,0.81],[0.9,0.63,0.48,0.36,0.38,0.54,0.46,0.84,0.46,0.46,0.47,0.79,0.66,0.63,0.43],[0.77,0.23,0.81,0.56,0.48,0.55,0.67,0.21,0.81,0.51,0.44,0.3,0.51,0.55,0.48],[0.68,0.49,0.87,0.62,0.77,0.28,0.48,0.44,0.6,0.8,0.25,0.25,0.8,0.35,0.67]]</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>[[0,5],[2,5],[1,5],[0,5],[2,5],[1,5],[1,5],[0,5],[2,5],[2,5],[1,5],[2,5],[1,5],[1,5],[1,5]]</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>[1,1,2,2,2,2,2,2,1,1]</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>[2,2,1,2,1,2,1,2,2,2]</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>[60,70,100,40,90,70,20,20,30,90]</t>
         </is>
       </c>
     </row>

</xml_diff>